<commit_message>
A Specification tab: what a row must carry before its calculation can be written
The index tabs say what exists and where it is shown. They cannot
produce code, because they never say what a number IS. This tab lists
the thirteen things that are missing, in four groups - what the number
is, what proves it, what connects it, and governance - each with why it
is needed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Reference" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="multiple_screens" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="home" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="networth" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="performance" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="plan" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="cashflow" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="menu" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="inputs" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Specification" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="multiple_screens" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="home" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="networth" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="performance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="plan" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="cashflow" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="menu" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="inputs" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +37,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
     </font>
     <font>
       <b val="1"/>
@@ -66,15 +71,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -502,364 +508,442 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TAB — Reference</t>
+          <t>TAB — Specification</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>This tab. What the file is, what each tab holds, what each column means, and what it must comply with.</t>
+          <t>Everything a row must carry before its calculation can be written in code. The index tabs say what exists and where it is shown; this tab says what is still needed to say what each number IS.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TAB — multiple_screens</t>
+          <t>TAB — Reference</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Figures shown on more than one parent screen. A figure lives here ONCE, with every screen and every label it wears listed, so the same figure can never have two definitions.</t>
+          <t>This tab. What the file is, what each tab holds, what each column means, and what it must comply with.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TAB — home</t>
+          <t>TAB — multiple_screens</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Figures shown only on Home and the screens reached from it.</t>
+          <t>Figures shown on more than one parent screen. A figure lives here ONCE, with every screen and every label it wears listed, so the same figure can never have two definitions.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TAB — networth</t>
+          <t>TAB — home</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Figures shown only on Net worth and the screens reached from it.</t>
+          <t>Figures shown only on Home and the screens reached from it.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TAB — performance</t>
+          <t>TAB — networth</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Figures shown only on Performance and the screens reached from it.</t>
+          <t>Figures shown only on Net worth and the screens reached from it.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TAB — plan</t>
+          <t>TAB — performance</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Figures shown only on Plan and the screens reached from it.</t>
+          <t>Figures shown only on Performance and the screens reached from it.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TAB — cashflow</t>
+          <t>TAB — plan</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Figures shown only on Cash flow and the screens reached from it.</t>
+          <t>Figures shown only on Plan and the screens reached from it.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TAB — menu</t>
+          <t>TAB — cashflow</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Screens reachable only from the menu, and the figures on them.</t>
+          <t>Figures shown only on Cash flow and the screens reached from it.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>TAB — menu</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Screens reachable only from the menu, and the figures on them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>TAB — inputs</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>The raw values the engines need before any calculation happens.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Metric ID</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Parent Screen Name</t>
+          <t>COLUMN — Metric ID</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
+          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Secondary Screen Name</t>
+          <t>COLUMN — Parent Screen Name</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
+          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name on Screen</t>
+          <t>COLUMN — Secondary Screen Name</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
+          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Metric</t>
+          <t>COLUMN — Name on Screen</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>The metric's name in the code.</t>
+          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Engine</t>
+          <t>COLUMN — Name of Underlying Metric</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
+          <t>The metric's name in the code.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engine ID</t>
+          <t>COLUMN — Name of Underlying Engine</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
+          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Your name for it (72-metric file)</t>
+          <t>COLUMN — Engine ID</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
+          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Core screen?</t>
+          <t>COLUMN — Your name for it (72-metric file)</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Core screen?</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Row status</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="3" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Input ID</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of a raw input, per the same standard.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Variable name</t>
+          <t>COLUMN — Input ID</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>What the raw value is called.</t>
+          <t>The identifier of a raw input, per the same standard.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Source</t>
+          <t>COLUMN — Variable name</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
+          <t>What the raw value is called.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which metric uses it</t>
+          <t>COLUMN — Source</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Every metric identifier that depends on this input.</t>
+          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Which metric uses it</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Every metric identifier that depends on this input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Which engine uses it</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Every engine identifier that reads this input.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="3" t="inlineStr"/>
-    </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Complies with — naming</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Complies with — identifiers</t>
+          <t>Complies with — naming</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>Complies with — identifiers</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>Complies with — objectives</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
-      <c r="B36" s="3" t="inlineStr"/>
-    </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>COVERAGE — screens read so far</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>1 of 49 (Home)</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>COVERAGE — screens read so far</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>1 of 49 (Home)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>COVERAGE — what that means</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Every screen in the app is listed on its tab. Only Home carries figures so far; the rest are marked NOT STARTED. A rising count is not completeness while screens remain unread.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Input ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Variable name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Which metric uses it</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Which engine uses it</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Row status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NOT STARTED — filled as each screen is read</t>
         </is>
       </c>
     </row>
@@ -869,6 +953,244 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>What is needed</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Why it is needed, and whether the file carries it today</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>SECTION — WHAT THE NUMBER IS</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The formula</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>The actual rules in plain English, followable by hand. Nothing in the index tabs carries it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>The inputs, one by one</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Every input named separately, with its unit, and where it comes from: the person typed it, an institution download, a connected provider, or another engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>The decisions and assumptions applied</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Rounding, timing conventions, inflation, which balance is used, which date wins. Each labelled with whose decision it was — the founder's, the person's, or built in. This is the fourth link of objective 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>What comes out</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Dollars, a percentage, a date, a count or a range; its unit and its rounding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>What it says when it cannot be computed</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>The exact refusal. This is where wrong numbers get invented, so the refusal is part of the specification, not an afterthought.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>The grain</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Whether the figure is per holding, per account, per person or per household. Without it a total and a single line look identical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>The period</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>As of when, and over what window — this month, twelve months, since the person owned it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>SECTION — WHAT PROVES IT</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Worked examples</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>These inputs give this answer. Rung 2 re-runs them through the real engine on every build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>An example for every case</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>One per case the grid names: input missing, input degraded, a different shape per institution, time-bounded, related events, account type. This is rung 3, the floor for every calculation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Verification level</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Whether this engine is marked for rung 4 (the written formula made executable and checked against the code on generated inputs) and rung 5 (laws that must hold for every input). Marked by the founder, recommended by me.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>SECTION — WHAT CONNECTS IT</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Which engines feed this engine</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>The engines it depends on. Without this, build order and the one-door design cannot be worked out — a metric points at an engine today, but engines do not point at each other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Where it is implemented</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>The file and function that carry it, so file and code can be checked against each other on every build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>SECTION — GOVERNANCE</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>The founder's verdict</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>His approval of the row. A row counts as documented only when he has approved it, so without this column the coverage count is meaningless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lifecycle</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Live, cut, or superseded by another identifier. Identifiers are never reused, so a retired one must say what replaced it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1032,508 +1354,6 @@
         </is>
       </c>
       <c r="J3" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="41" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Parent Screen Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Secondary Screen Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Name on Screen</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Name of Underlying Metric</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Name of Underlying Engine</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Engine ID</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Your name for it (72-metric file)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Core screen?</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Row status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>MK-HM-M-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>YOUR INVESTMENTS</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>investTotal</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>TOTAL_INVESTMENTS</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>MK-XS-E-003</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MK-HM-M-002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>▲ up / ▼ down $X (Y%) this month</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>youReturn</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>VALUE_WEIGHTED_RETURN</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>MK-XS-E-004</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MK-HM-M-003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>prices updated &lt;when&gt;</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>freshness</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PRICE_FRESHNESS</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>MK-XS-E-005</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MK-HM-M-004</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Your net worth just crossed X</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>milestone</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>NOT IN OLD MASTER — milestoneCrossed, src/domain/milestones.ts</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>MK-HM-E-001</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MK-HM-M-005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Needs your attention (1,2,3)</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>topInsights</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>NOT IN OLD MASTER — useInsights, src/domain/insights</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>MK-HM-E-002</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MK-HM-M-006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>thisMonthNet</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>NOT IN OLD MASTER — incomeMonthlyGrid, src/domain/income</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>MK-CF-E-001</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>MK-HM-M-007</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Spent so far</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>bva.spent_total</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>NOT IN OLD MASTER — budgetVsActual, src/domain/budget</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>MK-CF-E-002</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>MK-HM-M-008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Left / Over</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>derived on screen: Income − Spent so far</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>VERIFIED 2026-08-22</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MK-HM-M-009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>&lt;n&gt;% spent · day n of m</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>pctSpent</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>derived on screen: Spent so far ÷ Income</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -1618,10 +1438,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MK-HM-M-001</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1629,207 +1453,411 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>YOUR INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>investTotal</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TOTAL_INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>MK-XS-E-003</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MK-HM-M-002</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>/account-detail</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>▲ up / ▼ down $X (Y%) this month</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>youReturn</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>VALUE_WEIGHTED_RETURN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MK-XS-E-004</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MK-HM-M-003</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>/add-account</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>prices updated &lt;when&gt;</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>freshness</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PRICE_FRESHNESS</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>MK-XS-E-005</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MK-HM-M-004</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>/bonds</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Your net worth just crossed X</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NOT IN OLD MASTER — milestoneCrossed, src/domain/milestones.ts</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>MK-HM-E-001</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MK-HM-M-005</t>
+        </is>
+      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>/connect</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Needs your attention (1,2,3)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>topInsights</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NOT IN OLD MASTER — useInsights, src/domain/insights</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>MK-HM-E-002</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MK-HM-M-006</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>/holding-detail</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>thisMonthNet</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NOT IN OLD MASTER — incomeMonthlyGrid, src/domain/income</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>MK-CF-E-001</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MK-HM-M-007</t>
+        </is>
+      </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>/import-holdings</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Spent so far</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>bva.spent_total</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>NOT IN OLD MASTER — budgetVsActual, src/domain/budget</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>MK-CF-E-002</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MK-HM-M-008</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>/itemize</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Left / Over</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>derived on screen: Income − Spent so far</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MK-HM-M-009</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Networth</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>/look-back</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>&lt;n&gt;% spent · day n of m</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>pctSpent</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>derived on screen: Spent so far ÷ Income</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>NOT STARTED — screen not yet read</t>
+          <t>VERIFIED 2026-08-22</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1943,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1939,7 +1967,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1963,7 +1991,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1987,7 +2015,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2011,7 +2039,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2035,7 +2063,7 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2059,7 +2087,7 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2083,12 +2111,12 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>/look-back</t>
+          <t>/itemize</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -2107,12 +2135,12 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Networth</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>/what-if</t>
+          <t>/look-back</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -2133,6 +2161,300 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Parent Screen Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary Screen Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Name on Screen</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Name of Underlying Metric</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Name of Underlying Engine</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Engine ID</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Your name for it (72-metric file)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Core screen?</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Row status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>/account-detail</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>/add-account</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>/bonds</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>/connect</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>/holding-detail</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>/import-holdings</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>/look-back</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>/what-if</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>NOT STARTED — screen not yet read</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2690,7 +3012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3176,7 +3498,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3732,70 +4054,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Input ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Variable name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Which metric uses it</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Which engine uses it</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Row status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>NOT STARTED — filled as each screen is read</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
A database tab: what leaves the device, how often, and at what grain
Read from the code rather than from any document. One encrypted document
per person - or per household when two people share - rewritten in full
two seconds after any change. Twenty-eight rows covering every field, the
arrays inside the encrypted payload and their own grain, and the three
things deliberately never sent: prices, the economic feed, and the
transactions read from an institution download.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -17,6 +17,7 @@
     <sheet name="cashflow" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="menu" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="inputs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="database" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -616,290 +617,302 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>TAB — database</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>What the app saves in the cloud: where each thing is stored, what it holds, which figures depend on it, how often it is written and at what grain. Also names what is deliberately NOT saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>TAB — inputs</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>The raw values the engines need before any calculation happens.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Metric ID</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Parent Screen Name</t>
+          <t>COLUMN — Metric ID</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
+          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Secondary Screen Name</t>
+          <t>COLUMN — Parent Screen Name</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
+          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name on Screen</t>
+          <t>COLUMN — Secondary Screen Name</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
+          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Metric</t>
+          <t>COLUMN — Name on Screen</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>The metric's name in the code.</t>
+          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Engine</t>
+          <t>COLUMN — Name of Underlying Metric</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
+          <t>The metric's name in the code.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (mathematical)</t>
+          <t>COLUMN — Name of Underlying Engine</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
+          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (in words)</t>
+          <t>COLUMN — Formula (mathematical)</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
+          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engine ID</t>
+          <t>COLUMN — Formula (in words)</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
+          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Your name for it (72-metric file)</t>
+          <t>COLUMN — Engine ID</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
+          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Core screen?</t>
+          <t>COLUMN — Your name for it (72-metric file)</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Core screen?</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Row status</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-      <c r="B29" s="3" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Input ID</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of a raw input, per the same standard.</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Variable name</t>
+          <t>COLUMN — Input ID</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>What the raw value is called.</t>
+          <t>The identifier of a raw input, per the same standard.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Source</t>
+          <t>COLUMN — Variable name</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
+          <t>What the raw value is called.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which metric uses it</t>
+          <t>COLUMN — Source</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Every metric identifier that depends on this input.</t>
+          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Which metric uses it</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Every metric identifier that depends on this input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Which engine uses it</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Every engine identifier that reads this input.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-      <c r="B35" s="3" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Complies with — naming</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Complies with — identifiers</t>
+          <t>Complies with — naming</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>Complies with — identifiers</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>Complies with — objectives</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="3" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>COVERAGE — screens read so far</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>COVERAGE — screens read so far</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>COVERAGE — what that means</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Every screen in the app is listed on its tab. Only Home carries figures so far; the rest are marked NOT STARTED. A rising count is not completeness while screens remain unread.</t>
         </is>
@@ -1948,6 +1961,1102 @@
       <c r="F32" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Where it is stored</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Field name in the database</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>What it holds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Metric or input it serves</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>How often it is written</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Grain — one row per what</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Encrypted?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>users/{uid}</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>appStateEnc</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>THE WHOLE app state, encrypted on the device before it leaves it. Everything below lives inside this one field.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>every metric in this file, through the inputs tab</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2 seconds after any change in the app, the whole payload rewritten</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>ONE document per person — or per household when two people share</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Yes — the server cannot read it</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>users/{uid}</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>keyEnvelope</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>The encryption key, wrapped by the password and by the recovery code.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>when the password or recovery code is set or changed</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>the key itself is wrapped, never stored bare</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>users/{uid}</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>appState</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>The old plaintext copy from before encryption. Deleted on the first save by an updated app.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>never written now; removed on first save</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>No — which is why it is being removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>users/{uid}</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>householdId</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Whose document this person reads and writes — their own, or the partner who invited them.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>when an invite is redeemed</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>households/{owner}/members/{member}</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>code, householdId</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>The record that a partner joined a household, bound to a real invite.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>once, when the invite is redeemed</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>one per member</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>invites/{code}</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>householdId</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>An invite code and the household it points at.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>when an invite is created</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>one per invite</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>feedback/{doc}</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>the message</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Feedback sent from inside the app.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>when feedback is sent</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>one per message</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>snaptrade_users/{uid}</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>the connection record</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>The link to the brokerage connection service.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>when an account is connected</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>assetAccounts</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Every account: its name, institution, balance, class and where the figure came from.</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>account balance · account type · institution</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>one entry per account</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>liabilities</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Every debt: balance, rate, minimum payment, due day.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>debt balance · debt interest rate · debt minimum payment</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>one entry per debt</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>investments</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Holdings: ticker, quantity, price paid, lots.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>holding quantity · purchase price and date</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>one entry per holding</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>expenses</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Logged spending: date, amount, category, store.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>logged spending</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>one entry per expense</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>incomes · recurringIncomes</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Money received and the sources that repeat.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>salary and other income</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>one entry per payment or source</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>recurringExpenses</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Bills that repeat, and the day they fall.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>logged spending · the bill calendar</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>one entry per bill</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>monthlySnapshots</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Net worth as it stood at each month end.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>the trend line · beginning values</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>once a month, on the first open of a new month</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>one entry per month</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>nwDaily</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Net worth captured when the app is opened.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>the trend line · change in net worth</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>once a day, on the first open</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>one entry per day</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>onboardingProfile</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>What the person told us at setup: birth year, retirement age, spending, Social Security, pension, filing status.</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>birth year · retirement age · monthly spending · Social Security · pension · filing status</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>retirementAssumptions</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>The plan's settings: return, claim age, contributions, draw.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>assumed return · Social Security claim age</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>retirementScenarios</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Saved what-ifs.</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>the saved scenarios count</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>when a scenario is saved</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>one entry per scenario</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>bigCosts</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>One-off costs ahead, with the year each falls.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>big costs</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>one entry per cost</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>goals · selectedGoals</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Goals: target, saved so far, date.</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>goals</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>one entry per goal</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>budgetCategories · monthlyBudgetTarget · allocatedByMonth</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>The plan for spending, by category and by month.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>typical monthly essentials · planned spending</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>one entry per category or month</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>benchmarkReturns</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>The index returns the comparison uses.</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>benchmark return</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>when they are fetched</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>one entry per index and period</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>snaptradeConnections</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Which brokerages are connected.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>when a connection changes</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>one entry per connection</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>inside appStateEnc</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>estatePlan · badges · xp · streak · lastCheckIn</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Estate notes and the encouragement counters.</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>with every save</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>one per person</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>inside the encrypted blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>NOT SAVED</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>prices</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Prices are fetched fresh and held only on the device.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>holding price · price fetched at</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>never written to the cloud</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>NOT SAVED</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>economic figures (inflation, the 10-year yield)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Fetched from a feed each time; deliberately left out of the sync.</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>inflation rate</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>never written to the cloud</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>NOT SAVED</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>transactions from a download</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>The activity read from an institution file stays on the device.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>transaction amount · date · words</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>never written to the cloud</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
The database tab now names the three histories that never leave the phone
The daily record - every account and every holding, units and price kept
apart - the daily cash-plus-investments baseline, and the transaction
ledger. All three are read by the app but none is in the synced field
list, so a new phone starts with balances and no history.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -1975,7 +1975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2952,109 +2952,183 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>NOT SAVED</t>
+          <t>NOT SAVED — DEVICE ONLY</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>prices</t>
+          <t>snapshotDays</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Prices are fetched fresh and held only on the device.</t>
+          <t>THE DAILY RECORD: for each day, every account and every holding — units, price and value kept apart. This is what a beginning value is READ from instead of being back-solved.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>holding price · price fetched at</t>
+          <t>beginning value · change in account value · the performance walk</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>never written to the cloud</t>
+          <t>once a day, on the first open</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>one entry per day, per account, per holding</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>not sent at all</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>NOT SAVED</t>
+          <t>NOT SAVED — DEVICE ONLY</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>economic figures (inflation, the 10-year yield)</t>
+          <t>invDaily</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Fetched from a feed each time; deliberately left out of the sync.</t>
+          <t>Cash + investments captured daily — the baseline the Net worth return line is measured from.</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>inflation rate</t>
+          <t>Return on cash + investments</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>never written to the cloud</t>
+          <t>once a day, on the first open</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>one entry per day</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>not sent at all</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t>NOT SAVED — DEVICE ONLY</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>transactions</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>The append-only ledger read from institution downloads: every buy, sell, contribution, withdrawal, dividend and interest line. Read by 32 places in the app.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>contributions · withdrawals · income · realised gain · the change walk</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>when a file is imported or a connection syncs</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>one entry per transaction</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>not sent at all</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>NOT SAVED</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>transactions from a download</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>The activity read from an institution file stays on the device.</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>transaction amount · date · words</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>prices</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Prices are fetched fresh and held only on the device.</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>holding price · price fetched at</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>never written to the cloud</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>NOT SAVED</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>economic figures (inflation, the 10-year yield)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Fetched from a feed each time; deliberately left out of the sync.</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>inflation rate</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>never written to the cloud</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
My questions now sit on the row they are about, numbered, with a column for his answers
Thirty-three questions attached to the engine each concerns, each with a
number fixed for good - never reused, never renumbered - so an answer
can always be matched to its question without anyone mapping anything.
Beside it, a column for him to answer, starting each answer with the
same number.

A guard stops the build if any question lands on no row. A question he
cannot see is a question that never gets answered.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -741,226 +741,250 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Errors or findings to address</t>
+          <t>COLUMN — Questions for you (numbered)</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
+          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Decisions made</t>
+          <t>COLUMN — YOUR ANSWER — use the same number</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>The rulings that govern this figure, and why. The standing display and rounding rule applies to every row and is stated once at the top of this tab.</t>
+          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (mathematical)</t>
+          <t>COLUMN — Errors or findings to address</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
+          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (in words)</t>
+          <t>COLUMN — Decisions made</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
+          <t>The rulings that govern this figure, and why. The standing display and rounding rule applies to every row and is stated once at the top of this tab.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engine ID</t>
+          <t>COLUMN — Formula (mathematical)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
+          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Your name for it (72-metric file)</t>
+          <t>COLUMN — Formula (in words)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
+          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Core screen?</t>
+          <t>COLUMN — Engine ID</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Row status</t>
+          <t>COLUMN — Your name for it (72-metric file)</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
+          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
-      <c r="B34" s="3" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>COLUMN — Core screen?</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Input ID</t>
+          <t>COLUMN — Row status</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>The identifier of a raw input, per the same standard.</t>
+          <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Variable name</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>What the raw value is called.</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Source</t>
+          <t>COLUMN — Input ID</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
+          <t>The identifier of a raw input, per the same standard.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which metric uses it</t>
+          <t>COLUMN — Variable name</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Every metric identifier that depends on this input.</t>
+          <t>What the raw value is called.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which engine uses it</t>
+          <t>COLUMN — Source</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Every engine identifier that reads this input.</t>
+          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="3" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>COLUMN — Which metric uses it</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Every metric identifier that depends on this input.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Complies with — naming</t>
+          <t>COLUMN — Which engine uses it</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
+          <t>Every engine identifier that reads this input.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Complies with — identifiers</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
-        </is>
-      </c>
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Complies with — objectives</t>
+          <t>Complies with — naming</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="3" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Complies with — identifiers</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>Complies with — objectives</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr"/>
+      <c r="B46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>COVERAGE — screens read so far</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>COVERAGE — what that means</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Every screen in the app is listed on its tab. Only Home carries figures so far; the rest are marked NOT STARTED. A rising count is not completeness while screens remain unread.</t>
         </is>
@@ -3361,9 +3385,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3589,7 +3615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -3604,9 +3630,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3672,15 +3700,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -3741,12 +3779,14 @@
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -3810,13 +3850,19 @@
           <t>One thousand futures, and the odds are rounded to the nearest 5. A genuine 100 or 0 is shown literally; 98 shows as 95, never as 100 (fix B6). The best-to-worst band was removed.</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Q19 — The odds are rounded to the nearest 5 on screen but shown exact in the compare tables. Round everywhere, or show exact everywhere?</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -3872,12 +3918,14 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -3937,12 +3985,14 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -3998,12 +4048,14 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4059,12 +4111,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4116,12 +4170,14 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4138,7 +4194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -4153,9 +4209,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4221,15 +4279,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -4293,13 +4361,19 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Q22 — How old is too old for a price before the screen warns? Today it is a fixed limit in the code; you have never set it.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4355,12 +4429,14 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4416,12 +4492,14 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4473,12 +4551,14 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4518,12 +4598,14 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -4563,12 +4645,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -4608,12 +4692,14 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -4653,12 +4739,14 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -4698,12 +4786,14 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — the same screen as /invest, reached by a second route</t>
         </is>
@@ -4720,7 +4810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -4735,9 +4825,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4803,15 +4895,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -4873,13 +4975,19 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Q32 — The trend survives on a new device but the walk behind it does not. Should the trend say so, or show quietly?</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -4941,13 +5049,19 @@
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Q17 — "Return on cash + investments" counts money you paid in as a gain. Is the LABEL wrong, or the FORMULA? Fixing the formula means removing deposits and withdrawals before measuring.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5010,12 +5124,14 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5072,12 +5188,14 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5144,13 +5262,19 @@
           <t>Cash means checking, savings, high-yield savings and the uninvested sweep at a broker. Money-market funds are investments, because they pay dividends and are measured with the investments (founder, 2026-08-04).</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Q16 — Does foreign-currency cash count towards Cash, or sit apart until it is converted?</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5207,12 +5331,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5272,13 +5398,22 @@
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Q10 — What order of evidence decides an asset's class? Draft: the institution's own class field, then the shape of the identifier (option symbols, nine-character bond numbers, currency codes), then words in the name, then ask you.
+Q11 — When nothing matches: refuse the line and ask, or park it as unclassified? Parking keeps the totals right and hides a gap; refusing is honest and stops the import.
+Q12 — Does the person's own answer always win and stick, even when the next sync disagrees? That is today's rule for holdings — confirm it holds for every class.
+Q13 — Commodities: is a fund that tracks gold (GLD) simply a fund with a "commodity" label for allocation, and do you want PHYSICAL metal — weight, unit, purity, storage, spot price — supported at launch?</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5345,13 +5480,19 @@
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Q14 — What should a MIXED account be called on screen, when it holds several classes at once?</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5409,12 +5550,14 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5472,12 +5615,14 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5533,12 +5678,14 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5596,12 +5743,14 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5653,12 +5802,14 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5727,12 +5878,14 @@
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5801,13 +5954,19 @@
           <t>The recommended nest egg is 25× the yearly spending not covered by guaranteed income, counted from the start of the retirement year — which is why it differs from an outside calculator.</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Q18 — Net worth projects the pot WITHOUT your big costs; Cash flow, Budget, Goals and Social Security timing all include them. Which is right for the Net worth screen?</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5868,12 +6027,14 @@
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -5936,12 +6097,14 @@
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6001,13 +6164,19 @@
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Q23 — Same question for a value you typed by hand: after how long should the app ask you to check it?</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6062,13 +6231,19 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Q15 — An institution word we do not recognise: refuse the line and ask you, or book it as unclassified with no direction? The old sign-guess is what minted the $1.4 million.</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6136,12 +6311,14 @@
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6197,12 +6374,14 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6259,12 +6438,14 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6323,13 +6504,21 @@
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Q01 — Is Quantity for a bond the FACE amount (e.g. 227,000) with the price quoted per $100 of face, or the number of bonds? It decides how value and gain are worked out.
+Q02 — How should a bond be NAMED on screen? Draft: "US Treasury 4.25% Nov 2029", with the identifying number shown as a detail rather than the headline. Approve or rewrite.
+Q03 — Certificates of deposit: under Fixed Income, or their own class? They carry a term, a rate and an early-withdrawal penalty that a bond does not.</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6384,13 +6573,19 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Q04 — "Annual income" on a bond: the last twelve months actually received, or the forward estimate from today's coupon? Both are defensible and they differ.</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6446,12 +6641,14 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6508,13 +6705,19 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Q05 — Accrued interest: do we work it out ourselves — which needs a day-count rule per bond type — or only show what the institution gives us?</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6570,12 +6773,14 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6631,12 +6836,14 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6692,12 +6899,14 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6765,13 +6974,21 @@
           <t>A price is a ratio, not money: it keeps eight decimal places and is never rounded to cents. Rounding a Treasury bill price of $0.9888 to $0.99 invented $276 of gain on one row.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Q06 — Options: is quantity held in CONTRACTS with the price per share (so value = contracts x 100 x price), or is the price already per contract? Today neither is applied and the value may be a hundredth of the truth.
+Q07 — Crypto: how many decimal places should a quantity keep? Some coins are held in very small fractions.
+Q08 — Foreign currency: is this cash held at an institution, or currency trading? And should that tab's "Dividend" row be "Interest"?</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6830,13 +7047,19 @@
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Q09 — Should the app store the UNIT beside every quantity — shares, contracts, coins, units of face, currency units — so nothing can be multiplied by the wrong price? Today one field holds all of them with nothing marking which.</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6900,12 +7123,14 @@
         </is>
       </c>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -6969,12 +7194,14 @@
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7030,12 +7257,14 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7096,13 +7325,19 @@
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Q21 — On a second device the ledger is absent, so this reads nothing. Until history syncs, should it refuse in words rather than show a figure that looks like zero?</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7167,13 +7402,19 @@
           <t>Long-term is decided by DAYS, not calendar months (correction E7): 335 days used to count as long-term and be taxed at the lower rate.</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Q20 — A lot with no recorded purchase price is skipped, so its gain is simply absent. Should the screen SAY so — "gain not counted for N shares, no purchase price on record" — rather than quietly reporting less?</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7239,12 +7480,14 @@
         </is>
       </c>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7300,12 +7543,14 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7357,12 +7602,14 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7431,12 +7678,14 @@
         </is>
       </c>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7496,12 +7745,14 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7561,12 +7812,14 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7622,12 +7875,14 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O44" t="inlineStr">
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7683,12 +7938,14 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7748,12 +8005,14 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O46" t="inlineStr">
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -7793,12 +8052,14 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -7838,12 +8099,14 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -7883,12 +8146,14 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -7905,7 +8170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7920,9 +8185,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7988,15 +8255,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -8064,12 +8341,14 @@
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8137,12 +8416,14 @@
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8210,12 +8491,14 @@
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8283,12 +8566,14 @@
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8347,12 +8632,14 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8411,12 +8698,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8475,12 +8764,14 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8535,13 +8826,19 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Q33 — Which index should each asset class be compared against, and should the person be able to change it?</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8601,12 +8898,14 @@
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8665,12 +8964,14 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8729,12 +9030,14 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8793,12 +9096,14 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -8838,12 +9143,14 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -8883,12 +9190,14 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -8928,12 +9237,14 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -8950,7 +9261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -8965,9 +9276,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9033,15 +9346,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -9098,12 +9421,14 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9160,12 +9485,14 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9221,12 +9548,14 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9281,12 +9610,14 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9342,12 +9673,14 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9399,12 +9732,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9460,12 +9795,14 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9525,12 +9862,14 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9586,12 +9925,14 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9651,12 +9992,14 @@
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9716,12 +10059,14 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9781,12 +10126,14 @@
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9845,13 +10192,19 @@
           <t>One dated table. Start age is 73 for those born 1951–1959 and 75 for those born 1960 or later; a Roth 401(k) is exempt (fix B4).</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Q31 — Required withdrawals are estimated from balances we hold. When an institution states its own required figure, does theirs win?</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9903,12 +10256,14 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -9968,12 +10323,14 @@
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10034,12 +10391,14 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10099,12 +10458,14 @@
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10161,12 +10522,14 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10226,12 +10589,14 @@
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10287,12 +10652,14 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10348,12 +10715,14 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10409,12 +10778,14 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10470,12 +10841,14 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10531,12 +10904,14 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10592,12 +10967,14 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10667,12 +11044,14 @@
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10724,12 +11103,14 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10785,12 +11166,14 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10850,12 +11233,14 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10913,12 +11298,14 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -10974,12 +11361,14 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11036,12 +11425,14 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11111,12 +11502,14 @@
         </is>
       </c>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11181,12 +11574,14 @@
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11242,12 +11637,14 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11302,13 +11699,19 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Q26 — What education inflation rate should the college projection use, and should it be visible and editable on the screen?</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11364,12 +11767,14 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11409,12 +11814,14 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -11454,12 +11861,14 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr">
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -11499,12 +11908,14 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -11544,12 +11955,14 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — the same screen as /invest, reached by a second route</t>
         </is>
@@ -11589,12 +12002,14 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -11611,7 +12026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11626,9 +12041,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11694,15 +12111,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -11758,12 +12185,14 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11819,12 +12248,14 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11875,12 +12306,14 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11936,12 +12369,14 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -11992,12 +12427,14 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12054,12 +12491,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12116,12 +12555,14 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12178,12 +12619,14 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12239,12 +12682,14 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12301,12 +12746,14 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12363,12 +12810,14 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12424,12 +12873,14 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12485,12 +12936,14 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12546,12 +12999,14 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12608,12 +13063,14 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12669,12 +13126,14 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12730,12 +13189,14 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12791,12 +13252,14 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12852,12 +13315,14 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12909,12 +13374,14 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -12970,12 +13437,14 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13045,12 +13514,14 @@
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13106,12 +13577,14 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13168,12 +13641,14 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13229,12 +13704,14 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13293,13 +13770,19 @@
           <t>Withdrawals, including required ones, are NOT counted as guaranteed income — counting money coming out of the pot as income would count the same dollars twice (fix B5).</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Q30 — The draw from savings is shown as one figure a month. Should it hold steady in today's dollars, or rise with inflation each year?</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13356,12 +13839,14 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13417,12 +13902,14 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13462,12 +13949,14 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -13507,12 +13996,14 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -13552,12 +14043,14 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -13597,12 +14090,14 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -13642,12 +14137,14 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — the same screen as /invest, reached by a second route</t>
         </is>
@@ -13664,7 +14161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -13679,9 +14176,11 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="37" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="41" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13747,15 +14246,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Questions for you (numbered)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>YOUR ANSWER — use the same number</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Your name for it (72-metric file)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Core screen?</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Row status</t>
         </is>
@@ -13811,12 +14320,14 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13872,12 +14383,14 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13933,12 +14446,14 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -13994,12 +14509,14 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14051,12 +14568,14 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14112,12 +14631,14 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14174,12 +14695,14 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14234,13 +14757,19 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Q27 — "Typical free cash to save" uses the middle of recent months. How many months should it look back, and should a one-off windfall be excluded?</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14296,12 +14825,14 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14357,12 +14888,14 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14419,12 +14952,14 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14481,12 +15016,14 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14543,12 +15080,14 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14604,12 +15143,14 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14665,12 +15206,14 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14738,12 +15281,14 @@
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14798,13 +15343,19 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Q25 — How many years of income should the default life-cover estimate replace, and does it assume the mortgage is cleared?</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14860,12 +15411,14 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14921,12 +15474,14 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -14981,13 +15536,19 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Q28 — How many months of essentials should the app treat as safe by default — and is that number yours to set per person, or one figure for everyone?</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15043,12 +15604,14 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15104,12 +15667,14 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15165,12 +15730,14 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15225,13 +15792,19 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Q29 — What size of shock should the test use by default, and should it be a fixed dollar figure or a share of the person's spending?</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15287,12 +15860,14 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15349,12 +15924,14 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15413,13 +15990,19 @@
           <t>Explicit tables per filing status. A married band is not twice the single band — the 37% band starts at $768,700, not at double the single figure.</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Q24 — State tax is applied to taxable accounts only. Do you want a state rate captured per person, or to keep the single blended figure we use now?</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15479,12 +16062,14 @@
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15540,12 +16125,14 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15601,12 +16188,14 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
         </is>
@@ -15646,12 +16235,14 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -15691,12 +16282,14 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -15736,12 +16329,14 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -15781,12 +16376,14 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -15826,12 +16423,14 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -15871,12 +16470,14 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>
@@ -15916,12 +16517,14 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>READ 2026-08-22 — no calculated figure on this screen</t>
         </is>

</xml_diff>

<commit_message>
Core screen? said Yes on every row and nobody had decided it
The 55-70 core list has never been written down, so no row could
honestly claim to be in it. Every row now reads NOT DETERMINED, and the
Reference tab says why.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -842,7 +842,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope.</t>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -3859,7 +3859,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -3922,7 +3922,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -3989,7 +3989,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -4052,7 +4052,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -4115,7 +4115,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -4174,7 +4174,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -4370,7 +4370,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -4433,7 +4433,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -4496,7 +4496,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -4555,7 +4555,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -4602,7 +4602,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -4649,7 +4649,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -4696,7 +4696,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -4743,7 +4743,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -4790,7 +4790,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -4984,7 +4984,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -5058,7 +5058,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -5128,7 +5128,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -5192,7 +5192,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -5271,7 +5271,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -5335,7 +5335,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -5410,7 +5410,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -5489,7 +5489,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -5554,7 +5554,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -5619,7 +5619,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -5682,7 +5682,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -5747,7 +5747,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -5806,7 +5806,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -5882,7 +5882,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -5963,7 +5963,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -6031,7 +6031,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -6101,7 +6101,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -6173,7 +6173,7 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -6240,7 +6240,7 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -6315,7 +6315,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -6378,7 +6378,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -6442,7 +6442,7 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -6515,7 +6515,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -6582,7 +6582,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -6645,7 +6645,7 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -6714,7 +6714,7 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -6777,7 +6777,7 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -6840,7 +6840,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -6903,7 +6903,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -6985,7 +6985,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -7056,7 +7056,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -7127,7 +7127,7 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -7198,7 +7198,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -7261,7 +7261,7 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -7334,7 +7334,7 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -7411,7 +7411,7 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -7484,7 +7484,7 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -7547,7 +7547,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -7606,7 +7606,7 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -7682,7 +7682,7 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -7749,7 +7749,7 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -7816,7 +7816,7 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -7879,7 +7879,7 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -7942,7 +7942,7 @@
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -8009,7 +8009,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -8056,7 +8056,7 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -8103,7 +8103,7 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -8150,7 +8150,7 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -8345,7 +8345,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -8420,7 +8420,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -8495,7 +8495,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -8570,7 +8570,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -8636,7 +8636,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -8702,7 +8702,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -8768,7 +8768,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -8835,7 +8835,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -8902,7 +8902,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -8968,7 +8968,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -9034,7 +9034,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -9100,7 +9100,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -9147,7 +9147,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -9194,7 +9194,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -9241,7 +9241,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -9425,7 +9425,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -9489,7 +9489,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -9552,7 +9552,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -9614,7 +9614,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -9677,7 +9677,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -9736,7 +9736,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -9799,7 +9799,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -9866,7 +9866,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -9929,7 +9929,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -9996,7 +9996,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -10063,7 +10063,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -10130,7 +10130,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -10201,7 +10201,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -10260,7 +10260,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -10327,7 +10327,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -10395,7 +10395,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -10462,7 +10462,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -10526,7 +10526,7 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -10593,7 +10593,7 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -10656,7 +10656,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -10719,7 +10719,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -10782,7 +10782,7 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -10845,7 +10845,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -10908,7 +10908,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -10971,7 +10971,7 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -11048,7 +11048,7 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -11107,7 +11107,7 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -11170,7 +11170,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -11237,7 +11237,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -11302,7 +11302,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -11365,7 +11365,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -11429,7 +11429,7 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -11506,7 +11506,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -11578,7 +11578,7 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -11641,7 +11641,7 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -11708,7 +11708,7 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -11771,7 +11771,7 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -11818,7 +11818,7 @@
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -11865,7 +11865,7 @@
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -11912,7 +11912,7 @@
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -11959,7 +11959,7 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -12006,7 +12006,7 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -12189,7 +12189,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -12252,7 +12252,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -12310,7 +12310,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -12373,7 +12373,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -12431,7 +12431,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -12495,7 +12495,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -12559,7 +12559,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -12623,7 +12623,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -12686,7 +12686,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -12750,7 +12750,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -12814,7 +12814,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -12877,7 +12877,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -12940,7 +12940,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -13003,7 +13003,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -13067,7 +13067,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -13130,7 +13130,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -13193,7 +13193,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -13256,7 +13256,7 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -13319,7 +13319,7 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -13378,7 +13378,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -13441,7 +13441,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -13518,7 +13518,7 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -13581,7 +13581,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -13645,7 +13645,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -13708,7 +13708,7 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -13779,7 +13779,7 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -13843,7 +13843,7 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -13906,7 +13906,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -13953,7 +13953,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -14000,7 +14000,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -14047,7 +14047,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -14094,7 +14094,7 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -14141,7 +14141,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -14324,7 +14324,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -14387,7 +14387,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -14450,7 +14450,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -14513,7 +14513,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -14572,7 +14572,7 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -14635,7 +14635,7 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -14699,7 +14699,7 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -14766,7 +14766,7 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -14829,7 +14829,7 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -14892,7 +14892,7 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -14956,7 +14956,7 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -15020,7 +15020,7 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -15084,7 +15084,7 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -15147,7 +15147,7 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -15210,7 +15210,7 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -15285,7 +15285,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -15352,7 +15352,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -15415,7 +15415,7 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -15478,7 +15478,7 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -15545,7 +15545,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -15608,7 +15608,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -15671,7 +15671,7 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -15734,7 +15734,7 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -15801,7 +15801,7 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -15864,7 +15864,7 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -15928,7 +15928,7 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -15999,7 +15999,7 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -16066,7 +16066,7 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -16129,7 +16129,7 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -16192,7 +16192,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -16239,7 +16239,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -16286,7 +16286,7 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -16333,7 +16333,7 @@
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -16380,7 +16380,7 @@
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -16427,7 +16427,7 @@
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -16474,7 +16474,7 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -16521,7 +16521,7 @@
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NOT DETERMINED</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">

</xml_diff>

<commit_message>
The specification is numbered S01 to S17, each with where it stands today
So a piece of work can be named by its number instead of described. Four
columns now: the number, what is needed, why, and where this file
actually stands - one done, two part done, and fourteen missing or not
started, said plainly rather than implied.

Three items were not on the original thirteen and are added: the bridge
to his seventy-two metric names, the duplication pass he flagged, and
the fact that nobody has written down which screens are the 55-70 core.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -81,7 +81,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -526,7 +528,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Everything a row must carry before its calculation can be written in code. The index tabs say what exists and where it is shown; this tab says what is still needed to say what each number IS.</t>
+          <t>Everything a row must carry before its calculation can be written in code, NUMBERED S01 upwards so a piece of work can be named by its number. The last column says where each one stands in this file today.</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -3395,212 +3397,446 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>What is needed</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Why it is needed, and whether the file carries it today</t>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Why it is needed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Where it stands in this file today</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>SECTION — WHAT THE NUMBER IS</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
           <t>The formula</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>The actual rules in plain English, followable by hand. Nothing in the index tabs carries it.</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>The actual rules, both as arithmetic and in plain English, followable by hand.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>DONE — 163 of 163 rows carry both forms.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>The inputs, one by one</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Every input named separately, with its unit, and where it comes from: the person typed it, an institution download, a connected provider, or another engine.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>PART DONE — an inputs tab of 31 rows exists, but no row names ITS OWN inputs.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
           <t>The decisions and assumptions applied</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Rounding, timing conventions, inflation, which balance is used, which date wins. Each labelled with whose decision it was — the founder's, the person's, or built in. This is the fourth link of objective 4.</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Rounding, timing conventions, inflation, which balance is used, which date wins — each labelled with whose decision it was: the founder's, the person's, or built in. The fourth link of objective 4.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>PART DONE — 32 of 163 rows, and none says whose decision it was.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
           <t>What comes out</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Dollars, a percentage, a date, a count or a range; its unit and its rounding.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
           <t>What it says when it cannot be computed</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>The exact refusal. This is where wrong numbers get invented, so the refusal is part of the specification, not an afterthought.</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>The exact refusal. This is where wrong numbers get invented, so it is part of the specification, not an afterthought.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>The grain</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Whether the figure is per holding, per account, per person or per household. Without it a total and a single line look identical.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
           <t>The period</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>As of when, and over what window — this month, twelve months, since the person owned it.</t>
         </is>
       </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>SECTION — WHAT PROVES IT</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>S08</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
           <t>Worked examples</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>These inputs give this answer. Rung 2 re-runs them through the real engine on every build.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
           <t>An example for every case</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>One per case the grid names: input missing, input degraded, a different shape per institution, time-bounded, related events, account type. This is rung 3, the floor for every calculation.</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>One per case the grid names: input missing, input degraded, a different shape per institution, time-bounded, related events, account type. Rung 3, the floor for every calculation.</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>Verification level</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Whether this engine is marked for rung 4 (the written formula made executable and checked against the code on generated inputs) and rung 5 (laws that must hold for every input). Marked by the founder, recommended by me.</t>
         </is>
       </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>MISSING — the column does not exist yet.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>SECTION — WHAT CONNECTS IT</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
           <t>Which engines feed this engine</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>The engines it depends on. Without this, build order and the one-door design cannot be worked out — a metric points at an engine today, but engines do not point at each other.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
           <t>Where it is implemented</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>The file and function that carry it, so file and code can be checked against each other on every build.</t>
         </is>
       </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>SECTION — GOVERNANCE</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>The founder's verdict</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>His approval of the row. A row counts as documented only when he has approved it, so without this column the coverage count is meaningless.</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>MISSING — the column does not exist yet.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
           <t>Lifecycle</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Live, cut, or superseded by another identifier. Identifiers are never reused, so a retired one must say what replaced it.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>MISSING.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>SECTION — NOT ON THE ORIGINAL LIST, STILL NEEDED</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Your name for it, from the 72-metric file</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>The bridge between the founder's vocabulary and the code's. Today only four of his seventy-two names appear anywhere in the old master.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>MISSING — 0 of 163 rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>The duplication pass</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Figures that are the same thing under two identifiers — the Net worth figure that also sits on Plan. Objective 1 made real, and it must happen before the deeper columns are filled or the work gets done twice.</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>NOT STARTED — the founder flagged it; rows now exist, so it is due.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Which screens are the 55-70 core</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>The agreed first scope has never been written down, so no row can honestly say whether it is in or out.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>NOT DETERMINED on every row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inputs now carry their identifiers, and the map is checked in both directions
Every input an engine names now shows its identifier beside it, so a
figure can be traced to the input and the input to how it is captured.
Where a phrase matches no input on the tab the cell says so rather than
quietly dropping it.

The new reconciliation tab checks the two directions against each other:
what the inputs tab claims uses each input, against what each engine
actually names. Two agree. Twenty partly agree. Nine are declared and
never named by any engine. And sixty-two phrases name inputs that appear
on no row of the inputs tab at all.

That last number is the finding: the inputs tab holds thirty-one inputs
and the engines are reading far more than that.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -19,6 +19,7 @@
     <sheet name="inputs" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="database" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="core_screens" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="reconciliation" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +44,10 @@
     <font>
       <b val="1"/>
       <color rgb="001F3864"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
     <font>
       <b val="1"/>
@@ -73,16 +78,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -632,458 +640,470 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TAB — core_screens</t>
+          <t>TAB — reconciliation</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Every screen in the app, its parent, my recommendation on whether it belongs to the 55-70 core, and a column for the founder to decide. Until this is decided, no row in the file can honestly claim to be in scope (S17).</t>
+          <t>The input map checked in BOTH directions: what the inputs tab says uses each input, against what each engine actually names in its own input list. Where the two disagree the row says so. The section at the foot lists inputs an engine names that appear nowhere on the inputs tab.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TAB — database</t>
+          <t>TAB — core_screens</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>What the app saves in the cloud: where each thing is stored, what it holds, which figures depend on it, how often it is written and at what grain. Also names what is deliberately NOT saved.</t>
+          <t>Every screen in the app, its parent, my recommendation on whether it belongs to the 55-70 core, and a column for the founder to decide. Until this is decided, no row in the file can honestly claim to be in scope (S17).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>TAB — database</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>What the app saves in the cloud: where each thing is stored, what it holds, which figures depend on it, how often it is written and at what grain. Also names what is deliberately NOT saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>TAB — inputs</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>The raw values the engines need before any calculation happens.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Metric ID</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Parent Screen Name</t>
+          <t>COLUMN — Metric ID</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
+          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Secondary Screen Name</t>
+          <t>COLUMN — Parent Screen Name</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
+          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name on Screen</t>
+          <t>COLUMN — Secondary Screen Name</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
+          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Metric</t>
+          <t>COLUMN — Name on Screen</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>The metric's name in the code.</t>
+          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Engine</t>
+          <t>COLUMN — Name of Underlying Metric</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
+          <t>The metric's name in the code.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Inputs it needs (S02)</t>
+          <t>COLUMN — Name of Underlying Engine</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Every input the engine reads, named. Carried from the old master where it has a row there.</t>
+          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — What comes out (S04)</t>
+          <t>COLUMN — Inputs it needs (S02)</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Dollars, a percentage, a date, a count; how it is held and how it is shown. Marked "derived by rule" where it was worked out from the label and formula rather than read from the engine — those need confirming.</t>
+          <t>Every input the engine reads, named. Carried from the old master where it has a row there.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — What it says when it cannot be computed (S05)</t>
+          <t>COLUMN — What comes out (S04)</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>The refusal. Written where the engine has been read; NOT DETERMINED where it has not, rather than guessed.</t>
+          <t>Dollars, a percentage, a date, a count; how it is held and how it is shown. Marked "derived by rule" where it was worked out from the label and formula rather than read from the engine — those need confirming.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Grain (S06)</t>
+          <t>COLUMN — What it says when it cannot be computed (S05)</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>One figure per what: holding, account, debt, goal, category, month, or person.</t>
+          <t>The refusal. Written where the engine has been read; NOT DETERMINED where it has not, rather than guessed.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Period (S07)</t>
+          <t>COLUMN — Grain (S06)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>As of when, and over what window.</t>
+          <t>One figure per what: holding, account, debt, goal, category, month, or person.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engines it depends on (S11)</t>
+          <t>COLUMN — Period (S07)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>The engines this one calls, read from the code itself. "None found" means it reads raw values only.</t>
+          <t>As of when, and over what window.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Secondary calculations and decisions the engine makes</t>
+          <t>COLUMN — Engines it depends on (S11)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>The judgements an engine must make BEFORE its headline figure exists: what class an asset is, what to call it on screen, which units apply, whether a value is fresh. Each of these is a formula of its own and needs its own row.</t>
+          <t>The engines this one calls, read from the code itself. "None found" means it reads raw values only.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Same figure as (S16)</t>
+          <t>COLUMN — Secondary calculations and decisions the engine makes</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Where the same figure appears under more than one identifier, the row names the surviving identifier and why. Nothing is deleted: identifiers are never reused, so a folded row stays visible and says what it became.</t>
+          <t>The judgements an engine must make BEFORE its headline figure exists: what class an asset is, what to call it on screen, which units apply, whether a value is fresh. Each of these is a formula of its own and needs its own row.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Questions for you (numbered)</t>
+          <t>COLUMN — Same figure as (S16)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
+          <t>Where the same figure appears under more than one identifier, the row names the surviving identifier and why. Nothing is deleted: identifiers are never reused, so a folded row stays visible and says what it became.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — YOUR ANSWER — use the same number</t>
+          <t>COLUMN — Questions for you (numbered)</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
+          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Errors or findings to address</t>
+          <t>COLUMN — YOUR ANSWER — use the same number</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
+          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Decisions made (S03)</t>
+          <t>COLUMN — Errors or findings to address</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>The rulings and assumptions that govern this figure, each marked with WHOSE decision it was: [Founder] his own ruling, [The person] something the user set, [Built in] an assumption nobody chose on a screen — which is usually why a number looks wrong. The standing display and rounding rule applies to every row and is stated at the top of this tab.</t>
+          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (mathematical)</t>
+          <t>COLUMN — Decisions made (S03)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
+          <t>The rulings and assumptions that govern this figure, each marked with WHOSE decision it was: [Founder] his own ruling, [The person] something the user set, [Built in] an assumption nobody chose on a screen — which is usually why a number looks wrong. The standing display and rounding rule applies to every row and is stated at the top of this tab.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (in words)</t>
+          <t>COLUMN — Formula (mathematical)</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
+          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engine ID</t>
+          <t>COLUMN — Formula (in words)</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
+          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Your name for it (72-metric file)</t>
+          <t>COLUMN — Engine ID</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
+          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Core screen?</t>
+          <t>COLUMN — Your name for it (72-metric file)</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
+          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Core screen?</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Row status</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="3" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Input ID</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of a raw input, per the same standard.</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Variable name</t>
+          <t>COLUMN — Input ID</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>What the raw value is called.</t>
+          <t>The identifier of a raw input, per the same standard.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Source</t>
+          <t>COLUMN — Variable name</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
+          <t>What the raw value is called.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which metric uses it</t>
+          <t>COLUMN — Source</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Every metric identifier that depends on this input.</t>
+          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Which metric uses it</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Every metric identifier that depends on this input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Which engine uses it</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Every engine identifier that reads this input.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="3" t="inlineStr"/>
-    </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Complies with — naming</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
-        </is>
-      </c>
+      <c r="A51" s="2" t="inlineStr"/>
+      <c r="B51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Complies with — identifiers</t>
+          <t>Complies with — naming</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
+          <t>Complies with — identifiers</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
           <t>Complies with — objectives</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
-      <c r="B54" s="3" t="inlineStr"/>
-    </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>COVERAGE — screens read so far</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
-        </is>
-      </c>
+      <c r="A55" s="2" t="inlineStr"/>
+      <c r="B55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>COVERAGE — screens read so far</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
           <t>COVERAGE — what that means</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>Every screen in the app is listed on its tab. Only Home carries figures so far; the rest are marked NOT STARTED. A rising count is not completeness while screens remain unread.</t>
         </is>
@@ -4381,6 +4401,2587 @@
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E96"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Input ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Engines the inputs tab says use it</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Engines that actually name it in their own input list</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-001</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>account balance</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>NET_WORTH · REQUIRED_WITHDRAWAL · TOTAL_CASH · TOTAL_INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>ACCOUNT_SHARE_OF_TOTAL · ACCOUNT_SPLIT · ALLOCATION_BY_CLASS · DEBT_PICTURE · NET_WORTH · PLANNED_SPENDING · TOTAL_CASH · TOTAL_INVESTABLE · TOTAL_INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: REQUIRED_WITHDRAWAL  |  naming it but not declared: ACCOUNT_SHARE_OF_TOTAL, ACCOUNT_SPLIT, ALLOCATION_BY_CLASS, DEBT_PICTURE, PLANNED_SPENDING, TOTAL_INVESTABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-002</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>account type (taxable, pre-tax, Roth)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>REQUIRED_WITHDRAWAL · TAX_TREATMENT</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>institution name</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ACCOUNT_SPLIT</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-004</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>holding quantity (shares)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING_MARKET_VALUE · HOLDING_SHARES</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING_COST_BASIS · HOLDING_MARKET_VALUE · HOLDING_SHARES</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: HOLDING_COST_BASIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>holding price</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING_MARKET_VALUE · PRICE_FRESHNESS</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING_CAP_GAINS · HOLDING_MARKET_VALUE · PERFORMANCE_TABLE</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: PRICE_FRESHNESS  |  naming it but not declared: HOLDING_CAP_GAINS, PERFORMANCE_TABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-006</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>price fetched at</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_FRESHNESS</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_FRESHNESS</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>AGREES — both directions name the same engines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>purchase price and date (per lot)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING_CAP_GAINS · HOLDING_COST_BASIS</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING_CAP_GAINS · HOLDING_COST_BASIS · HOLDING_SHARES</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: HOLDING_SHARES</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>transaction amount</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>LEDGER · NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>LOOK_BACK · RETIREMENT_INCOME_NOW · SS_BENEFIT_AT_AGE · SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: LEDGER, NW_CHANGE_WALK  |  naming it but not declared: LOOK_BACK, RETIREMENT_INCOME_NOW, SS_BENEFIT_AT_AGE, SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>transaction date</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>LEDGER · NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>transaction words (the institution's own wording)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>LEDGER · the institution-words table</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>bond face value</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>BOND_FACTS</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>BOND_COUPON · BOND_FACTS · BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: BOND_COUPON, BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>bond coupon rate</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>BOND_COUPON · BOND_CURRENT_YIELD</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>BOND_COUPON · BOND_CURRENT_YIELD · BOND_FACTS · BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: BOND_FACTS, BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>bond maturity date</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>BOND_YEARS_LEFT · BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>BOND_YEARS_LEFT · BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>AGREES — both directions name the same engines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>debt balance</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_PICTURE</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_PICTURE · NET_WORTH</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: NET_WORTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>debt interest rate</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_PAYOFF</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_PICTURE · NET_WORTH</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: DEBT_PAYOFF  |  naming it but not declared: DEBT_PICTURE, NET_WORTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>debt minimum payment</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_REQUIRED_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_PICTURE · DEBT_REQUIRED_PAYMENT · NET_WORTH · SPENDING_BY_KIND</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: DEBT_PICTURE, NET_WORTH, SPENDING_BY_KIND</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>birth year</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>RMD_START_AGE · SS_BENEFIT_AT_AGE</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>SS_BENEFIT_AT_AGE · SS_CLAIM_FACTOR · WHAT_THE_PLAN_STILL_NEEDS · WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: RMD_START_AGE  |  naming it but not declared: SS_CLAIM_FACTOR, WHAT_THE_PLAN_STILL_NEEDS, WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>retirement age</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>POT_AT_RETIREMENT · WILL_IT_LAST_RESULT</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>SS_BENEFIT_AT_AGE · SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: POT_AT_RETIREMENT, WILL_IT_LAST_RESULT  |  naming it but not declared: SS_BENEFIT_AT_AGE, SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>monthly spending in retirement</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Social Security monthly amount</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME_NOW · SS_BENEFIT_AT_AGE</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>SS_BENEFIT_AT_AGE · SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: RETIREMENT_INCOME_NOW  |  naming it but not declared: SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-021</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Social Security claim age</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>SS_BENEFIT_AT_AGE · SS_CLAIM_FACTOR</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — naming it but not declared: SS_BENEFIT_AT_AGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>pension monthly amount</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME_NOW</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: RETIREMENT_INCOME_NOW  |  naming it but not declared: RETIREMENT_INCOME</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-023</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>salary and other income</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL_INCOME</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>RENTAL_INCOME_A_YEAR</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: TOTAL_INCOME  |  naming it but not declared: RENTAL_INCOME_A_YEAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>logged spending</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>PLANNED_SPENDING · SPENDING_BY_KIND</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>PLANNED_SPENDING · RETIREMENT_SPENDING · TOTAL_CASH · WHAT_THE_PLAN_STILL_NEEDS · WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: SPENDING_BY_KIND  |  naming it but not declared: RETIREMENT_SPENDING, TOTAL_CASH, WHAT_THE_PLAN_STILL_NEEDS, WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-025</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>typical monthly essentials</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>JOB_SAFETY_RUNWAY · PLANNED_SPENDING</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>big costs (amount and year)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>BIG_COSTS</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-027</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>goals (target, saved, date)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>GOAL_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-028</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>assumed return</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>POT_AT_RETIREMENT · WILL_IT_LAST_RESULT</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>ACCOUNT_SHARE_OF_TOTAL</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: POT_AT_RETIREMENT, WILL_IT_LAST_RESULT  |  naming it but not declared: ACCOUNT_SHARE_OF_TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-029</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>inflation rate</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>DECLARED BUT NEVER NAMED — the inputs tab says these engines use it, but no engine names it in its own input list. Unproved in one direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-030</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>tax filing status and age</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>TAXABLE_INCOME · TAX_ON_CONVERSION</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>PLANNED_SPENDING · TOTAL_CASH</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: TAXABLE_INCOME, TAX_ON_CONVERSION  |  naming it but not declared: PLANNED_SPENDING, TOTAL_CASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>MK-XS-I-031</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>daily and monthly snapshots</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK · TREND_SERIES</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_PCT · TREND_SERIES</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>PARTLY AGREES — declared but not naming it: NW_CHANGE_WALK  |  naming it but not declared: NW_CHANGE_PCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n"/>
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>GAPS — inputs an engine names that are on NO row of the inputs tab.</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Each one is either a missing input, or the same input under another name.</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>and how often each arrives → the matching frequency</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>any split → accountClassBreakdown</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>ALLOCATION_BY_CLASS</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>baseline date → sinceKey</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_PCT</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>chosen → monthly_payment</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_REQUIRED_PAYMENT · SPENDING_BY_KIND</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>debt paid down → debtPrincipal</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>dividends → dividends</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>do they receive it now → incomeSources</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME_NOW</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>each account's class → assetClassOf</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>ALLOCATION_BY_CLASS · PLANNED_SPENDING · TOTAL_CASH · TOTAL_INVESTABLE · TOTAL_INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>each holding's benchmark return → rows[].benchReturn</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>BENCHMARK_RETURN_BLENDED</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>each holding's return → rows[].periodReturn</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>VALUE_WEIGHTED_RETURN</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>each part → its own engine above</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL_INCOME</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>each source → ri_ss</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>ending value → ending</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>every debt → debts</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_PICTURE · NET_WORTH</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>everything → WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_RESULT</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>gross → gross</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>TAXABLE_INCOME</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>holdings → positions[]</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>ACCOUNT_SPLIT</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>how far back → months</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>LOOK_BACK</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>how they file → status</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>TAXABLE_INCOME</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>interest → interest</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>is a range wanted → withBand</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_RESULT</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>its value → rows[].marketValue</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>BENCHMARK_RETURN_BLENDED · VALUE_WEIGHTED_RETURN</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>money in → contributions</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>money out → withdrawals</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>money that counts toward retirement → NEST_EGG</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>WHAT_THE_PLAN_STILL_NEEDS</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>money to leave behind → legacyTarget</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>now → now</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>PRICE_FRESHNESS</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>optionally one account → opts.accountId</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>REALISED_GAIN</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>optionally one ticker → opts.ticker</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>REALISED_GAIN</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>options → option_holdings[]</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>ACCOUNT_SPLIT</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>or the three summary figures → b_fixed, b_nonmonthly, b_flexible</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_REQUIRED_PAYMENT · SPENDING_BY_KIND</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>percent or dollars → employerMatchMode</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>EMPLOYER_MATCH</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>ri_annuities</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>ri_other</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>ri_rmd</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>ri_withdrawals</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_INCOME</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>shape → paymentShape</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_REQUIRED_PAYMENT · SPENDING_BY_KIND</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>starting value → beginning</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_WALK</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>the account → a</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>ACCOUNT_SPLIT · HAND_VALUE_AGE</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>the categories → spendCats</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>DEBT_REQUIRED_PAYMENT · SPENDING_BY_KIND</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>the chosen chip → period</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>PERFORMANCE_TABLE</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>the dates in this sync → activityDates</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>HISTORY_DEPTH</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>the holding → position/account</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>BOND_COUPON · BOND_FACTS</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>the holdings → positions</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>PERFORMANCE_TABLE</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>the ledger → txns</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>REALISED_GAIN</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>the match → employerMatchValue</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>EMPLOYER_MATCH</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>the pot → NEST_EGG</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>the same inputs → inp</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>POT_AT_RETIREMENT</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>their own contribution → c_401k</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>EMPLOYER_MATCH</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>their own overrides → the Plan screen</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>WILL_IT_LAST_INPUTS</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>today → now</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>BOND_YEARS_LEFT · HAND_VALUE_AGE · HOLDING_CAP_GAINS · PERFORMANCE_TABLE</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>today → opts.now</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>REALISED_GAIN</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>today's value → currentInvestable</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>NW_CHANGE_PCT</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>value → value</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>BOND_YIELD_TO_MATURITY</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>what it is worth → value</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>BOND_CURRENT_YIELD</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>what we knew → existing</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>HISTORY_DEPTH</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>when the value was set → value_as_of</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>HAND_VALUE_AGE</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>where it might have gone → toSeries</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>LOOK_BACK</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>where it sat → fromSeries</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>LOOK_BACK</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>NO ID</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>where they will live → the location answer</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>RETIREMENT_SPENDING</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>MISSING FROM THE INPUTS TAB — add it, or point it at the input it already is.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4489,12 +7090,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Every input named, with its unit and where it comes from.</t>
+          <t>Every input named, with its INPUT IDENTIFIER beside it, its unit and where it comes from.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>PARTIAL — every row carries a cell; 91 name their inputs, 72 read NOT DETERMINED because the old master never held an input list for that engine.</t>
+          <t>PARTIAL — 59 rows name inputs carrying their identifiers; 72 rows name at least one input that appears nowhere on the inputs tab, and say so in the cell. The reconciliation tab checks both directions and is where the gap is counted.</t>
         </is>
       </c>
     </row>
@@ -5079,7 +7680,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>everything owned → grossAssets · everything owed → grossDebt</t>
+          <t>everything owned → grossAssets  [MK-XS-I-001] · everything owed → grossDebt  [MK-XS-I-014]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -5182,7 +7783,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>everything → WILL_IT_LAST_INPUTS · is a range wanted → withBand</t>
+          <t>everything → WILL_IT_LAST_INPUTS  [NO INPUT ID — not on the inputs tab] · is a range wanted → withBand  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -5289,7 +7890,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>each account's class → assetClassOf · each account's money → balance</t>
+          <t>each account's class → assetClassOf  [NO INPUT ID — not on the inputs tab] · each account's money → balance  [MK-XS-I-001]</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -5391,7 +7992,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>each holding's return → rows[].periodReturn · its value → rows[].marketValue</t>
+          <t>each holding's return → rows[].periodReturn  [NO INPUT ID — not on the inputs tab] · its value → rows[].marketValue  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -5946,7 +8547,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>when it was fetched → fetchedAt · now → now</t>
+          <t>when it was fetched → fetchedAt  [MK-XS-I-006] · now → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -6780,7 +9381,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>monthly snapshots → monthly · daily points → daily</t>
+          <t>monthly snapshots → monthly  [MK-XS-I-031] · daily points → daily  [MK-XS-I-031]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -6889,7 +9490,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>stored history → daily · today's value → currentInvestable · baseline date → sinceKey</t>
+          <t>stored history → daily  [MK-XS-I-031] · today's value → currentInvestable  [NO INPUT ID — not on the inputs tab] · baseline date → sinceKey  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -6998,7 +9599,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>monthly snapshots → monthly · daily points → daily</t>
+          <t>monthly snapshots → monthly  [MK-XS-I-031] · daily points → daily  [MK-XS-I-031]</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -7101,7 +9702,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>each balance → balance · each assumed return → target_return</t>
+          <t>each balance → balance  [MK-XS-I-001] · each assumed return → target_return  [MK-XS-I-028]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -7199,7 +9800,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>each account's class → assetClassOf · each account's money → balance</t>
+          <t>each account's class → assetClassOf  [NO INPUT ID — not on the inputs tab] · each account's money → balance  [MK-XS-I-001]</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -7310,7 +9911,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>each balance → balance · each assumed return → target_return</t>
+          <t>each balance → balance  [MK-XS-I-001] · each assumed return → target_return  [MK-XS-I-028]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -7413,7 +10014,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>each account's class → assetClassOf · each account's money → balance · any split → accountClassBreakdown</t>
+          <t>each account's class → assetClassOf  [NO INPUT ID — not on the inputs tab] · each account's money → balance  [MK-XS-I-001] · any split → accountClassBreakdown  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -7526,7 +10127,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>the account → a · its total → balance · uninvested → cash_balance · holdings → positions[] · options → option_holdings[]</t>
+          <t>the account → a  [NO INPUT ID — not on the inputs tab] · its total → balance  [MK-XS-I-001] · uninvested → cash_balance  [MK-XS-I-001] · holdings → positions[]  [NO INPUT ID — not on the inputs tab] · options → option_holdings[]  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -7638,7 +10239,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>every debt → debts · rates → interest_rate_apr · payments → the minimum and chosen payments</t>
+          <t>every debt → debts  [NO INPUT ID — not on the inputs tab] · rates → interest_rate_apr  [MK-XS-I-015] · payments → the minimum and chosen payments  [MK-XS-I-016]</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -7738,7 +10339,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>every debt → debts · rates → interest_rate_apr · payments → the minimum and chosen payments</t>
+          <t>every debt → debts  [NO INPUT ID — not on the inputs tab] · rates → interest_rate_apr  [MK-XS-I-015] · payments → the minimum and chosen payments  [MK-XS-I-016]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -7836,7 +10437,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>shape → paymentShape · minimum → minimum_monthly_payment · chosen → monthly_payment</t>
+          <t>shape → paymentShape  [NO INPUT ID — not on the inputs tab] · minimum → minimum_monthly_payment  [MK-XS-I-016] · chosen → monthly_payment  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -7936,7 +10537,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>every debt → debts · rates → interest_rate_apr · payments → the minimum and chosen payments</t>
+          <t>every debt → debts  [NO INPUT ID — not on the inputs tab] · rates → interest_rate_apr  [MK-XS-I-015] · payments → the minimum and chosen payments  [MK-XS-I-016]</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -8129,7 +10730,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>each account's class → assetClassOf · each account's money → balance · the categories → SPENDING_BY_KIND · the single figure → monthlySpending</t>
+          <t>each account's class → assetClassOf  [NO INPUT ID — not on the inputs tab] · each account's money → balance  [MK-XS-I-001] · the categories → SPENDING_BY_KIND  [MK-XS-I-024] · the single figure → monthlySpending  [MK-XS-I-024, MK-XS-I-030]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -8241,7 +10842,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>the same inputs → inp</t>
+          <t>the same inputs → inp  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -8354,7 +10955,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>everything owned → grossAssets · everything owed → grossDebt</t>
+          <t>everything owned → grossAssets  [MK-XS-I-001] · everything owed → grossDebt  [MK-XS-I-014]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -8459,7 +11060,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>everything owned → grossAssets · everything owed → grossDebt · every debt → debts · rates → interest_rate_apr · payments → the minimum and chosen payments</t>
+          <t>everything owned → grossAssets  [MK-XS-I-001] · everything owed → grossDebt  [MK-XS-I-014] · every debt → debts  [NO INPUT ID — not on the inputs tab] · rates → interest_rate_apr  [MK-XS-I-015] · payments → the minimum and chosen payments  [MK-XS-I-016]</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -8558,7 +11159,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>the account → a · when the value was set → value_as_of · today → now</t>
+          <t>the account → a  [NO INPUT ID — not on the inputs tab] · when the value was set → value_as_of  [NO INPUT ID — not on the inputs tab] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -8774,7 +11375,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>the account → a · its total → balance · uninvested → cash_balance · holdings → positions[] · options → option_holdings[]</t>
+          <t>the account → a  [NO INPUT ID — not on the inputs tab] · its total → balance  [MK-XS-I-001] · uninvested → cash_balance  [MK-XS-I-001] · holdings → positions[]  [NO INPUT ID — not on the inputs tab] · options → option_holdings[]  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -8979,7 +11580,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>what we knew → existing · the dates in this sync → activityDates</t>
+          <t>what we knew → existing  [NO INPUT ID — not on the inputs tab] · the dates in this sync → activityDates  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -9077,7 +11678,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>the holding → position/account</t>
+          <t>the holding → position/account  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -9185,7 +11786,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>face value → face · coupon rate → couponRate</t>
+          <t>face value → face  [MK-XS-I-011] · coupon rate → couponRate  [MK-XS-I-012]</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -9291,7 +11892,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>maturity → maturity · today → now</t>
+          <t>maturity → maturity  [MK-XS-I-013] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -9391,7 +11992,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>coupon → annualCoupon · face → face · value → value · years left → yearsToMaturity</t>
+          <t>coupon → annualCoupon  [MK-XS-I-012] · face → face  [MK-XS-I-011] · value → value  [NO INPUT ID — not on the inputs tab] · years left → yearsToMaturity  [MK-XS-I-013]</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -9493,7 +12094,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>coupon → annualCoupon · what it is worth → value</t>
+          <t>coupon → annualCoupon  [MK-XS-I-012] · what it is worth → value  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -9788,7 +12389,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>shares → totalShares · price → the latest close</t>
+          <t>shares → totalShares  [MK-XS-I-004] · price → the latest close  [MK-XS-I-005]</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -9904,7 +12505,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>each lot's shares → lots[].shares</t>
+          <t>each lot's shares → lots[].shares  [MK-XS-I-004, MK-XS-I-007]</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -10010,7 +12611,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>each lot's shares and cost → lots[].shares, lots[].cost_per_share</t>
+          <t>each lot's shares and cost → lots[].shares, lots[].cost_per_share  [MK-XS-I-004, MK-XS-I-007]</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -10112,7 +12713,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>each lot's shares and cost → lots[].shares, lots[].cost_per_share</t>
+          <t>each lot's shares and cost → lots[].shares, lots[].cost_per_share  [MK-XS-I-004, MK-XS-I-007]</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -10314,7 +12915,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>the ledger → txns · optionally one ticker → opts.ticker · optionally one account → opts.accountId · today → opts.now</t>
+          <t>the ledger → txns  [NO INPUT ID — not on the inputs tab] · optionally one ticker → opts.ticker  [NO INPUT ID — not on the inputs tab] · optionally one account → opts.accountId  [NO INPUT ID — not on the inputs tab] · today → opts.now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -10422,7 +13023,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>each lot → lots[] · price → the latest close · today → now</t>
+          <t>each lot → lots[]  [MK-XS-I-007] · price → the latest close  [MK-XS-I-005] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -10530,7 +13131,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>each lot → lots[] · price → the latest close · today → now</t>
+          <t>each lot → lots[]  [MK-XS-I-007] · price → the latest close  [MK-XS-I-005] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -10825,7 +13426,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>shares → totalShares · price → the latest close</t>
+          <t>shares → totalShares  [MK-XS-I-004] · price → the latest close  [MK-XS-I-005]</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -10935,7 +13536,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>the holding → position/account</t>
+          <t>the holding → position/account  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -11037,7 +13638,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>the holding → position/account</t>
+          <t>the holding → position/account  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -11139,7 +13740,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>face value → face · coupon rate → couponRate</t>
+          <t>face value → face  [MK-XS-I-011] · coupon rate → couponRate  [MK-XS-I-012]</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -11241,7 +13842,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>coupon → annualCoupon · what it is worth → value</t>
+          <t>coupon → annualCoupon  [MK-XS-I-012] · what it is worth → value  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -11339,7 +13940,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>the holding → position/account · face value → face · coupon rate → couponRate</t>
+          <t>the holding → position/account  [NO INPUT ID — not on the inputs tab] · face value → face  [MK-XS-I-011] · coupon rate → couponRate  [MK-XS-I-012]</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -11766,7 +14367,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>starting value → beginning · ending value → ending · money in → contributions · money out → withdrawals · dividends → dividends · interest → interest · debt paid down → debtPrincipal</t>
+          <t>starting value → beginning  [NO INPUT ID — not on the inputs tab] · ending value → ending  [NO INPUT ID — not on the inputs tab] · money in → contributions  [NO INPUT ID — not on the inputs tab] · money out → withdrawals  [NO INPUT ID — not on the inputs tab] · dividends → dividends  [NO INPUT ID — not on the inputs tab] · interest → interest  [NO INPUT ID — not on the inputs tab] · debt paid down → debtPrincipal  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -11876,7 +14477,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>starting value → beginning · ending value → ending · money in → contributions · money out → withdrawals · dividends → dividends · interest → interest · debt paid down → debtPrincipal</t>
+          <t>starting value → beginning  [NO INPUT ID — not on the inputs tab] · ending value → ending  [NO INPUT ID — not on the inputs tab] · money in → contributions  [NO INPUT ID — not on the inputs tab] · money out → withdrawals  [NO INPUT ID — not on the inputs tab] · dividends → dividends  [NO INPUT ID — not on the inputs tab] · interest → interest  [NO INPUT ID — not on the inputs tab] · debt paid down → debtPrincipal  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -11982,7 +14583,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>starting value → beginning · ending value → ending · money in → contributions · money out → withdrawals · dividends → dividends · interest → interest · debt paid down → debtPrincipal</t>
+          <t>starting value → beginning  [NO INPUT ID — not on the inputs tab] · ending value → ending  [NO INPUT ID — not on the inputs tab] · money in → contributions  [NO INPUT ID — not on the inputs tab] · money out → withdrawals  [NO INPUT ID — not on the inputs tab] · dividends → dividends  [NO INPUT ID — not on the inputs tab] · interest → interest  [NO INPUT ID — not on the inputs tab] · debt paid down → debtPrincipal  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -12092,7 +14693,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>starting value → beginning · ending value → ending · money in → contributions · money out → withdrawals · dividends → dividends · interest → interest · debt paid down → debtPrincipal</t>
+          <t>starting value → beginning  [NO INPUT ID — not on the inputs tab] · ending value → ending  [NO INPUT ID — not on the inputs tab] · money in → contributions  [NO INPUT ID — not on the inputs tab] · money out → withdrawals  [NO INPUT ID — not on the inputs tab] · dividends → dividends  [NO INPUT ID — not on the inputs tab] · interest → interest  [NO INPUT ID — not on the inputs tab] · debt paid down → debtPrincipal  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -12197,7 +14798,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>the holdings → positions · prices → priceOf(ticker) · the chosen chip → period · today → now</t>
+          <t>the holdings → positions  [NO INPUT ID — not on the inputs tab] · prices → priceOf(ticker)  [MK-XS-I-005] · the chosen chip → period  [NO INPUT ID — not on the inputs tab] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -12298,7 +14899,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>the holdings → positions · prices → priceOf(ticker) · the chosen chip → period · today → now</t>
+          <t>the holdings → positions  [NO INPUT ID — not on the inputs tab] · prices → priceOf(ticker)  [MK-XS-I-005] · the chosen chip → period  [NO INPUT ID — not on the inputs tab] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -12399,7 +15000,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>the holdings → positions · prices → priceOf(ticker) · the chosen chip → period · today → now</t>
+          <t>the holdings → positions  [NO INPUT ID — not on the inputs tab] · prices → priceOf(ticker)  [MK-XS-I-005] · the chosen chip → period  [NO INPUT ID — not on the inputs tab] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -12497,7 +15098,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>each holding's benchmark return → rows[].benchReturn · its value → rows[].marketValue</t>
+          <t>each holding's benchmark return → rows[].benchReturn  [NO INPUT ID — not on the inputs tab] · its value → rows[].marketValue  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -12700,7 +15301,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>the amount → amount · where it sat → fromSeries · where it might have gone → toSeries · how far back → months</t>
+          <t>the amount → amount  [MK-XS-I-008] · where it sat → fromSeries  [NO INPUT ID — not on the inputs tab] · where it might have gone → toSeries  [NO INPUT ID — not on the inputs tab] · how far back → months  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -12801,7 +15402,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>the amount → amount · where it sat → fromSeries · where it might have gone → toSeries · how far back → months</t>
+          <t>the amount → amount  [MK-XS-I-008] · where it sat → fromSeries  [NO INPUT ID — not on the inputs tab] · where it might have gone → toSeries  [NO INPUT ID — not on the inputs tab] · how far back → months  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -12902,7 +15503,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>the amount → amount · where it sat → fromSeries · where it might have gone → toSeries · how far back → months</t>
+          <t>the amount → amount  [MK-XS-I-008] · where it sat → fromSeries  [NO INPUT ID — not on the inputs tab] · where it might have gone → toSeries  [NO INPUT ID — not on the inputs tab] · how far back → months  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -13322,7 +15923,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>their age → birthYear or age · what they spend → monthlySpending · money that counts toward retirement → NEST_EGG</t>
+          <t>their age → birthYear or age  [MK-XS-I-017] · what they spend → monthlySpending  [MK-XS-I-024] · money that counts toward retirement → NEST_EGG  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -13421,7 +16022,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>their age → birthYear or age · what they spend → monthlySpending · money that counts toward retirement → NEST_EGG</t>
+          <t>their age → birthYear or age  [MK-XS-I-017] · what they spend → monthlySpending  [MK-XS-I-024] · money that counts toward retirement → NEST_EGG  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -14008,7 +16609,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>their age → birthYear · the pot → NEST_EGG · return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED · spending → RETIREMENT_SPENDING · guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE · money to leave behind → legacyTarget · their own overrides → the Plan screen</t>
+          <t>their age → birthYear  [MK-XS-I-017] · the pot → NEST_EGG  [NO INPUT ID — not on the inputs tab] · return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED  [NO INPUT ID — not on the inputs tab] · spending → RETIREMENT_SPENDING  [MK-XS-I-024] · guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE  [NO INPUT ID — not on the inputs tab] · money to leave behind → legacyTarget  [NO INPUT ID — not on the inputs tab] · their own overrides → the Plan screen  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -14106,7 +16707,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>the answer → the retirement-spending question · where they will live → the location answer</t>
+          <t>the answer → the retirement-spending question  [MK-XS-I-024] · where they will live → the location answer  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -14307,7 +16908,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>their age → birthYear · the pot → NEST_EGG · return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED · spending → RETIREMENT_SPENDING · guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE · money to leave behind → legacyTarget · their own overrides → the Plan screen</t>
+          <t>their age → birthYear  [MK-XS-I-017] · the pot → NEST_EGG  [NO INPUT ID — not on the inputs tab] · return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED  [NO INPUT ID — not on the inputs tab] · spending → RETIREMENT_SPENDING  [MK-XS-I-024] · guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE  [NO INPUT ID — not on the inputs tab] · money to leave behind → legacyTarget  [NO INPUT ID — not on the inputs tab] · their own overrides → the Plan screen  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -14802,7 +17403,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>the account → a · when the value was set → value_as_of · today → now</t>
+          <t>the account → a  [NO INPUT ID — not on the inputs tab] · when the value was set → value_as_of  [NO INPUT ID — not on the inputs tab] · today → now  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -14908,7 +17509,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>statement amount at their full retirement age (typed from their ssa.gov statement) → statement monthly · claim age (the slider) → the factor's input · birth year (setup) → the anchor</t>
+          <t>statement amount at their full retirement age (typed from their ssa.gov statement) → statement monthly  [MK-XS-I-008, MK-XS-I-018, MK-XS-I-020] · claim age (the slider) → the factor's input  [MK-XS-I-021] · birth year (setup) → the anchor  [MK-XS-I-017]</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -15009,7 +17610,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>do they receive it now → incomeSources · the amounts → retirementIncomeMonthly</t>
+          <t>do they receive it now → incomeSources  [NO INPUT ID — not on the inputs tab] · the amounts → retirementIncomeMonthly  [MK-XS-I-008]</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -15111,7 +17712,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>claim age (the slider, 62–70) → months early or late vs their full retirement age · birth year (their setup answer) → the full retirement age it anchors to · statement amount at their full retirement age (typed from their ssa.gov statement) → statement monthly · claim age (the slider) → the factor's input · birth year (setup) → the anchor</t>
+          <t>claim age (the slider, 62–70) → months early or late vs their full retirement age  [MK-XS-I-018, MK-XS-I-021] · birth year (their setup answer) → the full retirement age it anchors to  [MK-XS-I-017, MK-XS-I-018] · statement amount at their full retirement age (typed from their ssa.gov statement) → statement monthly  [MK-XS-I-008, MK-XS-I-018, MK-XS-I-020] · claim age (the slider) → the factor's input  [MK-XS-I-021] · birth year (setup) → the anchor  [MK-XS-I-017]</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -15805,7 +18406,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>the same inputs → inp</t>
+          <t>the same inputs → inp  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -16105,7 +18706,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>their age → birthYear · the pot → NEST_EGG · return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED · spending → RETIREMENT_SPENDING · guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE · money to leave behind → legacyTarget · their own overrides → the Plan screen</t>
+          <t>their age → birthYear  [MK-XS-I-017] · the pot → NEST_EGG  [NO INPUT ID — not on the inputs tab] · return and swing → EXPECTED_RETURN_BLENDED, EXPECTED_SWING_BLENDED  [NO INPUT ID — not on the inputs tab] · spending → RETIREMENT_SPENDING  [MK-XS-I-024] · guaranteed income → RETIREMENT_INCOME, SS_BENEFIT_AT_AGE  [NO INPUT ID — not on the inputs tab] · money to leave behind → legacyTarget  [NO INPUT ID — not on the inputs tab] · their own overrides → the Plan screen  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -16209,7 +18810,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>every debt → debts · rates → interest_rate_apr · payments → the minimum and chosen payments</t>
+          <t>every debt → debts  [NO INPUT ID — not on the inputs tab] · rates → interest_rate_apr  [MK-XS-I-015] · payments → the minimum and chosen payments  [MK-XS-I-016]</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -16410,7 +19011,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>do they receive it now → incomeSources · the amounts → retirementIncomeMonthly</t>
+          <t>do they receive it now → incomeSources  [NO INPUT ID — not on the inputs tab] · the amounts → retirementIncomeMonthly  [MK-XS-I-008]</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -16518,7 +19119,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>the same inputs → inp</t>
+          <t>the same inputs → inp  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -16627,7 +19228,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>everything → WILL_IT_LAST_INPUTS · is a range wanted → withBand</t>
+          <t>everything → WILL_IT_LAST_INPUTS  [NO INPUT ID — not on the inputs tab] · is a range wanted → withBand  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -17936,7 +20537,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -18035,7 +20636,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -18134,7 +20735,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -18331,7 +20932,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>each rental → rentalList</t>
+          <t>each rental → rentalList  [MK-XS-I-023]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -18430,7 +21031,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>do they receive it now → incomeSources · the amounts → retirementIncomeMonthly</t>
+          <t>do they receive it now → incomeSources  [NO INPUT ID — not on the inputs tab] · the amounts → retirementIncomeMonthly  [MK-XS-I-008]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -18630,7 +21231,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>the categories → spendCats · or the three summary figures → b_fixed, b_nonmonthly, b_flexible</t>
+          <t>the categories → spendCats  [NO INPUT ID — not on the inputs tab] · or the three summary figures → b_fixed, b_nonmonthly, b_flexible  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -18728,7 +21329,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>the categories → spendCats · or the three summary figures → b_fixed, b_nonmonthly, b_flexible</t>
+          <t>the categories → spendCats  [NO INPUT ID — not on the inputs tab] · or the three summary figures → b_fixed, b_nonmonthly, b_flexible  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -18827,7 +21428,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>the categories → SPENDING_BY_KIND · the single figure → monthlySpending</t>
+          <t>the categories → SPENDING_BY_KIND  [MK-XS-I-024] · the single figure → monthlySpending  [MK-XS-I-024, MK-XS-I-030]</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -19227,7 +21828,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>the categories → spendCats · or the three summary figures → b_fixed, b_nonmonthly, b_flexible · shape → paymentShape · minimum → minimum_monthly_payment · chosen → monthly_payment</t>
+          <t>the categories → spendCats  [NO INPUT ID — not on the inputs tab] · or the three summary figures → b_fixed, b_nonmonthly, b_flexible  [NO INPUT ID — not on the inputs tab] · shape → paymentShape  [NO INPUT ID — not on the inputs tab] · minimum → minimum_monthly_payment  [MK-XS-I-016] · chosen → monthly_payment  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -19523,7 +22124,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>the same inputs → inp</t>
+          <t>the same inputs → inp  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -19627,7 +22228,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>each source → ri_ss · ri_pension · ri_withdrawals · ri_rmd · ri_annuities · ri_other · and how often each arrives → the matching frequency</t>
+          <t>each source → ri_ss  [NO INPUT ID — not on the inputs tab] · ri_pension  [MK-XS-I-022] · ri_withdrawals  [NO INPUT ID — not on the inputs tab] · ri_rmd  [NO INPUT ID — not on the inputs tab] · ri_annuities  [NO INPUT ID — not on the inputs tab] · ri_other  [NO INPUT ID — not on the inputs tab] · and how often each arrives → the matching frequency  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -19726,7 +22327,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>do they receive it now → incomeSources · the amounts → retirementIncomeMonthly</t>
+          <t>do they receive it now → incomeSources  [NO INPUT ID — not on the inputs tab] · the amounts → retirementIncomeMonthly  [MK-XS-I-008]</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -20029,7 +22630,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -21237,7 +23838,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>the categories → SPENDING_BY_KIND · the single figure → monthlySpending</t>
+          <t>the categories → SPENDING_BY_KIND  [MK-XS-I-024] · the single figure → monthlySpending  [MK-XS-I-024, MK-XS-I-030]</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -21638,7 +24239,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -21737,7 +24338,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -21836,7 +24437,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>each part → its own engine above</t>
+          <t>each part → its own engine above  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -21934,7 +24535,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>the match → employerMatchValue · percent or dollars → employerMatchMode · their own contribution → c_401k</t>
+          <t>the match → employerMatchValue  [NO INPUT ID — not on the inputs tab] · percent or dollars → employerMatchMode  [NO INPUT ID — not on the inputs tab] · their own contribution → c_401k  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -22134,7 +24735,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>each account's class → assetClassOf · each account's money → balance · each account's class → assetClassOf · each account's money → balance</t>
+          <t>each account's class → assetClassOf  [NO INPUT ID — not on the inputs tab] · each account's money → balance  [MK-XS-I-001] · each account's class → assetClassOf  [NO INPUT ID — not on the inputs tab] · each account's money → balance  [MK-XS-I-001]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -22640,7 +25241,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>the categories → spendCats · or the three summary figures → b_fixed, b_nonmonthly, b_flexible</t>
+          <t>the categories → spendCats  [NO INPUT ID — not on the inputs tab] · or the three summary figures → b_fixed, b_nonmonthly, b_flexible  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -23135,7 +25736,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>the categories → SPENDING_BY_KIND · the single figure → monthlySpending</t>
+          <t>the categories → SPENDING_BY_KIND  [MK-XS-I-024] · the single figure → monthlySpending  [MK-XS-I-024, MK-XS-I-030]</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -23233,7 +25834,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>gross → gross · how they file → status</t>
+          <t>gross → gross  [NO INPUT ID — not on the inputs tab] · how they file → status  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -23335,7 +25936,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>gross → gross · how they file → status</t>
+          <t>gross → gross  [NO INPUT ID — not on the inputs tab] · how they file → status  [NO INPUT ID — not on the inputs tab]</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">

</xml_diff>

<commit_message>
Dependencies named by identifier and output, and the rule against generating one list from the other
The dependency column now names each engine it leans on by ITS identifier
and by the output it gives - MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) gives
what kind of thing an account is - so a chain can be followed without
knowing a single engine by name. Sixty-four rows name a dependency.

The founder rejected generating the engine input lists from the inputs
tab, and he is right: agreement by construction hides the failure that
matters, an input an engine reads that nobody ever captured. The orphan
would vanish into the generated list and the wrong number would reach the
screen with nothing flagged. Both records stay independent and a
reconciliation engine checks them as a build gate. Written into the
objectives standard and added to the specification as S18.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -824,12 +824,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engines it depends on (S11)</t>
+          <t>COLUMN — Dependency (S11)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>The engines this one calls, read from the code itself. "None found" means it reads raw values only.</t>
+          <t>The engines this one leans on, each named by ITS identifier and by the output it gives. Read from the code itself, never from a document. "None" means the engine reads raw inputs only.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MK-XS-E-001 · MK-XS-E-003 · MK-NW-E-004 · MK-PL-E-008</t>
+          <t>MK-XS-E-001 · MK-XS-E-009 · MK-NW-E-004 · MK-PL-E-006</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MK-PL-E-008</t>
+          <t>MK-PL-E-006</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MK-NW-E-006</t>
+          <t>MK-XS-E-015</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>MK-NW-E-023 · MK-NW-E-024</t>
+          <t>MK-XS-E-022 · MK-NW-E-022</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>MK-HM-E-001 · MK-NW-E-023</t>
+          <t>MK-HM-E-001 · MK-NW-E-022</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>MK-NW-E-025 · MK-NW-E-028</t>
+          <t>MK-NW-E-023 · MK-NW-E-026</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>MK-NW-E-016</t>
+          <t>MK-NW-E-015</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>MK-NW-E-017 · MK-NW-E-020</t>
+          <t>MK-NW-E-016 · MK-NW-E-019</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MK-NW-E-018 · MK-NW-E-019</t>
+          <t>MK-NW-E-017 · MK-NW-E-018</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>MK-NW-E-007</t>
+          <t>MK-NW-E-006</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>MK-PL-E-018</t>
+          <t>MK-PL-E-015</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>MK-NW-E-008</t>
+          <t>MK-NW-E-007</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>MK-PL-E-009</t>
+          <t>MK-XS-E-040</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>MK-XS-E-002 · MK-NW-E-010</t>
+          <t>MK-XS-E-007 · MK-NW-E-009</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>MK-PL-E-004</t>
+          <t>MK-XS-E-006</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>MK-PL-E-009 · MK-PL-E-010</t>
+          <t>MK-XS-E-040 · MK-PL-E-007</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1931,7 +1931,11 @@
           <t>SS_CLAIM_FACTOR</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>MK-XS-E-046</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>VERIFIED 2026-08-22</t>
@@ -1966,7 +1970,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>MK-PL-E-010</t>
+          <t>MK-PL-E-007</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2003,7 +2007,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2040,7 +2044,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MK-CF-E-006 · MK-CF-E-007</t>
+          <t>MK-XS-E-021 · MK-CF-E-004</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2077,7 +2081,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MK-CF-E-007 · MK-MN-E-010</t>
+          <t>MK-CF-E-004 · MK-MN-E-010</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2188,7 +2192,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>MK-XS-E-002 · MK-NW-E-010</t>
+          <t>MK-XS-E-007 · MK-NW-E-009</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2225,7 +2229,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>MK-PL-E-004</t>
+          <t>MK-XS-E-006</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2262,7 +2266,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>MK-PL-E-015 · MK-MN-E-014</t>
+          <t>MK-PL-E-012 · MK-MN-E-014</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -6994,7 +6998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7011,7 +7015,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -7308,12 +7312,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>The engines it depends on — without it, build order and the one-door design cannot be worked out.</t>
+          <t>Each dependency named by ITS engine identifier and by the output it gives, so a chain can be followed without knowing any engine by name.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>COMPLETE — read from the code itself, not from any document. 90 rows name their dependencies; the rest read raw values only.</t>
+          <t>COMPLETE — read from the code itself, not from any document. 64 rows name a dependency by identifier; the rest read raw inputs only.</t>
         </is>
       </c>
     </row>
@@ -7428,42 +7432,64 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S16</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The duplication pass</t>
+          <t>The reconciliation engine</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Figures that are the same thing under two identifiers.</t>
+          <t>Both records kept independently and checked against each other as a build gate — an input an engine names that is on no row, an input declared that no engine names, an engine identifier that does not exist, an engine no metric reaches. Founder, 2026-08-25: never generate one list from the other; agreement by construction hides the orphan.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>COMPLETE — every group judged one at a time. 11 figures were being shown under 24 identifiers; the 13 folded rows now name the identifier that survives and why. 18 groups were checked and are NOT duplicates — one engine legitimately producing several figures — and say so, so the question is not asked twice. Two mis-assigned engines were found and recorded as findings.</t>
+          <t>NOT STARTED — the reconciliation tab is today a report, run by hand. It has to become code with a test.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>The duplication pass</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Figures that are the same thing under two identifiers.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>COMPLETE — every group judged one at a time. 11 figures were being shown under 24 identifiers; the 13 folded rows now name the identifier that survives and why. 18 groups were checked and are NOT duplicates — one engine legitimately producing several figures — and say so, so the question is not asked twice. Two mis-assigned engines were found and recorded as findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>S17</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Which screens are the 55-70 core</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>The agreed first scope has never been written down.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>READY FOR THE FOUNDER — the core_screens tab lists all 49 screens with my recommendation (39 in, 5 out, 5 borderline) and a column for his decision.</t>
         </is>
@@ -7497,7 +7523,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -7582,7 +7608,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -7705,7 +7731,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -7767,7 +7793,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MK-XS-E-002</t>
+          <t>MK-XS-E-007</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -7808,7 +7834,11 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>NEST_EGG · ODDS_DISPLAY · RETIREMENT_SPENDING · WILL_IT_LAST · WILL_IT_LAST_INPUTS</t>
+          <t>MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?
+MK-XS-E-003 (ODDS_DISPLAY) → The retirement odds a person actually sees. Answers: 0, 5, 10 … 100 — the exact simulation
+MK-XS-E-004 (RETIREMENT_SPENDING) → What will be spent each month in retirement?
+MK-XS-E-005 (WILL_IT_LAST) → Will my money last?
+MK-XS-E-006 (WILL_IT_LAST_INPUTS) → What goes into working out the odds?</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -7875,7 +7905,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>MK-XS-E-003</t>
+          <t>MK-XS-E-009</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -7915,7 +7945,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>ASSET_CLASS_OF_ACCOUNT</t>
+          <t>MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -7973,7 +8003,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MK-XS-E-004</t>
+          <t>MK-XS-E-010</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -8017,7 +8047,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -8075,7 +8105,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>MK-XS-E-005</t>
+          <t>MK-XS-E-011</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -8173,7 +8203,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MK-XS-E-006</t>
+          <t>MK-XS-E-012</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -8364,7 +8394,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -8449,7 +8479,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -8572,7 +8602,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>FETCH_PRICES</t>
+          <t>MK-XS-E-013 (FETCH_PRICES) → What are these holdings worth?</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -9196,7 +9226,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -9281,7 +9311,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -9406,7 +9436,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>SNAPSHOT_READ_ALL</t>
+          <t>MK-XS-E-014 (SNAPSHOT_READ_ALL) → What history do we hold?</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -9515,7 +9545,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -9624,7 +9654,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>SNAPSHOT_READ_ALL</t>
+          <t>MK-XS-E-014 (SNAPSHOT_READ_ALL) → What history do we hold?</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -9727,7 +9757,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -9825,7 +9855,8 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>ACCOUNT_SPLIT · ASSET_CLASS_OF_ACCOUNT</t>
+          <t>MK-XS-E-015 (ACCOUNT_SPLIT) → This one brokerage account holds several different things — how much of it is each?
+MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -9936,7 +9967,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -10039,7 +10070,8 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>ACCOUNT_SPLIT · ASSET_CLASS_OF_ACCOUNT</t>
+          <t>MK-XS-E-015 (ACCOUNT_SPLIT) → This one brokerage account holds several different things — how much of it is each?
+MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -10108,7 +10140,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MK-NW-E-006</t>
+          <t>MK-XS-E-015</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -10152,7 +10184,8 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>ASSET_CLASS_OF_ACCOUNT · CLASS_FROM_NAME_TEXT</t>
+          <t>MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?
+MK-XS-E-016 (CLASS_FROM_NAME_TEXT) → Reading the NAME alone, is this cash, a money-market fund, or a CD / T-bill?</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -10222,7 +10255,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>MK-NW-E-007</t>
+          <t>MK-NW-E-006</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -10264,7 +10297,8 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>DEBT_MINIMUM_TOTAL · DEBT_PAYMENTS_ACTUAL</t>
+          <t>MK-XS-E-017 (DEBT_MINIMUM_TOTAL) → What must I pay across all debts to stay current?
+MK-XS-E-018 (DEBT_PAYMENTS_ACTUAL) → What is actually going out on debt each month?</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -10322,7 +10356,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MK-NW-E-007</t>
+          <t>MK-NW-E-006</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -10364,7 +10398,8 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>DEBT_MINIMUM_TOTAL · DEBT_PAYMENTS_ACTUAL</t>
+          <t>MK-XS-E-017 (DEBT_MINIMUM_TOTAL) → What must I pay across all debts to stay current?
+MK-XS-E-018 (DEBT_PAYMENTS_ACTUAL) → What is actually going out on debt each month?</t>
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -10422,7 +10457,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MK-NW-E-008</t>
+          <t>MK-NW-E-007</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -10462,7 +10497,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>DEBT_SHAPE</t>
+          <t>MK-XS-E-019 (DEBT_SHAPE) → How is THIS debt repaid?</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -10520,7 +10555,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MK-NW-E-007</t>
+          <t>MK-NW-E-006</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -10562,7 +10597,8 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>DEBT_MINIMUM_TOTAL · DEBT_PAYMENTS_ACTUAL</t>
+          <t>MK-XS-E-017 (DEBT_MINIMUM_TOTAL) → What must I pay across all debts to stay current?
+MK-XS-E-018 (DEBT_PAYMENTS_ACTUAL) → What is actually going out on debt each month?</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -10714,7 +10750,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>MK-NW-E-009</t>
+          <t>MK-NW-E-008</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -10755,7 +10791,10 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>ACCOUNT_SPLIT · ASSET_CLASS_OF_ACCOUNT · READ_A_NUMBER · SPENDING_BY_KIND</t>
+          <t>MK-XS-E-015 (ACCOUNT_SPLIT) → This one brokerage account holds several different things — how much of it is each?
+MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-021 (SPENDING_BY_KIND) → What is spent each month, split by kind?</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -10821,7 +10860,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>MK-NW-E-010</t>
+          <t>MK-NW-E-009</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -10867,7 +10906,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>WILL_IT_LAST</t>
+          <t>MK-XS-E-005 (WILL_IT_LAST) → Will my money last?</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -10980,7 +11019,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
@@ -11042,7 +11081,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MK-NW-E-011</t>
+          <t>MK-NW-E-010</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -11085,7 +11124,8 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>DEBT_MINIMUM_TOTAL · DEBT_PAYMENTS_ACTUAL</t>
+          <t>MK-XS-E-017 (DEBT_MINIMUM_TOTAL) → What must I pay across all debts to stay current?
+MK-XS-E-018 (DEBT_PAYMENTS_ACTUAL) → What is actually going out on debt each month?</t>
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
@@ -11143,7 +11183,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MK-NW-E-012</t>
+          <t>MK-NW-E-011</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -11184,7 +11224,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -11254,7 +11294,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>MK-NW-E-013</t>
+          <t>MK-NW-E-012</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -11356,7 +11396,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>MK-NW-E-006</t>
+          <t>MK-XS-E-015</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -11400,7 +11440,8 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>ASSET_CLASS_OF_ACCOUNT · CLASS_FROM_NAME_TEXT</t>
+          <t>MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?
+MK-XS-E-016 (CLASS_FROM_NAME_TEXT) → Reading the NAME alone, is this cash, a money-market fund, or a CD / T-bill?</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -11466,7 +11507,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MK-NW-E-014</t>
+          <t>MK-NW-E-013</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -11564,7 +11605,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>MK-NW-E-015</t>
+          <t>MK-NW-E-014</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -11605,7 +11646,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -11663,7 +11704,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>MK-NW-E-016</t>
+          <t>MK-NW-E-015</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -11703,7 +11744,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -11771,7 +11812,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>MK-NW-E-017</t>
+          <t>MK-NW-E-016</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -11811,7 +11852,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -11877,7 +11918,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>MK-NW-E-018</t>
+          <t>MK-NW-E-017</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -11917,7 +11958,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -11975,7 +12016,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MK-NW-E-019</t>
+          <t>MK-NW-E-018</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -12017,7 +12058,8 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>BOND_COUPON · BOND_YEARS_LEFT</t>
+          <t>MK-NW-E-016 (BOND_COUPON) → How much income does this bond pay in a year?
+MK-NW-E-017 (BOND_YEARS_LEFT) → How long until this bond pays back?</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
@@ -12079,7 +12121,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>MK-NW-E-020</t>
+          <t>MK-NW-E-019</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -12119,7 +12161,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>BOND_COUPON</t>
+          <t>MK-NW-E-016 (BOND_COUPON) → How much income does this bond pay in a year?</t>
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
@@ -12177,7 +12219,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MK-NW-E-021</t>
+          <t>MK-NW-E-020</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -12275,7 +12317,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MK-NW-E-022</t>
+          <t>MK-NW-E-021</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -12373,7 +12415,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>MK-NW-E-023</t>
+          <t>MK-NW-E-022</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -12414,7 +12456,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>HOLDING_SHARES</t>
+          <t>MK-XS-E-022 (HOLDING_SHARES) → How many shares of this do I own?</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -12490,7 +12532,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>MK-NW-E-024</t>
+          <t>MK-XS-E-022</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -12530,7 +12572,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -12596,7 +12638,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>MK-NW-E-025</t>
+          <t>MK-NW-E-023</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -12636,7 +12678,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
@@ -12698,7 +12740,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>MK-NW-E-025</t>
+          <t>MK-NW-E-023</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -12738,7 +12780,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
@@ -12800,7 +12842,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>MK-NW-E-026</t>
+          <t>MK-NW-E-024</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -12898,7 +12940,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>MK-NW-E-027</t>
+          <t>MK-NW-E-025</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -12940,7 +12982,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -13006,7 +13048,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>MK-NW-E-028</t>
+          <t>MK-NW-E-026</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -13048,7 +13090,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
@@ -13114,7 +13156,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>MK-NW-E-028</t>
+          <t>MK-NW-E-026</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -13156,7 +13198,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -13218,7 +13260,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>MK-NW-E-029</t>
+          <t>MK-NW-E-027</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -13410,7 +13452,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>MK-NW-E-023</t>
+          <t>MK-NW-E-022</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -13451,7 +13493,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>HOLDING_SHARES</t>
+          <t>MK-XS-E-022 (HOLDING_SHARES) → How many shares of this do I own?</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -13521,7 +13563,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>MK-NW-E-016</t>
+          <t>MK-NW-E-015</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -13561,7 +13603,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -13623,7 +13665,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>MK-NW-E-016</t>
+          <t>MK-NW-E-015</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -13663,7 +13705,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -13725,7 +13767,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>MK-NW-E-017</t>
+          <t>MK-NW-E-016</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -13765,7 +13807,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P44" t="inlineStr"/>
@@ -13827,7 +13869,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>MK-NW-E-020</t>
+          <t>MK-NW-E-019</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -13867,7 +13909,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>BOND_COUPON</t>
+          <t>MK-NW-E-016 (BOND_COUPON) → How much income does this bond pay in a year?</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>
@@ -13925,7 +13967,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>MK-NW-E-030</t>
+          <t>MK-NW-E-028</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -13965,7 +14007,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>NOT DETERMINED</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -14181,7 +14223,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -14266,7 +14308,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -14392,7 +14434,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -14502,7 +14544,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -14608,7 +14650,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -14718,7 +14760,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -14823,7 +14865,16 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>BENCHMARK_FOR_KIND · HOLDING_COST_BASIS · HOLDING_FIRST_BOUGHT · HOLDING_MARKET_VALUE · HOLDING_TOTAL_ROI · HOLDING_UNREALISED_GAIN · PERIOD_RETURN · PERIOD_START_DATE · PRICE_LATEST · RETURN_SINCE_A_DATE</t>
+          <t>MK-XS-E-023 (BENCHMARK_FOR_KIND) → What should this holding be compared against?
+MK-NW-E-023 (HOLDING_COST_BASIS) → What did I pay for this in total?
+MK-XS-E-024 (HOLDING_FIRST_BOUGHT) → When did I first buy this?
+MK-NW-E-022 (HOLDING_MARKET_VALUE) → What is this holding worth right now?
+MK-XS-E-025 (HOLDING_TOTAL_ROI) → How much am I up on this in percentage terms, since I bought it?
+MK-XS-E-026 (HOLDING_UNREALISED_GAIN) → How much am I up or down on this?
+MK-XS-E-027 (PERIOD_RETURN) → What did this holding do over the chosen period?
+MK-XS-E-028 (PERIOD_START_DATE) → Which date does the chosen period start from?
+MK-XS-E-029 (PRICE_LATEST) → What is the most recent price we hold for this?
+MK-XS-E-030 (RETURN_SINCE_A_DATE) → What did this do between a given date and today?</t>
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -14924,7 +14975,16 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>BENCHMARK_FOR_KIND · HOLDING_COST_BASIS · HOLDING_FIRST_BOUGHT · HOLDING_MARKET_VALUE · HOLDING_TOTAL_ROI · HOLDING_UNREALISED_GAIN · PERIOD_RETURN · PERIOD_START_DATE · PRICE_LATEST · RETURN_SINCE_A_DATE</t>
+          <t>MK-XS-E-023 (BENCHMARK_FOR_KIND) → What should this holding be compared against?
+MK-NW-E-023 (HOLDING_COST_BASIS) → What did I pay for this in total?
+MK-XS-E-024 (HOLDING_FIRST_BOUGHT) → When did I first buy this?
+MK-NW-E-022 (HOLDING_MARKET_VALUE) → What is this holding worth right now?
+MK-XS-E-025 (HOLDING_TOTAL_ROI) → How much am I up on this in percentage terms, since I bought it?
+MK-XS-E-026 (HOLDING_UNREALISED_GAIN) → How much am I up or down on this?
+MK-XS-E-027 (PERIOD_RETURN) → What did this holding do over the chosen period?
+MK-XS-E-028 (PERIOD_START_DATE) → Which date does the chosen period start from?
+MK-XS-E-029 (PRICE_LATEST) → What is the most recent price we hold for this?
+MK-XS-E-030 (RETURN_SINCE_A_DATE) → What did this do between a given date and today?</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -15025,7 +15085,16 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>BENCHMARK_FOR_KIND · HOLDING_COST_BASIS · HOLDING_FIRST_BOUGHT · HOLDING_MARKET_VALUE · HOLDING_TOTAL_ROI · HOLDING_UNREALISED_GAIN · PERIOD_RETURN · PERIOD_START_DATE · PRICE_LATEST · RETURN_SINCE_A_DATE</t>
+          <t>MK-XS-E-023 (BENCHMARK_FOR_KIND) → What should this holding be compared against?
+MK-NW-E-023 (HOLDING_COST_BASIS) → What did I pay for this in total?
+MK-XS-E-024 (HOLDING_FIRST_BOUGHT) → When did I first buy this?
+MK-NW-E-022 (HOLDING_MARKET_VALUE) → What is this holding worth right now?
+MK-XS-E-025 (HOLDING_TOTAL_ROI) → How much am I up on this in percentage terms, since I bought it?
+MK-XS-E-026 (HOLDING_UNREALISED_GAIN) → How much am I up or down on this?
+MK-XS-E-027 (PERIOD_RETURN) → What did this holding do over the chosen period?
+MK-XS-E-028 (PERIOD_START_DATE) → Which date does the chosen period start from?
+MK-XS-E-029 (PRICE_LATEST) → What is the most recent price we hold for this?
+MK-XS-E-030 (RETURN_SINCE_A_DATE) → What did this do between a given date and today?</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -15123,7 +15192,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
@@ -15326,7 +15395,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>PRICE_FACTOR_OVER_WINDOW</t>
+          <t>MK-XS-E-031 (PRICE_FACTOR_OVER_WINDOW) → By what multiple did this price move over the last N months?</t>
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -15427,7 +15496,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>PRICE_FACTOR_OVER_WINDOW</t>
+          <t>MK-XS-E-031 (PRICE_FACTOR_OVER_WINDOW) → By what multiple did this price move over the last N months?</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -15528,7 +15597,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>PRICE_FACTOR_OVER_WINDOW</t>
+          <t>MK-XS-E-031 (PRICE_FACTOR_OVER_WINDOW) → By what multiple did this price move over the last N months?</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -15740,7 +15809,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -15825,7 +15894,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -15948,7 +16017,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>NEST_EGG</t>
+          <t>MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -16047,7 +16116,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>NEST_EGG</t>
+          <t>MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -16590,7 +16659,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MK-PL-E-004</t>
+          <t>MK-XS-E-006</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -16634,7 +16703,21 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>EFFECTIVE_TAX_RATE · EXPECTED_RETURN_BLENDED · EXPECTED_SWING_BLENDED · FILING_STATUS · GUARANTEED_OUTSIDE_STREAMS · MONTHLY_SAVING · NEST_EGG · REPORTED_RETURN · RETIREMENT_SPENDING · SPLIT_BY_HOW_IT_IS_TAXED · SS_BENEFIT_AT_AGE · STATE_TAX_RATE · SWING_FROM_RETURN · TAX_OVER65_COUNT · TOTAL_INCOME</t>
+          <t>MK-XS-E-032 (EFFECTIVE_TAX_RATE) → What share of my income actually goes in tax?
+MK-XS-E-033 (EXPECTED_RETURN_BLENDED) → What return should I expect on everything I hold together?
+MK-XS-E-034 (EXPECTED_SWING_BLENDED) → How much does a year's return typically swing around that average?
+MK-XS-E-035 (FILING_STATUS) → How does this person file?
+MK-XS-E-036 (GUARANTEED_OUTSIDE_STREAMS) → The plan's guaranteed-income input as separate streams of OUTSIDE money only. Answers: zer
+MK-XS-E-037 (MONTHLY_SAVING) → How much goes in each month?
+MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?
+MK-XS-E-038 (REPORTED_RETURN) → What return did the person say they actually earned over the past year?
+MK-XS-E-004 (RETIREMENT_SPENDING) → What will be spent each month in retirement?
+MK-XS-E-039 (SPLIT_BY_HOW_IT_IS_TAXED) → How is the retirement money split by the tax that will be owed on it?
+MK-XS-E-040 (SS_BENEFIT_AT_AGE) → The monthly Social Security check at a chosen claim age, in today's dollars. Answers: a wh
+MK-XS-E-041 (STATE_TAX_RATE) → What state tax rate applies?
+MK-XS-E-042 (SWING_FROM_RETURN) → How much might a year's return swing, judged from the return alone?
+MK-XS-E-043 (TAX_OVER65_COUNT) → How many people on the tax return are 65 or older — the input the over-65 deduction needs 
+MK-XS-E-044 (TOTAL_INCOME) → What is the whole household income for the year, before tax?</t>
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
@@ -16692,7 +16775,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>MK-PL-E-005</t>
+          <t>MK-XS-E-004</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -16732,7 +16815,8 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>COST_OF_LIVING · READ_A_NUMBER</t>
+          <t>MK-XS-E-045 (COST_OF_LIVING) → How much more or less does life cost where they plan to live?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -16790,7 +16874,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MK-PL-E-006</t>
+          <t>MK-PL-E-004</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -16889,7 +16973,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MK-PL-E-004</t>
+          <t>MK-XS-E-006</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -16933,7 +17017,21 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>EFFECTIVE_TAX_RATE · EXPECTED_RETURN_BLENDED · EXPECTED_SWING_BLENDED · FILING_STATUS · GUARANTEED_OUTSIDE_STREAMS · MONTHLY_SAVING · NEST_EGG · REPORTED_RETURN · RETIREMENT_SPENDING · SPLIT_BY_HOW_IT_IS_TAXED · SS_BENEFIT_AT_AGE · STATE_TAX_RATE · SWING_FROM_RETURN · TAX_OVER65_COUNT · TOTAL_INCOME</t>
+          <t>MK-XS-E-032 (EFFECTIVE_TAX_RATE) → What share of my income actually goes in tax?
+MK-XS-E-033 (EXPECTED_RETURN_BLENDED) → What return should I expect on everything I hold together?
+MK-XS-E-034 (EXPECTED_SWING_BLENDED) → How much does a year's return typically swing around that average?
+MK-XS-E-035 (FILING_STATUS) → How does this person file?
+MK-XS-E-036 (GUARANTEED_OUTSIDE_STREAMS) → The plan's guaranteed-income input as separate streams of OUTSIDE money only. Answers: zer
+MK-XS-E-037 (MONTHLY_SAVING) → How much goes in each month?
+MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?
+MK-XS-E-038 (REPORTED_RETURN) → What return did the person say they actually earned over the past year?
+MK-XS-E-004 (RETIREMENT_SPENDING) → What will be spent each month in retirement?
+MK-XS-E-039 (SPLIT_BY_HOW_IT_IS_TAXED) → How is the retirement money split by the tax that will be owed on it?
+MK-XS-E-040 (SS_BENEFIT_AT_AGE) → The monthly Social Security check at a chosen claim age, in today's dollars. Answers: a wh
+MK-XS-E-041 (STATE_TAX_RATE) → What state tax rate applies?
+MK-XS-E-042 (SWING_FROM_RETURN) → How much might a year's return swing, judged from the return alone?
+MK-XS-E-043 (TAX_OVER65_COUNT) → How many people on the tax return are 65 or older — the input the over-65 deduction needs 
+MK-XS-E-044 (TOTAL_INCOME) → What is the whole household income for the year, before tax?</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -16995,7 +17093,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MK-PL-E-007</t>
+          <t>MK-PL-E-005</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -17093,7 +17191,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>MK-PL-E-008</t>
+          <t>MK-PL-E-006</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -17289,7 +17387,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>MK-PL-E-008</t>
+          <t>MK-PL-E-006</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -17387,7 +17485,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>MK-NW-E-012</t>
+          <t>MK-NW-E-011</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -17428,7 +17526,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>None found in the code — it reads raw values only</t>
+          <t>None — this engine reads raw inputs only</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -17494,7 +17592,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MK-PL-E-009</t>
+          <t>MK-XS-E-040</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -17534,7 +17632,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>SS_CLAIM_FACTOR</t>
+          <t>MK-XS-E-046 (SS_CLAIM_FACTOR) → How much of the statement amount a claim age actually pays, anchored at the person's OWN f</t>
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
@@ -17594,7 +17692,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MK-PL-E-010</t>
+          <t>MK-PL-E-007</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -17635,7 +17733,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>RETIREMENT_INCOME</t>
+          <t>MK-XS-E-047 (RETIREMENT_INCOME) → How much retirement income arrives monthly?</t>
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
@@ -17697,7 +17795,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>MK-PL-E-011</t>
+          <t>MK-PL-E-008</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -17737,7 +17835,8 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>SS_CLAIM_FACTOR · SS_FULL_RETIREMENT_AGE</t>
+          <t>MK-XS-E-048 (SS_FULL_RETIREMENT_AGE) → The person's own Social Security full retirement age. Answers: 66 (born through 1954) · 66
+MK-XS-E-046 (SS_CLAIM_FACTOR) → How much of the statement amount a claim age actually pays, anchored at the person's OWN f</t>
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
@@ -17796,7 +17895,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>MK-PL-E-012</t>
+          <t>MK-PL-E-009</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -17895,7 +17994,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MK-PL-E-013</t>
+          <t>MK-PL-E-010</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -17993,7 +18092,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>MK-PL-E-014</t>
+          <t>MK-PL-E-011</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -18091,7 +18190,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>MK-PL-E-015</t>
+          <t>MK-PL-E-012</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -18189,7 +18288,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>MK-PL-E-016</t>
+          <t>MK-PL-E-013</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -18287,7 +18386,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>MK-PL-E-014</t>
+          <t>MK-PL-E-011</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -18385,7 +18484,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MK-NW-E-010</t>
+          <t>MK-NW-E-009</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -18431,7 +18530,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>WILL_IT_LAST</t>
+          <t>MK-XS-E-005 (WILL_IT_LAST) → Will my money last?</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
@@ -18589,7 +18688,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MK-PL-E-017</t>
+          <t>MK-PL-E-014</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -18687,7 +18786,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>MK-PL-E-004</t>
+          <t>MK-XS-E-006</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -18731,7 +18830,21 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>EFFECTIVE_TAX_RATE · EXPECTED_RETURN_BLENDED · EXPECTED_SWING_BLENDED · FILING_STATUS · GUARANTEED_OUTSIDE_STREAMS · MONTHLY_SAVING · NEST_EGG · REPORTED_RETURN · RETIREMENT_SPENDING · SPLIT_BY_HOW_IT_IS_TAXED · SS_BENEFIT_AT_AGE · STATE_TAX_RATE · SWING_FROM_RETURN · TAX_OVER65_COUNT · TOTAL_INCOME</t>
+          <t>MK-XS-E-032 (EFFECTIVE_TAX_RATE) → What share of my income actually goes in tax?
+MK-XS-E-033 (EXPECTED_RETURN_BLENDED) → What return should I expect on everything I hold together?
+MK-XS-E-034 (EXPECTED_SWING_BLENDED) → How much does a year's return typically swing around that average?
+MK-XS-E-035 (FILING_STATUS) → How does this person file?
+MK-XS-E-036 (GUARANTEED_OUTSIDE_STREAMS) → The plan's guaranteed-income input as separate streams of OUTSIDE money only. Answers: zer
+MK-XS-E-037 (MONTHLY_SAVING) → How much goes in each month?
+MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?
+MK-XS-E-038 (REPORTED_RETURN) → What return did the person say they actually earned over the past year?
+MK-XS-E-004 (RETIREMENT_SPENDING) → What will be spent each month in retirement?
+MK-XS-E-039 (SPLIT_BY_HOW_IT_IS_TAXED) → How is the retirement money split by the tax that will be owed on it?
+MK-XS-E-040 (SS_BENEFIT_AT_AGE) → The monthly Social Security check at a chosen claim age, in today's dollars. Answers: a wh
+MK-XS-E-041 (STATE_TAX_RATE) → What state tax rate applies?
+MK-XS-E-042 (SWING_FROM_RETURN) → How much might a year's return swing, judged from the return alone?
+MK-XS-E-043 (TAX_OVER65_COUNT) → How many people on the tax return are 65 or older — the input the over-65 deduction needs 
+MK-XS-E-044 (TOTAL_INCOME) → What is the whole household income for the year, before tax?</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -18793,7 +18906,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>MK-NW-E-007</t>
+          <t>MK-NW-E-006</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -18835,7 +18948,8 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>DEBT_MINIMUM_TOTAL · DEBT_PAYMENTS_ACTUAL</t>
+          <t>MK-XS-E-017 (DEBT_MINIMUM_TOTAL) → What must I pay across all debts to stay current?
+MK-XS-E-018 (DEBT_PAYMENTS_ACTUAL) → What is actually going out on debt each month?</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -18897,7 +19011,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>MK-PL-E-018</t>
+          <t>MK-PL-E-015</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -18995,7 +19109,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>MK-PL-E-010</t>
+          <t>MK-PL-E-007</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -19036,7 +19150,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>RETIREMENT_INCOME</t>
+          <t>MK-XS-E-047 (RETIREMENT_INCOME) → How much retirement income arrives monthly?</t>
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
@@ -19098,7 +19212,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>MK-NW-E-010</t>
+          <t>MK-NW-E-009</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -19144,7 +19258,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>WILL_IT_LAST</t>
+          <t>MK-XS-E-005 (WILL_IT_LAST) → Will my money last?</t>
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
@@ -19212,7 +19326,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>MK-XS-E-002</t>
+          <t>MK-XS-E-007</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -19253,7 +19367,11 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>NEST_EGG · ODDS_DISPLAY · RETIREMENT_SPENDING · WILL_IT_LAST · WILL_IT_LAST_INPUTS</t>
+          <t>MK-XS-E-002 (NEST_EGG) → What is my retirement pot worth?
+MK-XS-E-003 (ODDS_DISPLAY) → The retirement odds a person actually sees. Answers: 0, 5, 10 … 100 — the exact simulation
+MK-XS-E-004 (RETIREMENT_SPENDING) → What will be spent each month in retirement?
+MK-XS-E-005 (WILL_IT_LAST) → Will my money last?
+MK-XS-E-006 (WILL_IT_LAST_INPUTS) → What goes into working out the odds?</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -19316,7 +19434,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>MK-PL-E-019</t>
+          <t>MK-PL-E-016</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -19414,7 +19532,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>MK-PL-E-020</t>
+          <t>MK-PL-E-017</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -19516,7 +19634,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>MK-PL-E-020</t>
+          <t>MK-PL-E-017</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -19874,7 +19992,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -19959,7 +20077,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -20330,7 +20448,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MK-XS-E-005</t>
+          <t>MK-XS-E-011</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -20521,7 +20639,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -20562,7 +20680,13 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -20620,7 +20744,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -20661,7 +20785,13 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -20719,7 +20849,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -20760,7 +20890,13 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
@@ -20818,7 +20954,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>MK-CF-E-003</t>
+          <t>MK-CF-E-002</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -20916,7 +21052,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MK-CF-E-004</t>
+          <t>MK-XS-E-051</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -20957,7 +21093,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>RENTALS</t>
+          <t>MK-XS-E-054 (RENTALS) → What rental properties are there, and what does each bring in?</t>
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -21015,7 +21151,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MK-PL-E-010</t>
+          <t>MK-PL-E-007</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -21056,7 +21192,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>RETIREMENT_INCOME</t>
+          <t>MK-XS-E-047 (RETIREMENT_INCOME) → How much retirement income arrives monthly?</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -21118,7 +21254,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MK-CF-E-005</t>
+          <t>MK-CF-E-003</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -21216,7 +21352,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>MK-CF-E-006</t>
+          <t>MK-XS-E-021</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -21256,7 +21392,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -21314,7 +21450,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>MK-CF-E-006</t>
+          <t>MK-XS-E-021</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -21354,7 +21490,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?</t>
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
@@ -21412,7 +21548,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>MK-CF-E-007</t>
+          <t>MK-CF-E-004</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -21453,7 +21589,8 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER · SPENDING_BY_KIND</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-021 (SPENDING_BY_KIND) → What is spent each month, split by kind?</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -21515,7 +21652,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>MK-CF-E-008</t>
+          <t>MK-CF-E-005</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -21613,7 +21750,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MK-CF-E-009</t>
+          <t>MK-CF-E-006</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -21711,7 +21848,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MK-XS-E-006</t>
+          <t>MK-XS-E-012</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -21813,7 +21950,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>MK-CF-E-010</t>
+          <t>MK-CF-E-007</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -21853,7 +21990,8 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>DEBT_SHAPE · READ_A_NUMBER</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-019 (DEBT_SHAPE) → How is THIS debt repaid?</t>
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
@@ -22005,7 +22143,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MK-CF-E-011</t>
+          <t>MK-CF-E-008</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -22103,7 +22241,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>MK-NW-E-010</t>
+          <t>MK-NW-E-009</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -22149,7 +22287,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>WILL_IT_LAST</t>
+          <t>MK-XS-E-005 (WILL_IT_LAST) → Will my money last?</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -22213,7 +22351,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>MK-CF-E-012</t>
+          <t>MK-XS-E-047</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -22253,7 +22391,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -22311,7 +22449,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>MK-PL-E-010</t>
+          <t>MK-PL-E-007</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -22352,7 +22490,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>RETIREMENT_INCOME</t>
+          <t>MK-XS-E-047 (RETIREMENT_INCOME) → How much retirement income arrives monthly?</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -22414,7 +22552,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>MK-CF-E-013</t>
+          <t>MK-CF-E-009</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -22512,7 +22650,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MK-CF-E-014</t>
+          <t>MK-CF-E-010</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -22614,7 +22752,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -22655,7 +22793,13 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
@@ -22713,7 +22857,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MK-CF-E-015</t>
+          <t>MK-CF-E-011</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -23071,7 +23215,7 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="37" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -23156,7 +23300,7 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Engines it depends on</t>
+          <t>Dependency — engine ID → the output it uses</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -23822,7 +23966,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>MK-CF-E-007</t>
+          <t>MK-CF-E-004</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -23863,7 +24007,8 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER · SPENDING_BY_KIND</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-021 (SPENDING_BY_KIND) → What is spent each month, split by kind?</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -24223,7 +24368,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -24264,7 +24409,13 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -24322,7 +24473,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -24363,7 +24514,13 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -24421,7 +24578,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>MK-CF-E-002</t>
+          <t>MK-XS-E-044</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -24462,7 +24619,13 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>EQUITY_THIS_YEAR · OTHER_INCOME · READ_A_NUMBER · RENTAL_INCOME_A_YEAR · RETIREMENT_INCOME_NOW · SALARY_A_YEAR · TIPS_A_YEAR</t>
+          <t>MK-XS-E-049 (EQUITY_THIS_YEAR) → How much equity vests this year?
+MK-XS-E-050 (OTHER_INCOME) → What else comes in?
+MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-051 (RENTAL_INCOME_A_YEAR) → What do the rentals net over a year?
+MK-PL-E-007 (RETIREMENT_INCOME_NOW) → How much retirement income is arriving TODAY?
+MK-XS-E-052 (SALARY_A_YEAR) → What is the salary for the year?
+MK-XS-E-053 (TIPS_A_YEAR) → What do tips come to over the year?</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -24560,7 +24723,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?</t>
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
@@ -24760,7 +24923,9 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>ACCOUNT_SPLIT · ASSET_CLASS_OF_ACCOUNT · IS_PHYSICAL_ASSET</t>
+          <t>MK-XS-E-055 (IS_PHYSICAL_ASSET) → Is this something physical you own rather than money you could spend?
+MK-XS-E-015 (ACCOUNT_SPLIT) → This one brokerage account holds several different things — how much of it is each?
+MK-XS-E-008 (ASSET_CLASS_OF_ACCOUNT) → What kind of thing is this account — cash, a bond, shares, or something else?</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -25226,7 +25391,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MK-CF-E-006</t>
+          <t>MK-XS-E-021</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -25266,7 +25431,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -25720,7 +25885,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>MK-CF-E-007</t>
+          <t>MK-CF-E-004</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -25761,7 +25926,8 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>READ_A_NUMBER · SPENDING_BY_KIND</t>
+          <t>MK-XS-E-020 (READ_A_NUMBER) → What number did the person actually type?
+MK-XS-E-021 (SPENDING_BY_KIND) → What is spent each month, split by kind?</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
@@ -25859,7 +26025,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>TAX_DEDUCTION</t>
+          <t>MK-XS-E-056 (TAX_DEDUCTION) → What amount of income is tax-free before the brackets start. Answers: $16,100 single · $32</t>
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
@@ -25961,7 +26127,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>TAX_DEDUCTION</t>
+          <t>MK-XS-E-056 (TAX_DEDUCTION) → What amount of income is tax-free before the brackets start. Answers: $16,100 single · $32</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>

</xml_diff>

<commit_message>
One word for one thing: feeder becomes dependent function
I introduced feeder without defining it, for something we had already
named. The columns and the wording now say dependent function
throughout - a function whose output is used by another function, in a
chain that ends at a screen.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -886,12 +886,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Every function that feeds it</t>
+          <t>COLUMN — Dependent functions</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Every function whose output reaches this one, however many steps away.</t>
+          <t>A dependent function is one whose output is used by another function, in a chain that ends at a screen. These columns list the dependent functions behind this one: those one step below it, how many there are in total, and all of them however many steps away.</t>
         </is>
       </c>
     </row>
@@ -10904,17 +10904,17 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Fed directly by (one step)</t>
+          <t>Dependent functions — one step below</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>How many functions feed it in total</t>
+          <t>Dependent functions — how many in total</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Every function that feeds it</t>
+          <t>Dependent functions — all of them</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -11254,12 +11254,12 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -11317,12 +11317,12 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -11380,12 +11380,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -11443,12 +11443,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -11704,12 +11704,12 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -11767,12 +11767,12 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -11830,12 +11830,12 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -12083,12 +12083,12 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -12146,12 +12146,12 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -12343,12 +12343,12 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -12406,12 +12406,12 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -12469,12 +12469,12 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -12980,12 +12980,12 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
@@ -13043,12 +13043,12 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
@@ -13106,12 +13106,12 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
@@ -13234,12 +13234,12 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
@@ -13486,12 +13486,12 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -13746,12 +13746,12 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -14335,12 +14335,12 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
@@ -14597,12 +14597,12 @@
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -15065,12 +15065,12 @@
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -15191,12 +15191,12 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L68" s="3" t="inlineStr">
@@ -15380,12 +15380,12 @@
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L71" s="3" t="inlineStr">
@@ -15443,12 +15443,12 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L72" s="3" t="inlineStr">
@@ -15707,12 +15707,12 @@
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L76" s="3" t="inlineStr">
@@ -15770,12 +15770,12 @@
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L77" s="3" t="inlineStr">
@@ -15833,12 +15833,12 @@
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L78" s="3" t="inlineStr">
@@ -16022,12 +16022,12 @@
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L81" s="3" t="inlineStr">
@@ -16085,12 +16085,12 @@
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
@@ -16148,12 +16148,12 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
@@ -16211,12 +16211,12 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
@@ -16274,12 +16274,12 @@
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L85" s="3" t="inlineStr">
@@ -16657,12 +16657,12 @@
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L91" s="3" t="inlineStr">
@@ -16720,12 +16720,12 @@
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L92" s="3" t="inlineStr">
@@ -16783,12 +16783,12 @@
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L93" s="3" t="inlineStr">
@@ -16846,12 +16846,12 @@
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L94" s="3" t="inlineStr">
@@ -16972,12 +16972,12 @@
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L96" s="3" t="inlineStr">
@@ -17035,12 +17035,12 @@
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L97" s="3" t="inlineStr">
@@ -17161,12 +17161,12 @@
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L99" s="3" t="inlineStr">
@@ -17413,12 +17413,12 @@
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L103" s="3" t="inlineStr">
@@ -17604,12 +17604,12 @@
       </c>
       <c r="J106" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L106" s="3" t="inlineStr">
@@ -17795,12 +17795,12 @@
       </c>
       <c r="J109" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L109" s="3" t="inlineStr">
@@ -17921,12 +17921,12 @@
       </c>
       <c r="J111" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L111" s="3" t="inlineStr">
@@ -18116,12 +18116,12 @@
       </c>
       <c r="J114" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K114" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L114" s="3" t="inlineStr">
@@ -18179,12 +18179,12 @@
       </c>
       <c r="J115" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K115" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L115" s="3" t="inlineStr">
@@ -18308,12 +18308,12 @@
       </c>
       <c r="J117" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L117" s="3" t="inlineStr">
@@ -19030,12 +19030,12 @@
       </c>
       <c r="J128" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K128" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L128" s="3" t="inlineStr">
@@ -19093,12 +19093,12 @@
       </c>
       <c r="J129" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K129" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L129" s="3" t="inlineStr">
@@ -19283,12 +19283,12 @@
       </c>
       <c r="J132" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L132" s="3" t="inlineStr">
@@ -19794,12 +19794,12 @@
       </c>
       <c r="J140" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L140" s="3" t="inlineStr">
@@ -19857,12 +19857,12 @@
       </c>
       <c r="J141" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L141" s="3" t="inlineStr">
@@ -19920,12 +19920,12 @@
       </c>
       <c r="J142" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L142" s="3" t="inlineStr">
@@ -19983,12 +19983,12 @@
       </c>
       <c r="J143" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L143" s="3" t="inlineStr">
@@ -20046,12 +20046,12 @@
       </c>
       <c r="J144" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L144" s="3" t="inlineStr">
@@ -20172,12 +20172,12 @@
       </c>
       <c r="J146" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L146" s="3" t="inlineStr">
@@ -20424,12 +20424,12 @@
       </c>
       <c r="J150" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K150" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L150" s="3" t="inlineStr">
@@ -20487,12 +20487,12 @@
       </c>
       <c r="J151" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K151" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L151" s="3" t="inlineStr">
@@ -20550,12 +20550,12 @@
       </c>
       <c r="J152" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L152" s="3" t="inlineStr">
@@ -20740,12 +20740,12 @@
       </c>
       <c r="J155" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L155" s="3" t="inlineStr">
@@ -21006,12 +21006,12 @@
       </c>
       <c r="J159" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L159" s="3" t="inlineStr">
@@ -21132,12 +21132,12 @@
       </c>
       <c r="J161" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K161" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L161" s="3" t="inlineStr">
@@ -21514,12 +21514,12 @@
       </c>
       <c r="J167" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K167" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L167" s="3" t="inlineStr">
@@ -21703,12 +21703,12 @@
       </c>
       <c r="J170" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K170" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L170" s="3" t="inlineStr">
@@ -21766,12 +21766,12 @@
       </c>
       <c r="J171" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K171" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L171" s="3" t="inlineStr">
@@ -21829,12 +21829,12 @@
       </c>
       <c r="J172" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K172" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L172" s="3" t="inlineStr">
@@ -22020,12 +22020,12 @@
       </c>
       <c r="J175" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K175" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L175" s="3" t="inlineStr">
@@ -22288,12 +22288,12 @@
       </c>
       <c r="J179" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K179" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L179" s="3" t="inlineStr">
@@ -22679,12 +22679,12 @@
       </c>
       <c r="J185" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K185" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L185" s="3" t="inlineStr">
@@ -22868,12 +22868,12 @@
       </c>
       <c r="J188" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K188" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L188" s="3" t="inlineStr">
@@ -23057,12 +23057,12 @@
       </c>
       <c r="J191" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K191" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L191" s="3" t="inlineStr">
@@ -23120,12 +23120,12 @@
       </c>
       <c r="J192" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K192" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L192" s="3" t="inlineStr">
@@ -23183,12 +23183,12 @@
       </c>
       <c r="J193" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K193" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L193" s="3" t="inlineStr">
@@ -23246,12 +23246,12 @@
       </c>
       <c r="J194" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K194" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L194" s="3" t="inlineStr">
@@ -23309,12 +23309,12 @@
       </c>
       <c r="J195" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K195" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L195" s="3" t="inlineStr">
@@ -23372,12 +23372,12 @@
       </c>
       <c r="J196" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K196" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L196" s="3" t="inlineStr">
@@ -23757,12 +23757,12 @@
       </c>
       <c r="J202" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K202" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L202" s="3" t="inlineStr">
@@ -23883,12 +23883,12 @@
       </c>
       <c r="J204" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K204" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L204" s="3" t="inlineStr">
@@ -24074,12 +24074,12 @@
       </c>
       <c r="J207" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K207" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L207" s="3" t="inlineStr">
@@ -24137,12 +24137,12 @@
       </c>
       <c r="J208" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K208" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L208" s="3" t="inlineStr">
@@ -24200,12 +24200,12 @@
       </c>
       <c r="J209" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K209" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L209" s="3" t="inlineStr">
@@ -24263,12 +24263,12 @@
       </c>
       <c r="J210" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K210" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L210" s="3" t="inlineStr">
@@ -24326,12 +24326,12 @@
       </c>
       <c r="J211" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K211" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L211" s="3" t="inlineStr">
@@ -24389,12 +24389,12 @@
       </c>
       <c r="J212" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K212" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L212" s="3" t="inlineStr">
@@ -24839,12 +24839,12 @@
       </c>
       <c r="J219" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K219" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L219" s="3" t="inlineStr">
@@ -24902,12 +24902,12 @@
       </c>
       <c r="J220" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K220" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L220" s="3" t="inlineStr">
@@ -25028,12 +25028,12 @@
       </c>
       <c r="J222" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K222" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L222" s="3" t="inlineStr">
@@ -25217,12 +25217,12 @@
       </c>
       <c r="J225" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K225" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L225" s="3" t="inlineStr">
@@ -25280,12 +25280,12 @@
       </c>
       <c r="J226" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K226" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L226" s="3" t="inlineStr">
@@ -25343,12 +25343,12 @@
       </c>
       <c r="J227" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K227" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L227" s="3" t="inlineStr">
@@ -25659,12 +25659,12 @@
       </c>
       <c r="J232" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K232" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L232" s="3" t="inlineStr">
@@ -25722,12 +25722,12 @@
       </c>
       <c r="J233" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K233" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L233" s="3" t="inlineStr">
@@ -25849,12 +25849,12 @@
       </c>
       <c r="J235" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K235" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L235" s="3" t="inlineStr">
@@ -25975,12 +25975,12 @@
       </c>
       <c r="J237" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K237" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L237" s="3" t="inlineStr">
@@ -26038,12 +26038,12 @@
       </c>
       <c r="J238" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K238" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L238" s="3" t="inlineStr">
@@ -26418,12 +26418,12 @@
       </c>
       <c r="J244" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K244" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L244" s="3" t="inlineStr">
@@ -26758,12 +26758,12 @@
       </c>
       <c r="J249" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K249" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L249" s="3" t="inlineStr">
@@ -26821,12 +26821,12 @@
       </c>
       <c r="J250" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K250" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L250" s="3" t="inlineStr">
@@ -26884,12 +26884,12 @@
       </c>
       <c r="J251" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K251" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L251" s="3" t="inlineStr">
@@ -27012,12 +27012,12 @@
       </c>
       <c r="J253" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K253" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L253" s="3" t="inlineStr">
@@ -27075,12 +27075,12 @@
       </c>
       <c r="J254" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K254" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L254" s="3" t="inlineStr">
@@ -27138,12 +27138,12 @@
       </c>
       <c r="J255" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K255" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L255" s="3" t="inlineStr">
@@ -27393,12 +27393,12 @@
       </c>
       <c r="J259" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K259" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L259" s="3" t="inlineStr">
@@ -27520,12 +27520,12 @@
       </c>
       <c r="J261" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K261" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L261" s="3" t="inlineStr">
@@ -27583,12 +27583,12 @@
       </c>
       <c r="J262" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K262" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L262" s="3" t="inlineStr">
@@ -27646,12 +27646,12 @@
       </c>
       <c r="J263" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K263" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L263" s="3" t="inlineStr">
@@ -27772,12 +27772,12 @@
       </c>
       <c r="J265" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K265" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L265" s="3" t="inlineStr">
@@ -27961,12 +27961,12 @@
       </c>
       <c r="J268" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K268" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L268" s="3" t="inlineStr">
@@ -28024,12 +28024,12 @@
       </c>
       <c r="J269" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K269" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L269" s="3" t="inlineStr">
@@ -28276,12 +28276,12 @@
       </c>
       <c r="J273" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K273" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L273" s="3" t="inlineStr">
@@ -28403,12 +28403,12 @@
       </c>
       <c r="J275" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K275" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L275" s="3" t="inlineStr">
@@ -28466,12 +28466,12 @@
       </c>
       <c r="J276" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K276" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L276" s="3" t="inlineStr">
@@ -28656,12 +28656,12 @@
       </c>
       <c r="J279" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K279" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L279" s="3" t="inlineStr">
@@ -28719,12 +28719,12 @@
       </c>
       <c r="J280" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K280" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L280" s="3" t="inlineStr">
@@ -28782,12 +28782,12 @@
       </c>
       <c r="J281" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K281" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L281" s="3" t="inlineStr">
@@ -29117,12 +29117,12 @@
       </c>
       <c r="J286" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K286" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L286" s="3" t="inlineStr">
@@ -29180,12 +29180,12 @@
       </c>
       <c r="J287" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K287" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L287" s="3" t="inlineStr">
@@ -29307,12 +29307,12 @@
       </c>
       <c r="J289" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K289" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L289" s="3" t="inlineStr">
@@ -29433,12 +29433,12 @@
       </c>
       <c r="J291" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K291" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L291" s="3" t="inlineStr">
@@ -29625,12 +29625,12 @@
       </c>
       <c r="J294" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K294" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L294" s="3" t="inlineStr">
@@ -29688,12 +29688,12 @@
       </c>
       <c r="J295" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K295" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L295" s="3" t="inlineStr">
@@ -29814,12 +29814,12 @@
       </c>
       <c r="J297" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K297" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L297" s="3" t="inlineStr">
@@ -29940,12 +29940,12 @@
       </c>
       <c r="J299" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K299" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L299" s="3" t="inlineStr">
@@ -30066,12 +30066,12 @@
       </c>
       <c r="J301" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K301" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L301" s="3" t="inlineStr">
@@ -30129,12 +30129,12 @@
       </c>
       <c r="J302" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K302" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L302" s="3" t="inlineStr">
@@ -30320,12 +30320,12 @@
       </c>
       <c r="J305" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K305" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L305" s="3" t="inlineStr">
@@ -30383,12 +30383,12 @@
       </c>
       <c r="J306" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K306" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L306" s="3" t="inlineStr">
@@ -30446,12 +30446,12 @@
       </c>
       <c r="J307" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K307" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L307" s="3" t="inlineStr">
@@ -30509,12 +30509,12 @@
       </c>
       <c r="J308" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K308" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L308" s="3" t="inlineStr">
@@ -30703,12 +30703,12 @@
       </c>
       <c r="J311" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K311" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L311" s="3" t="inlineStr">
@@ -30892,12 +30892,12 @@
       </c>
       <c r="J314" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K314" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L314" s="3" t="inlineStr">
@@ -30955,12 +30955,12 @@
       </c>
       <c r="J315" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K315" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L315" s="3" t="inlineStr">
@@ -31145,12 +31145,12 @@
       </c>
       <c r="J318" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K318" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L318" s="3" t="inlineStr">
@@ -31208,12 +31208,12 @@
       </c>
       <c r="J319" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K319" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L319" s="3" t="inlineStr">
@@ -31401,12 +31401,12 @@
       </c>
       <c r="J322" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K322" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L322" s="3" t="inlineStr">
@@ -31661,12 +31661,12 @@
       </c>
       <c r="J326" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K326" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L326" s="3" t="inlineStr">
@@ -31915,12 +31915,12 @@
       </c>
       <c r="J330" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K330" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L330" s="3" t="inlineStr">
@@ -31978,12 +31978,12 @@
       </c>
       <c r="J331" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K331" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L331" s="3" t="inlineStr">
@@ -32105,12 +32105,12 @@
       </c>
       <c r="J333" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K333" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L333" s="3" t="inlineStr">
@@ -32235,12 +32235,12 @@
       </c>
       <c r="J335" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K335" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L335" s="3" t="inlineStr">
@@ -32551,12 +32551,12 @@
       </c>
       <c r="J340" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K340" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L340" s="3" t="inlineStr">
@@ -32614,12 +32614,12 @@
       </c>
       <c r="J341" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K341" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L341" s="3" t="inlineStr">
@@ -32677,12 +32677,12 @@
       </c>
       <c r="J342" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K342" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L342" s="3" t="inlineStr">
@@ -32740,12 +32740,12 @@
       </c>
       <c r="J343" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K343" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L343" s="3" t="inlineStr">
@@ -32803,12 +32803,12 @@
       </c>
       <c r="J344" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K344" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L344" s="3" t="inlineStr">
@@ -33193,12 +33193,12 @@
       </c>
       <c r="J350" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K350" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L350" s="3" t="inlineStr">
@@ -33256,12 +33256,12 @@
       </c>
       <c r="J351" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K351" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L351" s="3" t="inlineStr">
@@ -33900,12 +33900,12 @@
       </c>
       <c r="J361" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K361" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L361" s="3" t="inlineStr">
@@ -33963,12 +33963,12 @@
       </c>
       <c r="J362" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K362" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L362" s="3" t="inlineStr">
@@ -34026,12 +34026,12 @@
       </c>
       <c r="J363" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K363" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L363" s="3" t="inlineStr">
@@ -34089,12 +34089,12 @@
       </c>
       <c r="J364" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K364" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L364" s="3" t="inlineStr">
@@ -34286,12 +34286,12 @@
       </c>
       <c r="J367" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K367" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L367" s="3" t="inlineStr">
@@ -34412,12 +34412,12 @@
       </c>
       <c r="J369" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K369" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L369" s="3" t="inlineStr">
@@ -34538,12 +34538,12 @@
       </c>
       <c r="J371" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K371" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L371" s="3" t="inlineStr">
@@ -34601,12 +34601,12 @@
       </c>
       <c r="J372" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K372" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L372" s="3" t="inlineStr">
@@ -34664,12 +34664,12 @@
       </c>
       <c r="J373" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K373" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L373" s="3" t="inlineStr">
@@ -34727,12 +34727,12 @@
       </c>
       <c r="J374" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K374" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L374" s="3" t="inlineStr">
@@ -34790,12 +34790,12 @@
       </c>
       <c r="J375" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K375" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L375" s="3" t="inlineStr">
@@ -34853,12 +34853,12 @@
       </c>
       <c r="J376" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K376" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L376" s="3" t="inlineStr">
@@ -34916,12 +34916,12 @@
       </c>
       <c r="J377" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K377" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L377" s="3" t="inlineStr">
@@ -35043,12 +35043,12 @@
       </c>
       <c r="J379" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K379" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L379" s="3" t="inlineStr">
@@ -35371,12 +35371,12 @@
       </c>
       <c r="J384" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K384" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L384" s="3" t="inlineStr">
@@ -35565,12 +35565,12 @@
       </c>
       <c r="J387" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K387" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L387" s="3" t="inlineStr">
@@ -35628,12 +35628,12 @@
       </c>
       <c r="J388" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K388" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L388" s="3" t="inlineStr">
@@ -36006,12 +36006,12 @@
       </c>
       <c r="J394" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K394" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L394" s="3" t="inlineStr">
@@ -36069,12 +36069,12 @@
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K395" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L395" s="3" t="inlineStr">
@@ -36132,12 +36132,12 @@
       </c>
       <c r="J396" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K396" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L396" s="3" t="inlineStr">
@@ -36195,12 +36195,12 @@
       </c>
       <c r="J397" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K397" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L397" s="3" t="inlineStr">
@@ -36321,12 +36321,12 @@
       </c>
       <c r="J399" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K399" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L399" s="3" t="inlineStr">
@@ -36384,12 +36384,12 @@
       </c>
       <c r="J400" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K400" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L400" s="3" t="inlineStr">
@@ -36447,12 +36447,12 @@
       </c>
       <c r="J401" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K401" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L401" s="3" t="inlineStr">
@@ -36581,12 +36581,12 @@
       </c>
       <c r="J403" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K403" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L403" s="3" t="inlineStr">
@@ -36715,12 +36715,12 @@
       </c>
       <c r="J405" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K405" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L405" s="3" t="inlineStr">
@@ -37041,12 +37041,12 @@
       </c>
       <c r="J410" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K410" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L410" s="3" t="inlineStr">
@@ -37246,12 +37246,12 @@
       </c>
       <c r="J413" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K413" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L413" s="3" t="inlineStr">
@@ -37504,12 +37504,12 @@
       </c>
       <c r="J417" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K417" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L417" s="3" t="inlineStr">
@@ -37567,12 +37567,12 @@
       </c>
       <c r="J418" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K418" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L418" s="3" t="inlineStr">
@@ -37695,12 +37695,12 @@
       </c>
       <c r="J420" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K420" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L420" s="3" t="inlineStr">
@@ -38148,12 +38148,12 @@
       </c>
       <c r="J427" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K427" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L427" s="3" t="inlineStr">
@@ -38211,12 +38211,12 @@
       </c>
       <c r="J428" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K428" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L428" s="3" t="inlineStr">
@@ -38409,12 +38409,12 @@
       </c>
       <c r="J431" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K431" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L431" s="3" t="inlineStr">
@@ -38472,12 +38472,12 @@
       </c>
       <c r="J432" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K432" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L432" s="3" t="inlineStr">
@@ -38599,12 +38599,12 @@
       </c>
       <c r="J434" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K434" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L434" s="3" t="inlineStr">
@@ -39051,12 +39051,12 @@
       </c>
       <c r="J441" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K441" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L441" s="3" t="inlineStr">
@@ -39185,12 +39185,12 @@
       </c>
       <c r="J443" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K443" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L443" s="3" t="inlineStr">
@@ -39248,12 +39248,12 @@
       </c>
       <c r="J444" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K444" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L444" s="3" t="inlineStr">
@@ -39644,12 +39644,12 @@
       </c>
       <c r="J450" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K450" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L450" s="3" t="inlineStr">
@@ -39707,12 +39707,12 @@
       </c>
       <c r="J451" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K451" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L451" s="3" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="J454" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K454" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L454" s="3" t="inlineStr">
@@ -39962,12 +39962,12 @@
       </c>
       <c r="J455" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K455" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L455" s="3" t="inlineStr">
@@ -40025,12 +40025,12 @@
       </c>
       <c r="J456" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K456" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L456" s="3" t="inlineStr">
@@ -40088,12 +40088,12 @@
       </c>
       <c r="J457" s="3" t="inlineStr">
         <is>
-          <t>Nothing — it is the start of its own chain</t>
+          <t>None — no dependent function stands behind it</t>
         </is>
       </c>
       <c r="K457" s="3" t="inlineStr">
         <is>
-          <t>Nothing feeds it — it reads its inputs and answers</t>
+          <t>No dependent function — it reads its inputs and answers</t>
         </is>
       </c>
       <c r="L457" s="3" t="inlineStr">

</xml_diff>

<commit_message>
A count per category, including what the code cannot say about itself
New functions_summary tab. Beside the count in each category, three
numbers worth knowing: how many functions are handed nothing and read no
stored data, how many are handed nothing but reach into the stored data,
and how many never declare what they give back.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -22,6 +22,7 @@
     <sheet name="reconciliation" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="engines" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="functions_from_code" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="functions_summary" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -80,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -93,6 +94,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -460,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -654,542 +658,554 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TAB — functions_from_code</t>
+          <t>TAB — functions_summary</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Every function in the calculation code, read from the code itself, sorted into the four categories by what it actually does. 1 ACTION does something and displays nothing. 2 DISPLAYED lands on a screen. 3 DEPENDENT feeds a chain that ends at a screen. 4 BRINGS DATA IN fetches from outside the app. A function that can reach a screen can put a wrong number in front of a person; one that cannot, cannot.</t>
+          <t>A count per category: how many functions there are, how many are handed nothing at all, how many are handed nothing but reach into the stored data, and how many never say what they give back.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TAB — reconciliation</t>
+          <t>TAB — functions_from_code</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>The input map checked in BOTH directions: what the inputs tab says uses each input, against what each engine actually names in its own input list. Where the two disagree the row says so. The section at the foot lists inputs an engine names that appear nowhere on the inputs tab.</t>
+          <t>Every function in the calculation code, read from the code itself, sorted into the four categories by what it actually does. 1 ACTION does something and displays nothing. 2 DISPLAYED lands on a screen. 3 DEPENDENT feeds a chain that ends at a screen. 4 BRINGS DATA IN fetches from outside the app. A function that can reach a screen can put a wrong number in front of a person; one that cannot, cannot.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TAB — core_screens</t>
+          <t>TAB — reconciliation</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Every screen in the app, its parent, my recommendation on whether it belongs to the 55-70 core, and a column for the founder to decide. Until this is decided, no row in the file can honestly claim to be in scope (S17).</t>
+          <t>The input map checked in BOTH directions: what the inputs tab says uses each input, against what each engine actually names in its own input list. Where the two disagree the row says so. The section at the foot lists inputs an engine names that appear nowhere on the inputs tab.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TAB — database</t>
+          <t>TAB — core_screens</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>What the app saves in the cloud: where each thing is stored, what it holds, which figures depend on it, how often it is written and at what grain. Also names what is deliberately NOT saved.</t>
+          <t>Every screen in the app, its parent, my recommendation on whether it belongs to the 55-70 core, and a column for the founder to decide. Until this is decided, no row in the file can honestly claim to be in scope (S17).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>TAB — database</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>What the app saves in the cloud: where each thing is stored, what it holds, which figures depend on it, how often it is written and at what grain. Also names what is deliberately NOT saved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>TAB — inputs</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>The raw values the engines need before any calculation happens.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Metric ID</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Parent Screen Name</t>
+          <t>COLUMN — Metric ID</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
+          <t>The identifier of the figure, per moneykeel_naming_spec_unique-identifier_v01.md. Given once, never changed, never reused.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Secondary Screen Name</t>
+          <t>COLUMN — Parent Screen Name</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
+          <t>One of: Home, Networth, Performance, Cashflow, Plan, Menu. Menu means reachable only from the menu.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name on Screen</t>
+          <t>COLUMN — Secondary Screen Name</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
+          <t>The screen reached from the parent, or NA when the figure is on the parent screen itself.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Metric</t>
+          <t>COLUMN — Name on Screen</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>The metric's name in the code.</t>
+          <t>The label copied exactly as it is worded on screen, including capitals. Where a figure wears different labels on different screens, all are listed.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Name of Underlying Engine</t>
+          <t>COLUMN — Name of Underlying Metric</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
+          <t>The metric's name in the code.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Inputs it needs (S02)</t>
+          <t>COLUMN — Name of Underlying Engine</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Every input the engine reads, named. Carried from the old master where it has a row there.</t>
+          <t>The engine that produces the figure. NOT IN OLD MASTER means the engine exists in the code but has no row in the old master file.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — What comes out (S04)</t>
+          <t>COLUMN — Inputs it needs (S02)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Dollars, a percentage, a date, a count; how it is held and how it is shown. Marked "derived by rule" where it was worked out from the label and formula rather than read from the engine — those need confirming.</t>
+          <t>Every input the engine reads, named. Carried from the old master where it has a row there.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — What it says when it cannot be computed (S05)</t>
+          <t>COLUMN — What comes out (S04)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>The refusal. Written where the engine has been read; NOT DETERMINED where it has not, rather than guessed.</t>
+          <t>Dollars, a percentage, a date, a count; how it is held and how it is shown. Marked "derived by rule" where it was worked out from the label and formula rather than read from the engine — those need confirming.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Grain (S06)</t>
+          <t>COLUMN — What it says when it cannot be computed (S05)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>One figure per what: holding, account, debt, goal, category, month, or person.</t>
+          <t>The refusal. Written where the engine has been read; NOT DETERMINED where it has not, rather than guessed.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Period (S07)</t>
+          <t>COLUMN — Grain (S06)</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>As of when, and over what window.</t>
+          <t>One figure per what: holding, account, debt, goal, category, month, or person.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Dependency (S11)</t>
+          <t>COLUMN — Period (S07)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>The engines this one leans on, each named by ITS identifier and by the output it gives. Read from the code itself, never from a document. "None" means the engine reads raw inputs only.</t>
+          <t>As of when, and over what window.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Secondary calculations and decisions the engine makes</t>
+          <t>COLUMN — Dependency (S11)</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>The judgements an engine must make BEFORE its headline figure exists: what class an asset is, what to call it on screen, which units apply, whether a value is fresh. Each of these is a formula of its own and needs its own row.</t>
+          <t>The engines this one leans on, each named by ITS identifier and by the output it gives. Read from the code itself, never from a document. "None" means the engine reads raw inputs only.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Function ID</t>
+          <t>COLUMN — Secondary calculations and decisions the engine makes</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Every function in the code carries one, MK-[family]-F-[number]. The family comes from the folder the code sits in.</t>
+          <t>The judgements an engine must make BEFORE its headline figure exists: what class an asset is, what to call it on screen, which units apply, whether a value is fresh. Each of these is a formula of its own and needs its own row.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — What it is handed / what it gives back</t>
+          <t>COLUMN — Function ID</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Read from the function's own signature: the values passed to it, whether it also reads the stored data, and what it returns. NOT DECLARED means the code does not say what comes back.</t>
+          <t>Every function in the code carries one, MK-[family]-F-[number]. The family comes from the folder the code sits in.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Label on screen</t>
+          <t>COLUMN — What it is handed / what it gives back</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>For a function whose answer is displayed, the words printed beside it, found by following the name the screen stores the answer in. NOT FOUND means a screen calls it but the label could not be traced automatically and needs reading.</t>
+          <t>Read from the function's own signature: the values passed to it, whether it also reads the stored data, and what it returns. NOT DECLARED means the code does not say what comes back.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Dependent functions</t>
+          <t>COLUMN — Label on screen</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>A dependent function is one whose output is used by another function, in a chain that ends at a screen. These columns list the dependent functions behind this one: those one step below it, how many there are in total, and all of them however many steps away.</t>
+          <t>For a function whose answer is displayed, the words printed beside it, found by following the name the screen stores the answer in. NOT FOUND means a screen calls it but the label could not be traced automatically and needs reading.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — The chain, ending in this function</t>
+          <t>COLUMN — Dependent functions</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Read left to right. The function that shows the answer sits at the END, and everything feeding it comes before it. A loop is marked where a chain turns back on itself. Chains are cut at five levels and eight paths, and say so.</t>
+          <t>A dependent function is one whose output is used by another function, in a chain that ends at a screen. These columns list the dependent functions behind this one: those one step below it, how many there are in total, and all of them however many steps away.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Same figure as (S16)</t>
+          <t>COLUMN — The chain, ending in this function</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Where the same figure appears under more than one identifier, the row names the surviving identifier and why. Nothing is deleted: identifiers are never reused, so a folded row stays visible and says what it became.</t>
+          <t>Read left to right. The function that shows the answer sits at the END, and everything feeding it comes before it. A loop is marked where a chain turns back on itself. Chains are cut at five levels and eight paths, and say so.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Questions for you (numbered)</t>
+          <t>COLUMN — Same figure as (S16)</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
+          <t>Where the same figure appears under more than one identifier, the row names the surviving identifier and why. Nothing is deleted: identifiers are never reused, so a folded row stays visible and says what it became.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — YOUR ANSWER — use the same number</t>
+          <t>COLUMN — Questions for you (numbered)</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
+          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Errors or findings to address</t>
+          <t>COLUMN — YOUR ANSWER — use the same number</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
+          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Decisions made (S03)</t>
+          <t>COLUMN — Errors or findings to address</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>The rulings and assumptions that govern this figure, each marked with WHOSE decision it was: [Founder] his own ruling, [The person] something the user set, [Built in] an assumption nobody chose on a screen — which is usually why a number looks wrong. The standing display and rounding rule applies to every row and is stated at the top of this tab.</t>
+          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (mathematical)</t>
+          <t>COLUMN — Decisions made (S03)</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
+          <t>The rulings and assumptions that govern this figure, each marked with WHOSE decision it was: [Founder] his own ruling, [The person] something the user set, [Built in] an assumption nobody chose on a screen — which is usually why a number looks wrong. The standing display and rounding rule applies to every row and is stated at the top of this tab.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (in words)</t>
+          <t>COLUMN — Formula (mathematical)</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
+          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engine ID</t>
+          <t>COLUMN — Formula (in words)</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
+          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Your name for it (72-metric file)</t>
+          <t>COLUMN — Engine ID</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
+          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Core screen?</t>
+          <t>COLUMN — Your name for it (72-metric file)</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
+          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Core screen?</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Row status</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
-      <c r="B52" s="3" t="inlineStr"/>
-    </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Input ID</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of a raw input, per the same standard.</t>
-        </is>
-      </c>
+      <c r="A53" s="2" t="inlineStr"/>
+      <c r="B53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Variable name</t>
+          <t>COLUMN — Input ID</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>What the raw value is called.</t>
+          <t>The identifier of a raw input, per the same standard.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Source</t>
+          <t>COLUMN — Variable name</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
+          <t>What the raw value is called.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which metric uses it</t>
+          <t>COLUMN — Source</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Every metric identifier that depends on this input.</t>
+          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Which metric uses it</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Every metric identifier that depends on this input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Which engine uses it</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Every engine identifier that reads this input.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
-      <c r="B58" s="3" t="inlineStr"/>
-    </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Complies with — naming</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
-        </is>
-      </c>
+      <c r="A59" s="2" t="inlineStr"/>
+      <c r="B59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Complies with — identifiers</t>
+          <t>Complies with — naming</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
+          <t>Complies with — identifiers</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>Complies with — objectives</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
-      <c r="B62" s="3" t="inlineStr"/>
-    </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>COVERAGE — screens read so far</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
-        </is>
-      </c>
+      <c r="A63" s="2" t="inlineStr"/>
+      <c r="B63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>COVERAGE — screens read so far</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
           <t>COVERAGE — what that means</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>Every screen in the app is listed on its tab. Only Home carries figures so far; the rest are marked NOT STARTED. A rising count is not completeness while screens remain unread.</t>
         </is>
@@ -46975,6 +46991,226 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Functions</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Handed nothing, and reads no stored data</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Handed nothing, but reads the stored data</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Does not declare what it gives back</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Neither: nothing in, nothing declared out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>A function handed nothing that reads no stored data has its answer from a constant, the clock, or something the code does not show. A function that does not declare what it gives back cannot be checked for returning the right shape. Both are counted here rather than described.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1 · ACTION</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2 · DISPLAYED</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>228</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2 · DISPLAYED (presentation only)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>3 · DEPENDENT</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>3 · DEPENDENT (feeds an action only)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>4 · BRINGS DATA IN</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>455</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Labels were being cut at the first bracket, and column I was wrong
The founder checked a row and found a label that appears on no screen:
"In". The real label is "In (received)". My pattern for capturing label
text allowed only letters, digits and a little punctuation, so every
label containing a bracket, a colon or a slash was truncated at that
character - the column was not merely incomplete, parts of it were
wrong.

Labels are now taken whole. A hundred of the two hundred and thirty-one
displayed functions carry one, and they read as they read on the screen:
"In (take-home)", "Your contribution (per month)", "Interest payments".

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -11292,7 +11292,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Bonds &amp; alternatives — recorded on their own pages   (PerformanceScreen.tsx)</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -11762,7 +11762,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>In   (CashFlowScreen.tsx)</t>
+          <t>In (take-home)   (CashFlowScreen.tsx)</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
@@ -12083,7 +12083,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Set a target date to track on-track / behind.   (GoalsScreen.tsx)</t>
+          <t>Allocate to this goal ›   (GoalsScreen.tsx)</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
@@ -12474,7 +12474,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Your contribution   (modules.tsx)</t>
+          <t>Your contribution (per month)   (modules.tsx)</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -13268,7 +13268,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Bonds &amp; alternatives — recorded on their own pages   (PerformanceScreen.tsx)</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -14051,7 +14051,7 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>You are   (HoldingDetailScreen.tsx)</t>
+          <t>Name (optional)   (PerformanceScreen.tsx) · You are   (HoldingDetailScreen.tsx)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Ending market value   (PerformanceScreen.tsx) · Wealth generated   (PerformanceScreen.tsx)</t>
+          <t>Ending market value   (PerformanceScreen.tsx) · Ending market value (today)   (PerformanceScreen.tsx) · Wealth generated   (PerformanceScreen.tsx)</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
@@ -16302,7 +16302,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>IF YOU SOLD TODAY   (HoldingDetailScreen.tsx)</t>
+          <t>Gain — long-term (held over 1 yr)   (HoldingDetailScreen.tsx) · Gain — short-term (under 1 yr)   (HoldingDetailScreen.tsx)</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
@@ -16380,7 +16380,7 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Annuity / other   (modules.tsx) · Capital needed   (modules.tsx) · Leave behind   (modules.tsx) · To fund from savings   (modules.tsx) · What are you saving for   (modules.tsx) · Your retirement outlook   (modules.tsx)</t>
+          <t>Annuity / other   (modules.tsx) · Capital needed   (modules.tsx) · Leave behind (your legacy goal)   (modules.tsx) · To fund from savings   (modules.tsx) · What are you saving for?   (modules.tsx) · Your retirement outlook   (modules.tsx)</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
@@ -18191,7 +18191,7 @@
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Your credit score (optional)   (CreditScreen.tsx)</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
@@ -18347,7 +18347,7 @@
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>Amount   (LookBackScreen.tsx) · Estimated benefit   (RetirementCockpit.tsx) · How much   (modules.tsx) · How much per month   (modules.tsx) · Leave blank to use a 40-hour week.   (modules.tsx) · Market price   (modules.tsx)</t>
+          <t>Amount   (LookBackScreen.tsx) · Break this into specific stocks, bonds, options…   (NetWorthScreen.tsx) · Estimated benefit   (RetirementCockpit.tsx) · HOW MUCH WILL YOU INVEST PER YEAR?   (modules.tsx) · How much   (modules.tsx) · How much (this disbursement)   (modules.tsx)</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
@@ -18425,7 +18425,7 @@
       </c>
       <c r="I96" s="3" t="inlineStr">
         <is>
-          <t>How long should your money last   (modules.tsx) · Operating expense / mo   (modules.tsx) · Projected to last to age   (modules.tsx) · Set by month   (modules.tsx) · Surplus by month   (modules.tsx) · Your contribution   (modules.tsx)</t>
+          <t>How long should your money last?   (modules.tsx) · Operating expense / mo   (modules.tsx) · Projected to last to age   (modules.tsx) · Set by month   (modules.tsx) · Surplus by month   (modules.tsx) · Your contribution (per month)   (modules.tsx)</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
@@ -18737,7 +18737,7 @@
       </c>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>Yield on today's value   (AccountDetailScreen.tsx)</t>
+          <t>Yield on today   (AccountDetailScreen.tsx)</t>
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr">
@@ -18971,7 +18971,7 @@
       </c>
       <c r="I103" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Add a debt →   (NetWorthScreen.tsx)</t>
         </is>
       </c>
       <c r="J103" s="3" t="inlineStr">
@@ -20154,7 +20154,7 @@
       </c>
       <c r="I118" s="3" t="inlineStr">
         <is>
-          <t>WHAT COUNTS TOWARD RETIREMENT   (PlanInputs.tsx)</t>
+          <t>Test retiring earlier, saving more, market ups &amp; downs.   (RetirementCockpit.tsx) · WHAT COUNTS TOWARD RETIREMENT   (PlanInputs.tsx) · What counts toward retirement?   (RetirementCockpit.tsx)</t>
         </is>
       </c>
       <c r="J118" s="3" t="inlineStr">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="I135" s="3" t="inlineStr">
         <is>
-          <t>Annual vesting cash flow   (modules.tsx) · Monthly   (modules.tsx) · Monthly cash flow   (modules.tsx)</t>
+          <t>Annual vesting cash flow   (modules.tsx) · Monthly (retirement)   (modules.tsx) · Monthly cash flow   (modules.tsx)</t>
         </is>
       </c>
       <c r="J135" s="3" t="inlineStr">
@@ -22453,7 +22453,7 @@
       </c>
       <c r="I147" s="3" t="inlineStr">
         <is>
-          <t>Annual vesting cash flow   (modules.tsx) · Annuity / other   (modules.tsx) · Available / yr   (modules.tsx) · Capital needed   (modules.tsx) · Critical   (modules.tsx) · Do you manage money with a partner   (modules.tsx)</t>
+          <t>Annual vesting cash flow   (modules.tsx) · Annuity / other   (modules.tsx) · Available / yr   (modules.tsx) · Capital needed   (modules.tsx) · Count money you receive to live on. We won't tax this.   (modules.tsx) · Critical   (modules.tsx)</t>
         </is>
       </c>
       <c r="J147" s="3" t="inlineStr">
@@ -23638,7 +23638,7 @@
       </c>
       <c r="I162" s="3" t="inlineStr">
         <is>
-          <t>Complete   (RewardsScreen.tsx)</t>
+          <t>Complete! 🎉   (RewardsScreen.tsx)</t>
         </is>
       </c>
       <c r="J162" s="3" t="inlineStr">
@@ -27820,7 +27820,7 @@
       </c>
       <c r="I215" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Pay off over (years)   (modules.tsx)</t>
         </is>
       </c>
       <c r="J215" s="3" t="inlineStr">
@@ -29778,7 +29778,7 @@
       </c>
       <c r="I240" s="3" t="inlineStr">
         <is>
-          <t>ACCOUNTS   (TaxOrganizerScreen.tsx) · Amount   (BudgetScreen.tsx) · Annual vesting cash flow   (modules.tsx) · Annuity / other   (modules.tsx) · Available / yr   (modules.tsx) · COUPON / YR   (BondsScreen.tsx)</t>
+          <t>ACCOUNTS (year-end)   (TaxOrganizerScreen.tsx) · Allocate to this goal ›   (GoalsScreen.tsx) · Amount   (BudgetScreen.tsx) · Annual vesting cash flow   (modules.tsx) · Annuity / other   (modules.tsx) · Available / yr   (modules.tsx)</t>
         </is>
       </c>
       <c r="J240" s="3" t="inlineStr">
@@ -31448,7 +31448,7 @@
       </c>
       <c r="I261" s="3" t="inlineStr">
         <is>
-          <t>WILL MY MONEY LAST   (HomeScreen.tsx)</t>
+          <t>WILL MY MONEY LAST?   (HomeScreen.tsx)</t>
         </is>
       </c>
       <c r="J261" s="3" t="inlineStr">
@@ -32462,7 +32462,7 @@
       </c>
       <c r="I274" s="3" t="inlineStr">
         <is>
-          <t>Extra / month   (BudgetScreen.tsx) · No budget yet   (BudgetScreen.tsx) · Payoff plan   (BudgetScreen.tsx) · Your monthly plan   (BudgetScreen.tsx)</t>
+          <t>Add any loans or credit cards to plan your payoff.   (BudgetScreen.tsx) · Extra / month   (BudgetScreen.tsx) · Extra / month (beyond minimums)   (GoalsScreen.tsx) · Income (take-home)   (BudgetScreen.tsx) · Payoff plan   (BudgetScreen.tsx) · Tap “Set limits” to plan what you'll spend, by category.   (BudgetScreen.tsx)</t>
         </is>
       </c>
       <c r="J274" s="3" t="inlineStr">
@@ -33254,7 +33254,7 @@
       </c>
       <c r="I284" s="3" t="inlineStr">
         <is>
-          <t>Your monthly plan   (BudgetScreen.tsx)</t>
+          <t>Income (take-home)   (BudgetScreen.tsx)</t>
         </is>
       </c>
       <c r="J284" s="3" t="inlineStr">
@@ -35142,7 +35142,7 @@
       </c>
       <c r="I308" s="3" t="inlineStr">
         <is>
-          <t>Certain months   (modules.tsx)</t>
+          <t>Certain months   (modules.tsx) · HOW MUCH WILL YOU INVEST PER YEAR?   (modules.tsx) · When does it land? (pick the months)   (modules.tsx) · When is it due? (pick the months)   (modules.tsx)</t>
         </is>
       </c>
       <c r="J308" s="3" t="inlineStr">
@@ -36084,7 +36084,7 @@
       </c>
       <c r="I320" s="3" t="inlineStr">
         <is>
-          <t>Everything in MoneyKeel   (TopBar.tsx) · WILL MY MONEY LAST   (HomeScreen.tsx)</t>
+          <t>WILL MY MONEY LAST?   (HomeScreen.tsx) · YOUR FIVE TABS — same order as the bar below   (TopBar.tsx)</t>
         </is>
       </c>
       <c r="J320" s="3" t="inlineStr">
@@ -37034,7 +37034,7 @@
       </c>
       <c r="I332" s="3" t="inlineStr">
         <is>
-          <t>Required Minimum Distributions   (RetirementCockpit.tsx) · WHAT IT BUYS LATER   (RothScreen.tsx) · Yours starts in   (RequiredWithdrawalsScreen.tsx)</t>
+          <t>Required Minimum Distributions   (RetirementCockpit.tsx) · Required withdrawal — first   (DrawSteerSheet.tsx) · WHAT IT BUYS LATER   (RothScreen.tsx) · Yours starts in   (RequiredWithdrawalsScreen.tsx)</t>
         </is>
       </c>
       <c r="J332" s="3" t="inlineStr">
@@ -37273,7 +37273,7 @@
       </c>
       <c r="I335" s="3" t="inlineStr">
         <is>
-          <t>Operating expense / mo   (modules.tsx) · Set by month   (modules.tsx) · Surplus by month   (modules.tsx) · Your contribution   (modules.tsx) · Your retirement outlook   (modules.tsx)</t>
+          <t>Operating expense / mo   (modules.tsx) · Set by month   (modules.tsx) · Surplus by month   (modules.tsx) · Your contribution (per month)   (modules.tsx) · Your retirement outlook   (modules.tsx)</t>
         </is>
       </c>
       <c r="J335" s="3" t="inlineStr">
@@ -37351,7 +37351,7 @@
       </c>
       <c r="I336" s="3" t="inlineStr">
         <is>
-          <t>Required Minimum Distributions   (RetirementCockpit.tsx) · Roth conversion   (RothScreen.tsx) · Suggested withdrawal order   (RetirementCockpit.tsx) · WHAT IT BUYS LATER   (RothScreen.tsx) · WHAT THIS IS   (RequiredWithdrawalsScreen.tsx) · Yours starts in   (RequiredWithdrawalsScreen.tsx)</t>
+          <t>Required Minimum Distributions   (RetirementCockpit.tsx) · Required withdrawal — first   (DrawSteerSheet.tsx) · Roth conversion   (RothScreen.tsx) · Suggested withdrawal order   (RetirementCockpit.tsx) · WHAT IT BUYS LATER   (RothScreen.tsx) · WHAT THIS IS   (RequiredWithdrawalsScreen.tsx)</t>
         </is>
       </c>
       <c r="J336" s="3" t="inlineStr">
@@ -37664,7 +37664,7 @@
       </c>
       <c r="I340" s="3" t="inlineStr">
         <is>
-          <t>Required Minimum Distributions   (RetirementCockpit.tsx)</t>
+          <t>Roth conversion window:   (RetirementCockpit.tsx)</t>
         </is>
       </c>
       <c r="J340" s="3" t="inlineStr">
@@ -41461,7 +41461,7 @@
       </c>
       <c r="I388" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Can I spend more?   (SpendMoreControl.tsx)</t>
         </is>
       </c>
       <c r="J388" s="3" t="inlineStr">
@@ -41617,7 +41617,7 @@
       </c>
       <c r="I390" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>When should I claim Social Security?   (ClaimAgeRow.tsx)</t>
         </is>
       </c>
       <c r="J390" s="3" t="inlineStr">
@@ -42639,7 +42639,7 @@
       </c>
       <c r="I403" s="3" t="inlineStr">
         <is>
-          <t>Everything in MoneyKeel   (TopBar.tsx)</t>
+          <t>YOUR FIVE TABS — same order as the bar below   (TopBar.tsx)</t>
         </is>
       </c>
       <c r="J403" s="3" t="inlineStr">
@@ -42717,7 +42717,7 @@
       </c>
       <c r="I404" s="3" t="inlineStr">
         <is>
-          <t>Itemized   (modules.tsx) · Net   (modules.tsx) · Net Worth   (modules.tsx) · Surplus / year   (modules.tsx) · Take-home   (modules.tsx) · Take-home / year   (modules.tsx)</t>
+          <t>Income (take-home)   (BudgetScreen.tsx) · Itemized   (modules.tsx) · Net   (modules.tsx) · Net Worth   (modules.tsx) · Surplus / year   (modules.tsx) · Take-home   (modules.tsx)</t>
         </is>
       </c>
       <c r="J404" s="3" t="inlineStr">
@@ -42881,7 +42881,7 @@
       </c>
       <c r="I406" s="3" t="inlineStr">
         <is>
-          <t>Required Minimum Distributions   (RetirementCockpit.tsx) · Suggested withdrawal order   (RetirementCockpit.tsx) · Where your money sits   (RetirementCockpit.tsx) · Yours starts in   (RequiredWithdrawalsScreen.tsx)</t>
+          <t>Healthcare:   (RetirementCockpit.tsx) · Required Minimum Distributions   (RetirementCockpit.tsx) · Required withdrawal — first   (DrawSteerSheet.tsx) · Roth conversion window:   (RetirementCockpit.tsx) · Suggested withdrawal order   (RetirementCockpit.tsx) · Where your money sits   (RetirementCockpit.tsx)</t>
         </is>
       </c>
       <c r="J406" s="3" t="inlineStr">
@@ -43282,7 +43282,7 @@
       </c>
       <c r="I411" s="3" t="inlineStr">
         <is>
-          <t>Self-employment income   (modules.tsx) · WHAT'S TAKEN OUT   (modules.tsx)</t>
+          <t>Count money you receive to live on. We won't tax this.   (modules.tsx) · Each month: tax · spending · savings   (modules.tsx) · How often?   (modules.tsx) · WHAT'S TAKEN OUT   (modules.tsx)</t>
         </is>
       </c>
       <c r="J411" s="3" t="inlineStr">
@@ -44008,7 +44008,7 @@
       </c>
       <c r="I420" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Activity ›   (PerformanceScreen.tsx)</t>
         </is>
       </c>
       <c r="J420" s="3" t="inlineStr">
@@ -44242,7 +44242,7 @@
       </c>
       <c r="I423" s="3" t="inlineStr">
         <is>
-          <t>DEBT-TO-INCOME   (GoalsScreen.tsx) · Your monthly plan   (BudgetScreen.tsx)</t>
+          <t>DEBT-TO-INCOME   (GoalsScreen.tsx) · Income (take-home)   (BudgetScreen.tsx)</t>
         </is>
       </c>
       <c r="J423" s="3" t="inlineStr">
@@ -44320,7 +44320,7 @@
       </c>
       <c r="I424" s="3" t="inlineStr">
         <is>
-          <t>Net Worth   (modules.tsx) · Operating expense / mo   (modules.tsx) · STUDENT LOAN OUTLOOK   (GoalsScreen.tsx) · Total income / yr   (modules.tsx) · Total value   (modules.tsx) · YOUR INCOME   (IncomeManagerScreen.tsx)</t>
+          <t>Net Worth   (modules.tsx) · Operating expense / mo   (modules.tsx) · Pay off over (years)   (modules.tsx) · STUDENT LOAN OUTLOOK   (GoalsScreen.tsx) · Total income / yr   (modules.tsx) · Total value   (modules.tsx)</t>
         </is>
       </c>
       <c r="J424" s="3" t="inlineStr">
@@ -46563,7 +46563,7 @@
       </c>
       <c r="I452" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND — a screen calls it but no label was found near the call</t>
+          <t>Why this order?   (CashFlowScreen.tsx) · Why? ›   (CashFlowScreen.tsx)</t>
         </is>
       </c>
       <c r="J452" s="3" t="inlineStr">
@@ -46644,7 +46644,7 @@
       </c>
       <c r="I453" s="3" t="inlineStr">
         <is>
-          <t>From your portfolio   (RetirementCockpit.tsx) · You plan to spend   (RetirementCockpit.tsx)</t>
+          <t>From your portfolio   (RetirementCockpit.tsx) · WILL YOUR MONEY LAST?   (RetirementCockpit.tsx) · You plan to spend   (RetirementCockpit.tsx)</t>
         </is>
       </c>
       <c r="J453" s="3" t="inlineStr">

</xml_diff>

<commit_message>
The why column said nothing; it now says what each function is for
It restated the category - a screen calls it, so its answer is on a
screen - which the category column already said. Replaced with the
purpose of the function in one sentence, taken from the note the author
wrote above it in the code, falling back to the old inventory, and
saying NOT DETERMINED where neither exists rather than inventing one.

Three hundred and nineteen functions carry their own note. The rest are
named honestly as needing a read.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -902,310 +902,322 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — What it is handed / what it gives back</t>
+          <t>COLUMN — What it is for</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Read from the function's own signature: the values passed to it, whether it also reads the stored data, and what it returns. NOT DECLARED means the code does not say what comes back.</t>
+          <t>The purpose of the function in one sentence, taken from the note written above it in the code, or from the old inventory when the code carries none. NOT DETERMINED where neither exists — never invented.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Label on screen</t>
+          <t>COLUMN — What it is handed / what it gives back</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>For a function whose answer is displayed, the words printed beside it, found by following the name the screen stores the answer in. NOT FOUND means a screen calls it but the label could not be traced automatically and needs reading.</t>
+          <t>Read from the function's own signature: the values passed to it, whether it also reads the stored data, and what it returns. NOT DECLARED means the code does not say what comes back.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Dependent functions</t>
+          <t>COLUMN — Label on screen</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>A dependent function is one whose output is used by another function, in a chain that ends at a screen. These columns list the dependent functions behind this one: those one step below it, how many there are in total, and all of them however many steps away.</t>
+          <t>For a function whose answer is displayed, the words printed beside it, found by following the name the screen stores the answer in. NOT FOUND means a screen calls it but the label could not be traced automatically and needs reading.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — The chain, ending in this function</t>
+          <t>COLUMN — Dependent functions</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Read left to right. The function that shows the answer sits at the END, and everything feeding it comes before it. A loop is marked where a chain turns back on itself. Chains are cut at five levels and eight paths, and say so.</t>
+          <t>A dependent function is one whose output is used by another function, in a chain that ends at a screen. These columns list the dependent functions behind this one: those one step below it, how many there are in total, and all of them however many steps away.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Same figure as (S16)</t>
+          <t>COLUMN — The chain, ending in this function</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Where the same figure appears under more than one identifier, the row names the surviving identifier and why. Nothing is deleted: identifiers are never reused, so a folded row stays visible and says what it became.</t>
+          <t>Read left to right. The function that shows the answer sits at the END, and everything feeding it comes before it. A loop is marked where a chain turns back on itself. Chains are cut at five levels and eight paths, and say so.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Questions for you (numbered)</t>
+          <t>COLUMN — Same figure as (S16)</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
+          <t>Where the same figure appears under more than one identifier, the row names the surviving identifier and why. Nothing is deleted: identifiers are never reused, so a folded row stays visible and says what it became.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — YOUR ANSWER — use the same number</t>
+          <t>COLUMN — Questions for you (numbered)</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
+          <t>My open questions about that engine or figure, each with a number that never changes. A number is never reused or renumbered, so an answer can always be matched to its question.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Errors or findings to address</t>
+          <t>COLUMN — YOUR ANSWER — use the same number</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
+          <t>Answer here, starting each answer with the question number. Nothing else in the file needs to line up.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Decisions made (S03)</t>
+          <t>COLUMN — Errors or findings to address</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>The rulings and assumptions that govern this figure, each marked with WHOSE decision it was: [Founder] his own ruling, [The person] something the user set, [Built in] an assumption nobody chose on a screen — which is usually why a number looks wrong. The standing display and rounding rule applies to every row and is stated at the top of this tab.</t>
+          <t>What is known to be wrong or unproved about this figure, in plain English. Blank means nothing is on record yet — not that nothing is wrong.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (mathematical)</t>
+          <t>COLUMN — Decisions made (S03)</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
+          <t>The rulings and assumptions that govern this figure, each marked with WHOSE decision it was: [Founder] his own ruling, [The person] something the user set, [Built in] an assumption nobody chose on a screen — which is usually why a number looks wrong. The standing display and rounding rule applies to every row and is stated at the top of this tab.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Formula (in words)</t>
+          <t>COLUMN — Formula (mathematical)</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
+          <t>The rule written as arithmetic, so it can be followed symbol by symbol and checked against the code.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Engine ID</t>
+          <t>COLUMN — Formula (in words)</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
+          <t>The same rule in plain English, followable by hand. Where the engine has a row in the old master this is its wording, carried over; where it does not, it is written here from reading the code.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Your name for it (72-metric file)</t>
+          <t>COLUMN — Engine ID</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
+          <t>The identifier of that engine. Blank where the figure is worked out on the screen itself rather than by an engine — which is itself a finding.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Core screen?</t>
+          <t>COLUMN — Your name for it (72-metric file)</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
+          <t>The founder's own name for the same figure, from METRICS-DELIVERABLE-ANSWERED-2026-08-20.xlsx. This column is the bridge between his vocabulary and the code's.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Core screen?</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Whether the screen is part of the 55-70 core, the agreed first scope. Currently NOT DETERMINED on every row: the core list has never been written down, so no row can honestly claim to be in or out of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Row status</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>VERIFIED with its date means a person read the screen and confirmed the chain. NOT STARTED means the screen has not been read yet. Nothing in between is claimed.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-      <c r="B53" s="3" t="inlineStr"/>
-    </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>COLUMN — Input ID</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>The identifier of a raw input, per the same standard.</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="inlineStr"/>
+      <c r="B54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Variable name</t>
+          <t>COLUMN — Input ID</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>What the raw value is called.</t>
+          <t>The identifier of a raw input, per the same standard.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Source</t>
+          <t>COLUMN — Variable name</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
+          <t>What the raw value is called.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>COLUMN — Which metric uses it</t>
+          <t>COLUMN — Source</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Every metric identifier that depends on this input.</t>
+          <t>Where the value comes from: the person typed it, an institution download, a connected provider, or another engine computed it.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>COLUMN — Which metric uses it</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Every metric identifier that depends on this input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
           <t>COLUMN — Which engine uses it</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Every engine identifier that reads this input.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr"/>
-      <c r="B59" s="3" t="inlineStr"/>
-    </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Complies with — naming</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
-        </is>
-      </c>
+      <c r="A60" s="2" t="inlineStr"/>
+      <c r="B60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Complies with — identifiers</t>
+          <t>Complies with — naming</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_file-and-folder-naming_v01.md</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
+          <t>Complies with — identifiers</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>MoneyKeel/documents/standards/moneykeel_naming_spec_unique-identifier_v01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
           <t>Complies with — objectives</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>MoneyKeel/documents/standards/moneykeel_calc_spec_objectives-and-verification_v01.md</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr"/>
-      <c r="B63" s="3" t="inlineStr"/>
-    </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>COVERAGE — screens read so far</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
-        </is>
-      </c>
+      <c r="A64" s="2" t="inlineStr"/>
+      <c r="B64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
+          <t>COVERAGE — screens read so far</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>49 of 49. Every screen in the app has been read: the five parent screens, every secondary screen and every menu screen. Twelve screens carry no calculated figure and say so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
           <t>COVERAGE — what that means</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Every screen in the app is listed on its tab. Only Home carries figures so far; the rest are marked NOT STARTED. A rising count is not completeness while screens remain unread.</t>
         </is>
@@ -10937,7 +10949,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Why it was put there</t>
+          <t>What it is for</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -11039,7 +11051,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Can this account hold individual ticker securities?</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -11117,7 +11129,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>APPROVED v6 (2026-07-19): a CONNECTED account splits across the asset classes it actually holds — CDs under bonds, money market + sleeve under cash, options under alternatives, stocks under stocks — with the slices summing EXACTLY to the broker's authoritative balance.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -11197,7 +11209,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The ONE display name for an account row (build-43 finding #1): institution prefixes the label ONLY when the label doesn't already say it (E*TRADE's own name is "E*Trade Individual Brokerage" — prefixing the institution again rendered "E-Trade E*Trade Individual…"), and the broker's mask suffixes when present so two same-named accounts are tellable apart (wireframe: "Brokerage ...4821").</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -11277,7 +11289,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Display names for a whole LIST of accounts.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -11357,7 +11369,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -11435,7 +11447,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The last four digits of an account, or null when we genuinely don't have them.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -11513,7 +11525,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Which currency is the app showing?</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -11591,7 +11603,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The one lookup the UI uses.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -11669,7 +11681,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>── duplicate-proofing ───────────────────────────────────────────────────────────────────────── SnapTrade activity ids can change when they reprocess history, so identity = the composite of everything that makes the row THAT row.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -11747,7 +11759,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Σ ACTUAL payments (override ≥ minimum) — what actually leaves your account.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -11826,7 +11838,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Actual money flow for a month from LOGGED data — the exact figures behind the Home cash-flow card, so every screen (Home, Goals) shows the SAME surplus.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -11912,7 +11924,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>── Listen for notification taps ───────────────────────────────────</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -11990,7 +12002,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The account ids a transaction can touch.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -12068,7 +12080,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What's LEFT of this month's surplus to put to work = surplus − already-allocated this month (never &lt; 0).</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -12146,7 +12158,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How is my invested money spread?</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -12224,7 +12236,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -12303,7 +12315,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -12381,7 +12393,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>What is worth saying about this spending?</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -12459,7 +12471,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Annual employee 401(k) limit for the user's age (adds the 50+ catch-up).</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -12537,7 +12549,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>ONE annual cash-flow roll-up, derived entirely from the per-month income grid + spendByMonth — the SAME bases the savings-plan and budget already use.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -12623,7 +12635,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Annual coupon income = face value × coupon rate (paid as cash).</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -12701,7 +12713,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -12779,7 +12791,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -12857,7 +12869,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Annual NET contribution of a source: jobs use gross; rentals net out operating expenses.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -12935,7 +12947,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Annual amount of what the user ENTERED (not grossed up) — for display.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -13013,7 +13025,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Apply one transaction to the accounts (pure).</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -13092,7 +13104,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Approximate yield to maturity (standard approximation), decimal.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -13171,7 +13183,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How much money sits in each of the seven classes?</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -13253,7 +13265,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>WHAT the account is (asset class).</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -13331,7 +13343,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What do we know about this kind of account?</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -13409,7 +13421,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Build asset accounts from onboarding answers (accumulation: retirement savings + holdings).</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -13488,7 +13500,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Per-holding contribution to the portfolio's period return = weight × the holding's return (pts).</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -13566,7 +13578,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Prompt for Face ID / Touch ID / device passcode.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -13644,7 +13656,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Summarize per-month available-to-save from a 12-month cash-flow grid.</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -13722,7 +13734,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -13802,7 +13814,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -13880,7 +13892,7 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Benchmark return + its source/period for an asset kind.</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -13958,7 +13970,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Benchmark expected annual return for an asset kind — user override if set, else the ASSET_KINDS default.</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -14036,7 +14048,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What should this holding be compared against?</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -14114,7 +14126,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Calendar months (1-12) benefits are received — e.g.</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -14192,7 +14204,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Annual benefits = monthly amount × the months it's actually received.</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -14271,7 +14283,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Blended expected return across the EARMARKED nest egg, weighted by each holding's share.</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -14353,7 +14365,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The volatility of THIS portfolio — each account's own class volatility, weighted the way the money actually is (the same weighting `blendedReturn` uses, so the pair always describes one portfolio).</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -14434,7 +14446,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What are this holding's bond facts?</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -14512,7 +14524,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What happens to this bond if interest rates move?</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -14591,7 +14603,7 @@
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -14670,7 +14682,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -14756,7 +14768,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Month-to-date actual spending vs the planned budget, bucketed.</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -14838,7 +14850,7 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How much of everything sits in each account, and what return do they blend to?</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -14916,7 +14928,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>projected_to_save = net monthly income − monthly spending.</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -14994,7 +15006,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>My net worth changed since last time — what actually caused it?</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -15072,7 +15084,7 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Build the dated 12-month grid.</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
@@ -15158,7 +15170,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Today's SnapshotDay, observed from the live account state.</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -15236,7 +15248,7 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What is the whole debt picture?</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
@@ -15318,7 +15330,7 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Months to reach each goal at the given monthly savings capacity.</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -15397,7 +15409,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -15480,7 +15492,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Ranked insights (highest priority first).</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -15558,7 +15570,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Build the new accounts to CREATE when committing an itemization.</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -15638,7 +15650,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What is this household worth?</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -15716,7 +15728,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Build the month-by-month paycheck.</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -15802,7 +15814,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Build the per-holding rows for a period from positions + a price-series lookup.</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -15888,7 +15900,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -15967,7 +15979,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Build a snapshot from EXPLICIT net-worth rows.</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -16053,7 +16065,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>── DEK lifecycle (the cached, unwrapped key the sync layer uses) ───── Cache the unwrapped DEK (memory + keychain).</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -16131,7 +16143,7 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Is there any record at all on or before this date?</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -16209,7 +16221,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>── Cancel streak reminder (e.g.</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -16287,7 +16299,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>If I sold this today, how much of the gain is long-term and how much short-term?</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -16365,7 +16377,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -16443,7 +16455,7 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Report a caught error.</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -16521,7 +16533,7 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Signed cash effect on the primary account (for display).</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
@@ -16599,7 +16611,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Cash &amp; cash equivalents (Term #3) — THE cash number, and the same one the Net Worth CASH group shows.</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -16681,7 +16693,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Build the 12-month cash-flow picture.</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -16767,7 +16779,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Canonical per-category planned $/month — the ONE conversion the buckets AND the Budget screen share, so a category's on-screen line item ALWAYS reconciles with its bucket total (build-34 #3).</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -16845,7 +16857,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The claim window: the month the person turns 62 → the month they turn 70.</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -16923,7 +16935,7 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Plain words for an account's slice inside a class row.</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -17001,7 +17013,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Classify one institution word.</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -17079,7 +17091,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>B7 (founder brief 2026-08-20): classification lives in the ONE engine — this road only adapts.</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -17157,7 +17169,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -17235,7 +17247,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Forget the DEK (on logout / account deletion).</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -17313,7 +17325,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Cost-of-living factor for a free-text location.</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -17391,7 +17403,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Compare paying `extraMonthly` into the mortgage against putting the same money into Treasuries.</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -17469,7 +17481,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Mark an account's wrapper as USER-CONFIRMED — future syncs never override it.</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -17547,7 +17559,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How old a connected account's last successful sync is.</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -17625,7 +17637,7 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The class an account SHOULD carry under the current rule.</t>
         </is>
       </c>
       <c r="G86" s="3" t="inlineStr">
@@ -17704,7 +17716,7 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What did I pay for this in total?</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -17782,7 +17794,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Total annual coupon income across the user's INDIVIDUAL bonds (kept for the Bonds screen summary).</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -17862,7 +17874,7 @@
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What can we honestly say about a window starting on `from`?</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -17942,7 +17954,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Does the record actually cover this window?</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -18020,7 +18032,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Whether reports are actually shipping to Sentry (DSN + SDK present).</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
@@ -18098,7 +18110,7 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it, but it only changes how a value LOOKS — it does no arithmetic.</t>
+          <t>Create an invite code pointing at this household's shared data doc.</t>
         </is>
       </c>
       <c r="G92" s="3" t="inlineStr">
@@ -18176,7 +18188,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -18254,7 +18266,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
@@ -18332,7 +18344,7 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
@@ -18410,7 +18422,7 @@
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Age in whole years from birth month/year, as of `asOf` (defaults to now).</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
@@ -18488,7 +18500,7 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The email of the account currently signed in to Firebase — the authoritative identity that account-level actions (delete, reauth) operate on.</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
@@ -18566,7 +18578,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Retirement income (ri_*) counts as CURRENT income only when the user actually receives it now — i.e.</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
@@ -18644,7 +18656,7 @@
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
@@ -18722,7 +18734,7 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Current yield = annual coupon ÷ current price/value.</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
@@ -18800,7 +18812,7 @@
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Every incomplete promise across the given accounts.</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr">
@@ -18878,7 +18890,7 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>"14 March 2022".</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
@@ -18956,7 +18968,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What do we know about this kind of debt?</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
@@ -19034,7 +19046,7 @@
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G104" s="3" t="inlineStr">
@@ -19112,7 +19124,7 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What debts should exist from the setup answers?</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
@@ -19192,7 +19204,7 @@
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What is the text of the file that was picked?</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
@@ -19270,7 +19282,7 @@
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Decrypt a synced value: ciphertext → object; legacy plaintext object → returned as-is; null if it's ciphertext we can't decrypt (no key).</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
@@ -19350,7 +19362,7 @@
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Decrypt an 'enc:'-tagged blob.</t>
         </is>
       </c>
       <c r="G108" s="3" t="inlineStr">
@@ -19428,7 +19440,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The standard deduction with the age-65 additions (E8).</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
@@ -19506,7 +19518,7 @@
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Which of these activities are new since the last sync?</t>
         </is>
       </c>
       <c r="G110" s="3" t="inlineStr">
@@ -19584,7 +19596,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>B47 finding 11 — a debt's repayment SHAPE.</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -19662,7 +19674,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Permanently delete the signed-in user's account (App Store Guideline 5.1.1(v)).</t>
         </is>
       </c>
       <c r="G112" s="3" t="inlineStr">
@@ -19744,7 +19756,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>---- deterministic depletion ---- Age the portfolio runs out (deterministic), or null if it lasts to the horizon.</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
@@ -19824,7 +19836,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The direction an event implies, where the event itself decides it.</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr">
@@ -19902,7 +19914,7 @@
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>B6 (founder brief 2026-08-20): the odds a person sees, to the nearest 5 — with one honesty guard at each end: 100 means "every simulated future worked" and 0 means "none did", and neither claim may be minted by rounding.</t>
         </is>
       </c>
       <c r="G115" s="3" t="inlineStr">
@@ -19980,7 +19992,7 @@
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr">
@@ -20061,7 +20073,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Earliest dated lot — the day this holding became YOUR money.</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
@@ -20139,7 +20151,7 @@
       </c>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Default % of an account that's earmarked for retirement (rest funds other goals).</t>
         </is>
       </c>
       <c r="G118" s="3" t="inlineStr">
@@ -20218,7 +20230,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The retirement-earmarked $ for one account (uses the saved % or the smart default).</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr">
@@ -20298,7 +20310,7 @@
       </c>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Distinct investment kinds present in the earmarked nest egg (for the benchmark editor).</t>
         </is>
       </c>
       <c r="G120" s="3" t="inlineStr">
@@ -20378,7 +20390,7 @@
       </c>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G121" s="3" t="inlineStr">
@@ -20456,7 +20468,7 @@
       </c>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NEGATIVE CASH FLOW DRAINS WEALTH — committed contributions don't create money.</t>
         </is>
       </c>
       <c r="G122" s="3" t="inlineStr">
@@ -20542,7 +20554,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G123" s="3" t="inlineStr">
@@ -20628,7 +20640,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Blended effective rate (total tax / gross).</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
@@ -20706,7 +20718,7 @@
       </c>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What share of my income actually goes in tax?</t>
         </is>
       </c>
       <c r="G125" s="3" t="inlineStr">
@@ -20784,7 +20796,7 @@
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G126" s="3" t="inlineStr">
@@ -20862,7 +20874,7 @@
       </c>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>"What if a $X emergency hit right now?" — can your cash absorb it, and how long would you last.</t>
         </is>
       </c>
       <c r="G127" s="3" t="inlineStr">
@@ -20948,7 +20960,7 @@
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr">
@@ -21026,7 +21038,7 @@
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
@@ -21104,7 +21116,7 @@
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Employer match resolved to $/month.</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr">
@@ -21182,7 +21194,7 @@
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>── The sync layer's interface (operates on the cached DEK) ─────────── Encrypt a payload with the cached DEK.</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr">
@@ -21261,7 +21273,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
@@ -21339,7 +21351,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr">
@@ -21417,7 +21429,7 @@
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Level annual equity spread across the months it vests (0 for most students).</t>
         </is>
       </c>
       <c r="G134" s="3" t="inlineStr">
@@ -21498,7 +21510,7 @@
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Per-calendar-year vesting cash flow across all schedule rows — drives the chart &amp; table.</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr">
@@ -21577,7 +21589,7 @@
       </c>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Value of one vesting-schedule row.</t>
         </is>
       </c>
       <c r="G136" s="3" t="inlineStr">
@@ -21655,7 +21667,7 @@
       </c>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Vest-month weights (Jan→Dec, summing to 1) from the equity grant rows — THE one placement rule.</t>
         </is>
       </c>
       <c r="G137" s="3" t="inlineStr">
@@ -21733,7 +21745,7 @@
       </c>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G138" s="3" t="inlineStr">
@@ -21811,7 +21823,7 @@
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Extra income sources beyond salary/rental/equity (self-employment, investment, benefits, support, scholarship, other), split into taxable vs non-taxable steady monthly amounts + a one-time Jan amount.</t>
         </is>
       </c>
       <c r="G139" s="3" t="inlineStr">
@@ -21892,7 +21904,7 @@
       </c>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Price factor over the trailing window: last close ÷ the close at (now − months).</t>
         </is>
       </c>
       <c r="G140" s="3" t="inlineStr">
@@ -21970,7 +21982,7 @@
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>What are inflation and the 10-year Treasury yield?</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr">
@@ -22048,7 +22060,7 @@
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Fetch many tickers in parallel; returns only the ones that resolved.</t>
         </is>
       </c>
       <c r="G142" s="3" t="inlineStr">
@@ -22126,7 +22138,7 @@
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Effective tax rate in use: the user's manual rate, else the IRS-schedule estimate on taxable income.</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr">
@@ -22204,7 +22216,7 @@
       </c>
       <c r="F144" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The first date the record covers — so a change figure can say what it is measured FROM, rather than presenting a figure measured from install day as though it covered the year.</t>
         </is>
       </c>
       <c r="G144" s="3" t="inlineStr">
@@ -22282,7 +22294,7 @@
       </c>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G145" s="3" t="inlineStr">
@@ -22360,7 +22372,7 @@
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The plain-English comparison sentence for the detail view — fixed, human-reviewed templates.</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr">
@@ -22438,7 +22450,7 @@
       </c>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Full amount, no minor units (matches the app's whole-number money style), locale-grouped.</t>
         </is>
       </c>
       <c r="G147" s="3" t="inlineStr">
@@ -22516,7 +22528,7 @@
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Same as formatMoney but keeps 2 decimal places — for precise amounts (transactions, holdings, recurring lines).</t>
         </is>
       </c>
       <c r="G148" s="3" t="inlineStr">
@@ -22594,7 +22606,7 @@
       </c>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The FRA as words a person recognises — "67", or "66 and 4 months".</t>
         </is>
       </c>
       <c r="G149" s="3" t="inlineStr">
@@ -22672,7 +22684,7 @@
       </c>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Full retirement age in YEARS (fractional — 66y4m = 66.333…), from the birth year.</t>
         </is>
       </c>
       <c r="G150" s="3" t="inlineStr">
@@ -22750,7 +22762,7 @@
       </c>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it, but it only changes how a value LOOKS — it does no arithmetic.</t>
+          <t>The banner sentence — plural-correct, and absent (null) when nothing is missing.</t>
         </is>
       </c>
       <c r="G151" s="3" t="inlineStr">
@@ -22828,7 +22840,7 @@
       </c>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>── Key generation ─────────────────────────────────────────────────── A fresh random 256-bit data key (hex).</t>
         </is>
       </c>
       <c r="G152" s="3" t="inlineStr">
@@ -22906,7 +22918,7 @@
       </c>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>A human-friendly recovery code, e.g.</t>
         </is>
       </c>
       <c r="G153" s="3" t="inlineStr">
@@ -22984,7 +22996,7 @@
       </c>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G154" s="3" t="inlineStr">
@@ -23063,7 +23075,7 @@
       </c>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The cached DEK (memory → keychain), or null if it hasn't been unwrapped on this install yet.</t>
         </is>
       </c>
       <c r="G155" s="3" t="inlineStr">
@@ -23141,7 +23153,7 @@
       </c>
       <c r="F156" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G156" s="3" t="inlineStr">
@@ -23224,7 +23236,7 @@
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The public read-model (spec IncomeState): totals, effective rate, monthly grid.</t>
         </is>
       </c>
       <c r="G157" s="3" t="inlineStr">
@@ -23308,7 +23320,7 @@
       </c>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Profile + derived planning values (current age, years to retirement, horizon).</t>
         </is>
       </c>
       <c r="G158" s="3" t="inlineStr">
@@ -23389,7 +23401,7 @@
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>Read a single-document-per-user collection (e.g.</t>
         </is>
       </c>
       <c r="G159" s="3" t="inlineStr">
@@ -23467,7 +23479,7 @@
       </c>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Months remaining: from the target date if set, else the goal's `duration` (months).</t>
         </is>
       </c>
       <c r="G160" s="3" t="inlineStr">
@@ -23545,7 +23557,7 @@
       </c>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Funded %, clamped 0–100.</t>
         </is>
       </c>
       <c r="G161" s="3" t="inlineStr">
@@ -23623,7 +23635,7 @@
       </c>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G162" s="3" t="inlineStr">
@@ -23702,7 +23714,7 @@
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G163" s="3" t="inlineStr">
@@ -23781,7 +23793,7 @@
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Gross annual baseline = jobs (gross) + rentals (gross − expenses), all annualized.</t>
         </is>
       </c>
       <c r="G164" s="3" t="inlineStr">
@@ -23859,7 +23871,7 @@
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Invert the schedule: the gross income whose take-home equals `net` (bisection).</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr">
@@ -23937,7 +23949,7 @@
       </c>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>A representative full-month GROSS salary (the highest month — undiluted by $0 gap months).</t>
         </is>
       </c>
       <c r="G166" s="3" t="inlineStr">
@@ -24017,7 +24029,7 @@
       </c>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>── Deterministic projection (instant — drives the live sliders; no RNG) ────────────── Assumes the average return every year (no market swings).</t>
         </is>
       </c>
       <c r="G167" s="3" t="inlineStr">
@@ -24095,7 +24107,7 @@
       </c>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The plan's guaranteed-income input as separate streams of OUTSIDE money only. Answers: zer</t>
         </is>
       </c>
       <c r="G168" s="3" t="inlineStr">
@@ -24173,7 +24185,7 @@
       </c>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The dated guaranteed-income rows for the next 12 months (the F2 grid seam).</t>
         </is>
       </c>
       <c r="G169" s="3" t="inlineStr">
@@ -24251,7 +24263,7 @@
       </c>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G170" s="3" t="inlineStr">
@@ -24329,7 +24341,7 @@
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>True iff every measured account's story begins IN the ledger (openable honestly).</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
@@ -24407,7 +24419,7 @@
       </c>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G172" s="3" t="inlineStr">
@@ -24485,7 +24497,7 @@
       </c>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Where the money to close the gap actually comes from — the breakdown that stops a person subtracting and concluding the app cannot add up (founder, 2026-08-14).</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
@@ -24564,7 +24576,7 @@
       </c>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What holdings are in this file?</t>
         </is>
       </c>
       <c r="G174" s="3" t="inlineStr">
@@ -24643,7 +24655,7 @@
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G175" s="3" t="inlineStr">
@@ -24721,7 +24733,7 @@
       </c>
       <c r="F176" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>FOUNDER RULE 2026-08-04 (supersedes the money-market=cash rule and the 12-month CD split): CASH means cash only — a sweep/settlement balance.</t>
         </is>
       </c>
       <c r="G176" s="3" t="inlineStr">
@@ -24799,7 +24811,7 @@
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G177" s="3" t="inlineStr">
@@ -24885,7 +24897,7 @@
       </c>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>A representative 12-month cash-flow grid (Jan→Dec) that honors lumpiness: salary &amp; net rental are steady every month; the annual bonus lands in December; the signing bonus is one-time (January); equity is the level annual vesting spread across the month-of-year its vest dates fall on (so quarterly vesting shows up as quarterly spikes).</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
@@ -24971,7 +24983,7 @@
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>B-30: infer the debt type from its name so a "Mortgage" is treated as a mortgage (homeowner DTI guideline), not lumped into OTHER (renter guideline).</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
@@ -25049,7 +25061,7 @@
       </c>
       <c r="F180" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>A broker just sent us data — what changes?</t>
         </is>
       </c>
       <c r="G180" s="3" t="inlineStr">
@@ -25135,7 +25147,7 @@
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Initialise crash reporting once, at app start.</t>
         </is>
       </c>
       <c r="G181" s="3" t="inlineStr">
@@ -25213,7 +25225,7 @@
       </c>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Canonical annual INTEREST income across all interest-bearing holdings (Term #6).</t>
         </is>
       </c>
       <c r="G182" s="3" t="inlineStr">
@@ -25294,7 +25306,7 @@
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Legacy fallback for rows recorded before undo_prev: a synthetic opposite transaction.</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
@@ -25372,7 +25384,7 @@
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Investable assets (Term #4) = all financial assets (cash + investments + retirement balances), EXCLUDING real estate + personal property.</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr">
@@ -25452,7 +25464,7 @@
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>FOUNDER RULE 2026-08-04: the NW change PERCENT is measured on cash + investments only — property values move only when someone retypes them, so a total-net-worth percent is noise.</t>
         </is>
       </c>
       <c r="G185" s="3" t="inlineStr">
@@ -25530,7 +25542,7 @@
       </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Investment income (cash dividends/interest/coupons, not reinvested) over the trailing window — feeds the Income module.</t>
         </is>
       </c>
       <c r="G186" s="3" t="inlineStr">
@@ -25608,7 +25620,7 @@
       </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Investments / holdings (allocation view, Term #4) = equities + fixed income + alternatives, ACROSS all wrappers (so a 401(k)'s stocks count).</t>
         </is>
       </c>
       <c r="G187" s="3" t="inlineStr">
@@ -25686,7 +25698,7 @@
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Is this account an "other investment" — an alternative held at a manual value (not a bond, not cash/property)?</t>
         </is>
       </c>
       <c r="G188" s="3" t="inlineStr">
@@ -25764,7 +25776,7 @@
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>An AssetAccount is a bond if its ASSET CLASS is bonds (spec §2: "detected by assetClass, NOT maturity date").</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr">
@@ -25842,7 +25854,7 @@
       </c>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Does this account type sit under the Cash heading on screen?</t>
         </is>
       </c>
       <c r="G190" s="3" t="inlineStr">
@@ -25920,7 +25932,7 @@
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G191" s="3" t="inlineStr">
@@ -25998,7 +26010,7 @@
       </c>
       <c r="F192" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>── Low-level AES helpers (also used to wrap the DEK) ─────────────────</t>
         </is>
       </c>
       <c r="G192" s="3" t="inlineStr">
@@ -26076,7 +26088,7 @@
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>True only when the device has biometric hardware AND the user has enrolled a biometric/passcode.</t>
         </is>
       </c>
       <c r="G193" s="3" t="inlineStr">
@@ -26154,7 +26166,7 @@
       </c>
       <c r="F194" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Money leaves the account: withdrawals, fees, and transfers with no recognized counter-account.</t>
         </is>
       </c>
       <c r="G194" s="3" t="inlineStr">
@@ -26232,7 +26244,7 @@
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Did the personal return produce a number, or a reason it could not?</t>
         </is>
       </c>
       <c r="G195" s="3" t="inlineStr">
@@ -26310,7 +26322,7 @@
       </c>
       <c r="F196" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Is a ticker plausibly valid before we spend a network call?</t>
         </is>
       </c>
       <c r="G196" s="3" t="inlineStr">
@@ -26388,7 +26400,7 @@
       </c>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>True when the asset is a real/physical asset (real estate or personal property) — excluded from investable assets and the nest egg (Term #4/#7).</t>
         </is>
       </c>
       <c r="G197" s="3" t="inlineStr">
@@ -26467,7 +26479,7 @@
       </c>
       <c r="F198" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Lump balance − Σ holdings.</t>
         </is>
       </c>
       <c r="G198" s="3" t="inlineStr">
@@ -26546,7 +26558,7 @@
       </c>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The account total AFTER itemizing.</t>
         </is>
       </c>
       <c r="G199" s="3" t="inlineStr">
@@ -26627,7 +26639,7 @@
       </c>
       <c r="F200" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Σ of the itemized holding values.</t>
         </is>
       </c>
       <c r="G200" s="3" t="inlineStr">
@@ -26705,7 +26717,7 @@
       </c>
       <c r="F201" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Is base salary present in calendar month i (0-11)?</t>
         </is>
       </c>
       <c r="G201" s="3" t="inlineStr">
@@ -26785,7 +26797,7 @@
       </c>
       <c r="F202" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Claim membership in {householdId} by writing the member doc the security rules gate access on.</t>
         </is>
       </c>
       <c r="G202" s="3" t="inlineStr">
@@ -26863,7 +26875,7 @@
       </c>
       <c r="F203" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How much more you can still put into your 401(k) this year (incl.</t>
         </is>
       </c>
       <c r="G203" s="3" t="inlineStr">
@@ -26941,7 +26953,7 @@
       </c>
       <c r="F204" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What is the most recent price we hold for this?</t>
         </is>
       </c>
       <c r="G204" s="3" t="inlineStr">
@@ -27019,7 +27031,7 @@
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr">
@@ -27099,7 +27111,7 @@
       </c>
       <c r="F206" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G206" s="3" t="inlineStr">
@@ -27177,7 +27189,7 @@
       </c>
       <c r="F207" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G207" s="3" t="inlineStr">
@@ -27255,7 +27267,7 @@
       </c>
       <c r="F208" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G208" s="3" t="inlineStr">
@@ -27333,7 +27345,7 @@
       </c>
       <c r="F209" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G209" s="3" t="inlineStr">
@@ -27411,7 +27423,7 @@
       </c>
       <c r="F210" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G210" s="3" t="inlineStr">
@@ -27489,7 +27501,7 @@
       </c>
       <c r="F211" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G211" s="3" t="inlineStr">
@@ -27567,7 +27579,7 @@
       </c>
       <c r="F212" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G212" s="3" t="inlineStr">
@@ -27645,7 +27657,7 @@
       </c>
       <c r="F213" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G213" s="3" t="inlineStr">
@@ -27725,7 +27737,7 @@
       </c>
       <c r="F214" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>The member's own top-level doc fields (householdId + decrypted appState) in one read.</t>
         </is>
       </c>
       <c r="G214" s="3" t="inlineStr">
@@ -27805,7 +27817,7 @@
       </c>
       <c r="F215" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>UNIT LANDMINE (P0): `aprPct` is a PERCENT (7 = 7%), unlike Debt.interest_rate_apr which is a DECIMAL (0.07).</t>
         </is>
       </c>
       <c r="G215" s="3" t="inlineStr">
@@ -27883,7 +27895,7 @@
       </c>
       <c r="F216" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>Returns the user plus the unlock status: • needsRecovery=true → the password can't open the data (it was reset); prompt for the recovery code.</t>
         </is>
       </c>
       <c r="G216" s="3" t="inlineStr">
@@ -27965,7 +27977,7 @@
       </c>
       <c r="F217" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G217" s="3" t="inlineStr">
@@ -28043,7 +28055,7 @@
       </c>
       <c r="F218" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What if I had moved this money?</t>
         </is>
       </c>
       <c r="G218" s="3" t="inlineStr">
@@ -28122,7 +28134,7 @@
       </c>
       <c r="F219" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Fixed income by its words.</t>
         </is>
       </c>
       <c r="G219" s="3" t="inlineStr">
@@ -28200,7 +28212,7 @@
       </c>
       <c r="F220" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G220" s="3" t="inlineStr">
@@ -28278,7 +28290,7 @@
       </c>
       <c r="F221" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The user's own long-term capital-gains rate, from their income + filing status (federal).</t>
         </is>
       </c>
       <c r="G221" s="3" t="inlineStr">
@@ -28356,7 +28368,7 @@
       </c>
       <c r="F222" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Build the stored envelope: the DEK locked by both the password and the recovery code.</t>
         </is>
       </c>
       <c r="G222" s="3" t="inlineStr">
@@ -28434,7 +28446,7 @@
       </c>
       <c r="F223" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The ONE writer — stamps the version and keeps the arithmetic identity by construction.</t>
         </is>
       </c>
       <c r="G223" s="3" t="inlineStr">
@@ -28512,7 +28524,7 @@
       </c>
       <c r="F224" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Build a full transaction (id + created_at) from a partial.</t>
         </is>
       </c>
       <c r="G224" s="3" t="inlineStr">
@@ -28590,7 +28602,7 @@
       </c>
       <c r="F225" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>What kind of account is this, and how is it taxed?</t>
         </is>
       </c>
       <c r="G225" s="3" t="inlineStr">
@@ -28668,7 +28680,7 @@
       </c>
       <c r="F226" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>A line arrived from the broker. Is this money you paid IN, money you took OUT, or something that happened inside the account?</t>
         </is>
       </c>
       <c r="G226" s="3" t="inlineStr">
@@ -28746,7 +28758,7 @@
       </c>
       <c r="F227" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>What is this option position worth, and what do we call it?</t>
         </is>
       </c>
       <c r="G227" s="3" t="inlineStr">
@@ -28824,7 +28836,7 @@
       </c>
       <c r="F228" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>B7 (founder brief 2026-08-20): classification lives in the ONE engine — name first, broker tag as fallback only.</t>
         </is>
       </c>
       <c r="G228" s="3" t="inlineStr">
@@ -28902,7 +28914,7 @@
       </c>
       <c r="F229" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The marginal bracket rate (decimal) for an income (on taxable income, after deduction).</t>
         </is>
       </c>
       <c r="G229" s="3" t="inlineStr">
@@ -28980,7 +28992,7 @@
       </c>
       <c r="F230" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G230" s="3" t="inlineStr">
@@ -29058,7 +29070,7 @@
       </c>
       <c r="F231" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What is this holding worth right now?</t>
         </is>
       </c>
       <c r="G231" s="3" t="inlineStr">
@@ -29137,7 +29149,7 @@
       </c>
       <c r="F232" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The existing account a fresh import from `institution` should offer to update (or null).</t>
         </is>
       </c>
       <c r="G232" s="3" t="inlineStr">
@@ -29215,7 +29227,7 @@
       </c>
       <c r="F233" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>FOUNDER RULE 2026-08-04 (supersedes build-34 #8's 12-month split): ANY maturity-dated instrument is a BOND — it pays interest, so it must sit in the measured bucket regardless of how soon it matures.</t>
         </is>
       </c>
       <c r="G233" s="3" t="inlineStr">
@@ -29293,7 +29305,7 @@
       </c>
       <c r="F234" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The short label that rides beside a change figure, always — whether the window is covered or not.</t>
         </is>
       </c>
       <c r="G234" s="3" t="inlineStr">
@@ -29372,7 +29384,7 @@
       </c>
       <c r="F235" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>FOUNDER RULE 2026-08-04: record how far back the broker's OWN activity feed reaches, so a "past year" income figure can label itself honestly.</t>
         </is>
       </c>
       <c r="G235" s="3" t="inlineStr">
@@ -29450,7 +29462,7 @@
       </c>
       <c r="F236" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The one decision rule.</t>
         </is>
       </c>
       <c r="G236" s="3" t="inlineStr">
@@ -29528,7 +29540,7 @@
       </c>
       <c r="F237" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The highest ladder rung at or below `netWorth` (0 when below the first rung).</t>
         </is>
       </c>
       <c r="G237" s="3" t="inlineStr">
@@ -29606,7 +29618,7 @@
       </c>
       <c r="F238" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>'$500k' / '$1M' — the label the celebration line uses.</t>
         </is>
       </c>
       <c r="G238" s="3" t="inlineStr">
@@ -29684,7 +29696,7 @@
       </c>
       <c r="F239" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Term #9 — TWO clearly-named monthly-debt numbers (they're different concepts, not a bug to pick one): Σ MINIMUM required payments — the contractual obligation.</t>
         </is>
       </c>
       <c r="G239" s="3" t="inlineStr">
@@ -29763,7 +29775,7 @@
       </c>
       <c r="F240" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Currency/locale-aware (delegates to the active money format; defaults to USD/en-US).</t>
         </is>
       </c>
       <c r="G240" s="3" t="inlineStr">
@@ -29841,7 +29853,7 @@
       </c>
       <c r="F241" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Same, but keeps cents — for precise amounts (transactions, holdings).</t>
         </is>
       </c>
       <c r="G241" s="3" t="inlineStr">
@@ -29919,7 +29931,7 @@
       </c>
       <c r="F242" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Compact form for tight spaces (chart labels, donut center).</t>
         </is>
       </c>
       <c r="G242" s="3" t="inlineStr">
@@ -29997,7 +30009,7 @@
       </c>
       <c r="F243" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>XIRR via bisection — deterministic, no derivative games.</t>
         </is>
       </c>
       <c r="G243" s="3" t="inlineStr">
@@ -30076,7 +30088,7 @@
       </c>
       <c r="F244" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>"March 2022" — a month a person reads, not a date stamp.</t>
         </is>
       </c>
       <c r="G244" s="3" t="inlineStr">
@@ -30154,7 +30166,7 @@
       </c>
       <c r="F245" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Total monthly contributions across types + employer match (feeds the retirement projection).</t>
         </is>
       </c>
       <c r="G245" s="3" t="inlineStr">
@@ -30233,7 +30245,7 @@
       </c>
       <c r="F246" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Monthly money you MUST keep paying — the recurring (non-monthly excluded) Critical + Important bills.</t>
         </is>
       </c>
       <c r="G246" s="3" t="inlineStr">
@@ -30319,7 +30331,7 @@
       </c>
       <c r="F247" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Monthly savings (the FLOW) — Build-47 walk row 7: DERIVED as the 12-month average of surplusByMonth, so the flat figure and the by-month figures can never drift apart (they used to be two parallel formulas that merely CLAIMED to reconcile).</t>
         </is>
       </c>
       <c r="G247" s="3" t="inlineStr">
@@ -30405,7 +30417,7 @@
       </c>
       <c r="F248" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>PRD F2#11 — the ONE per-calendar-month effective tax-rate vector (Jan→Dec).</t>
         </is>
       </c>
       <c r="G248" s="3" t="inlineStr">
@@ -30491,7 +30503,7 @@
       </c>
       <c r="F249" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>── B47 finding 11: the installment two-way math — enter the payment OR the end date, the app computes the other.</t>
         </is>
       </c>
       <c r="G249" s="3" t="inlineStr">
@@ -30569,7 +30581,7 @@
       </c>
       <c r="F250" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Months to reach the goal at a given monthly contribution (0 if funded; null if contribution &lt;= 0).</t>
         </is>
       </c>
       <c r="G250" s="3" t="inlineStr">
@@ -30647,7 +30659,7 @@
       </c>
       <c r="F251" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Whole months from `now` to the target month ('YYYY-MM'); &gt;=1, or null if no/!invalid date.</t>
         </is>
       </c>
       <c r="G251" s="3" t="inlineStr">
@@ -30725,7 +30737,7 @@
       </c>
       <c r="F252" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Run the plan twice and report both results.</t>
         </is>
       </c>
       <c r="G252" s="3" t="inlineStr">
@@ -30805,7 +30817,7 @@
       </c>
       <c r="F253" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What the NAME (symbol + description together) says, or null when it says nothing.</t>
         </is>
       </c>
       <c r="G253" s="3" t="inlineStr">
@@ -30883,7 +30895,7 @@
       </c>
       <c r="F254" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>── the cash sleeve, deduped ─────────────────────────────────────────────────────────────────── SnapTrade counts money-market (cash_equivalent) positions INSIDE balances.cash too.</t>
         </is>
       </c>
       <c r="G254" s="3" t="inlineStr">
@@ -30961,7 +30973,7 @@
       </c>
       <c r="F255" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What do we call this new thing?</t>
         </is>
       </c>
       <c r="G255" s="3" t="inlineStr">
@@ -31039,7 +31051,7 @@
       </c>
       <c r="F256" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G256" s="3" t="inlineStr">
@@ -31120,7 +31132,7 @@
       </c>
       <c r="F257" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Label basis for the non-monthly bucket (e.g.</t>
         </is>
       </c>
       <c r="G257" s="3" t="inlineStr">
@@ -31198,7 +31210,7 @@
       </c>
       <c r="F258" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Normalize ONE stored entry: v1 passes validated; a legacy blob (no `v`) maps best-effort; anything without a real month + net worth is dropped (null), never charted.</t>
         </is>
       </c>
       <c r="G258" s="3" t="inlineStr">
@@ -31276,7 +31288,7 @@
       </c>
       <c r="F259" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G259" s="3" t="inlineStr">
@@ -31354,7 +31366,7 @@
       </c>
       <c r="F260" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it, but it only changes how a value LOOKS — it does no arithmetic.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G260" s="3" t="inlineStr">
@@ -31433,7 +31445,7 @@
       </c>
       <c r="F261" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How do we state the odds in words?</t>
         </is>
       </c>
       <c r="G261" s="3" t="inlineStr">
@@ -31511,7 +31523,7 @@
       </c>
       <c r="F262" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G262" s="3" t="inlineStr">
@@ -31589,7 +31601,7 @@
       </c>
       <c r="F263" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G263" s="3" t="inlineStr">
@@ -31667,7 +31679,7 @@
       </c>
       <c r="F264" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>In one sentence, how is this plan doing?</t>
         </is>
       </c>
       <c r="G264" s="3" t="inlineStr">
@@ -31745,7 +31757,7 @@
       </c>
       <c r="F265" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The latest day at or before a date, or nothing when the record does not reach back that far.</t>
         </is>
       </c>
       <c r="G265" s="3" t="inlineStr">
@@ -31823,7 +31835,7 @@
       </c>
       <c r="F266" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Calendar month (1-12) a one-time "other income" lands in (default January).</t>
         </is>
       </c>
       <c r="G266" s="3" t="inlineStr">
@@ -31901,7 +31913,7 @@
       </c>
       <c r="F267" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>E8 (founder brief 2026-08-20): how many people on the return are 65+.</t>
         </is>
       </c>
       <c r="G267" s="3" t="inlineStr">
@@ -31979,7 +31991,7 @@
       </c>
       <c r="F268" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Minimal RFC-4180-ish CSV parser: handles quoted fields, embedded commas, "" escapes, CR/LF, BOM.</t>
         </is>
       </c>
       <c r="G268" s="3" t="inlineStr">
@@ -32057,7 +32069,7 @@
       </c>
       <c r="F269" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>── Receipt OCR simulation ─────────────────────────────────────────── In production, integrate Google Vision API or AWS Textract.</t>
         </is>
       </c>
       <c r="G269" s="3" t="inlineStr">
@@ -32135,7 +32147,7 @@
       </c>
       <c r="F270" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G270" s="3" t="inlineStr">
@@ -32213,7 +32225,7 @@
       </c>
       <c r="F271" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>Sends a receipt image to Google Cloud Vision API for OCR, then parses the raw text to extract store, total, date, category.</t>
         </is>
       </c>
       <c r="G271" s="3" t="inlineStr">
@@ -32291,7 +32303,7 @@
       </c>
       <c r="F272" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How is THIS debt repaid?</t>
         </is>
       </c>
       <c r="G272" s="3" t="inlineStr">
@@ -32369,7 +32381,7 @@
       </c>
       <c r="F273" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Monthly payment that clears `principal` in `months` at decimal APR (amortization).</t>
         </is>
       </c>
       <c r="G273" s="3" t="inlineStr">
@@ -32447,7 +32459,7 @@
       </c>
       <c r="F274" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Simulate paying off debts with a constant monthly budget (sum of minimums + extra), rolling each cleared debt's freed-up payment into the next per the chosen method.</t>
         </is>
       </c>
       <c r="G274" s="3" t="inlineStr">
@@ -32526,7 +32538,7 @@
       </c>
       <c r="F275" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>── the later cloud sync ──────────────────────────────────────────────────────────────────────── Everything not yet uploaded, oldest first.</t>
         </is>
       </c>
       <c r="G275" s="3" t="inlineStr">
@@ -32604,7 +32616,7 @@
       </c>
       <c r="F276" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The DOLLAR change implied by a period return on today's total — the approved Home hero shows "up $11,200 (1.4%) this month": dollars AND percent from the SAME measured return, so the two figures can never disagree (one concept, one source).</t>
         </is>
       </c>
       <c r="G276" s="3" t="inlineStr">
@@ -32682,7 +32694,7 @@
       </c>
       <c r="F277" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Price return of a ticker over a period (decimal).</t>
         </is>
       </c>
       <c r="G277" s="3" t="inlineStr">
@@ -32761,7 +32773,7 @@
       </c>
       <c r="F278" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Price return from an explicit start DATE to now (for purchase-capped windows).</t>
         </is>
       </c>
       <c r="G278" s="3" t="inlineStr">
@@ -32839,7 +32851,7 @@
       </c>
       <c r="F279" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G279" s="3" t="inlineStr">
@@ -32917,7 +32929,7 @@
       </c>
       <c r="F280" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Capture (camera) or pick (library) a receipt image; returns its uri or null if cancelled/denied.</t>
         </is>
       </c>
       <c r="G280" s="3" t="inlineStr">
@@ -32995,7 +33007,7 @@
       </c>
       <c r="F281" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
@@ -33073,7 +33085,7 @@
       </c>
       <c r="F282" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Is there enough to show this person their own odds?</t>
         </is>
       </c>
       <c r="G282" s="3" t="inlineStr">
@@ -33156,7 +33168,7 @@
       </c>
       <c r="F283" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>One call, everything the second gauge and the bridge sentence need.</t>
         </is>
       </c>
       <c r="G283" s="3" t="inlineStr">
@@ -33239,7 +33251,7 @@
       </c>
       <c r="F284" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The single canonical "planned monthly spend": the itemized buckets OR the stated total, whichever is larger (the stated total can include an uncategorized remainder the buckets don't capture).</t>
         </is>
       </c>
       <c r="G284" s="3" t="inlineStr">
@@ -33325,7 +33337,7 @@
       </c>
       <c r="F285" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Value-weighted ACTUAL trailing-12mo return across holdings that have one reported.</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
@@ -33405,7 +33417,7 @@
       </c>
       <c r="F286" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Value-weighted benchmark ("the market, matched to your mix") return across holdings that have one (decimal), or null.</t>
         </is>
       </c>
       <c r="G286" s="3" t="inlineStr">
@@ -33483,7 +33495,7 @@
       </c>
       <c r="F287" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Value-weighted portfolio period return across holdings that have one (decimal), or null.</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
@@ -33561,7 +33573,7 @@
       </c>
       <c r="F288" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How has my portfolio moved over the period, against its benchmark?</t>
         </is>
       </c>
       <c r="G288" s="3" t="inlineStr">
@@ -33640,7 +33652,7 @@
       </c>
       <c r="F289" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Human freshness of the price cache + whether it's stale enough to warn (markets move daily, so anything older than ~4 days — a long weekend/holiday — is worth a "may be out of date" note).</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
@@ -33718,7 +33730,7 @@
       </c>
       <c r="F290" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The vehicle treated as "the car you drive" — the most valuable one, so a second car stays a real asset.</t>
         </is>
       </c>
       <c r="G290" s="3" t="inlineStr">
@@ -33796,7 +33808,7 @@
       </c>
       <c r="F291" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>`op` is the consolidated onboardingProfile: { status, name, ...answers }.</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
@@ -33874,7 +33886,7 @@
       </c>
       <c r="F292" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>PRD F2#11 — progressive PER-MONTH tax: brackets fill as the year's taxable income accumulates month by month (Jan→Dec), so tax_m = taxOwed(cumulative through m) − taxOwed(cumulative through m−1).</t>
         </is>
       </c>
       <c r="G292" s="3" t="inlineStr">
@@ -33953,7 +33965,7 @@
       </c>
       <c r="F293" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What will the pot be worth at retirement, and how big does it need to be?</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
@@ -34033,7 +34045,7 @@
       </c>
       <c r="F294" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Which days survive.</t>
         </is>
       </c>
       <c r="G294" s="3" t="inlineStr">
@@ -34111,7 +34123,7 @@
       </c>
       <c r="F295" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Prune helper for the store writer: newest DAILY_KEEP days survive.</t>
         </is>
       </c>
       <c r="G295" s="3" t="inlineStr">
@@ -34189,7 +34201,7 @@
       </c>
       <c r="F296" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Publish the authoritative surplus for Goals/Retirement to consume.</t>
         </is>
       </c>
       <c r="G296" s="3" t="inlineStr">
@@ -34267,7 +34279,7 @@
       </c>
       <c r="F297" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G297" s="3" t="inlineStr">
@@ -34345,7 +34357,7 @@
       </c>
       <c r="F298" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The ONE reader every history surface uses: normalized, garbage-free, sorted by month.</t>
         </is>
       </c>
       <c r="G298" s="3" t="inlineStr">
@@ -34423,7 +34435,7 @@
       </c>
       <c r="F299" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Read a raw amount into a Money, given how that source signs things.</t>
         </is>
       </c>
       <c r="G299" s="3" t="inlineStr">
@@ -34501,7 +34513,7 @@
       </c>
       <c r="F300" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G300" s="3" t="inlineStr">
@@ -34579,7 +34591,7 @@
       </c>
       <c r="F301" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Real-estate use (primary/rental/secondary/land); only meaningful when assetClassOf === 'real_estate'.</t>
         </is>
       </c>
       <c r="G301" s="3" t="inlineStr">
@@ -34657,7 +34669,7 @@
       </c>
       <c r="F302" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How much profit have I actually taken?</t>
         </is>
       </c>
       <c r="G302" s="3" t="inlineStr">
@@ -34735,7 +34747,7 @@
       </c>
       <c r="F303" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G303" s="3" t="inlineStr">
@@ -34815,7 +34827,7 @@
       </c>
       <c r="F304" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>── the outside check ─────────────────────────────────────────────────────────────────────────── Our figure against the broker's own stated total.</t>
         </is>
       </c>
       <c r="G304" s="3" t="inlineStr">
@@ -34893,7 +34905,7 @@
       </c>
       <c r="F305" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>ASSERTION 1 — holdings + cash = the broker's stated total.</t>
         </is>
       </c>
       <c r="G305" s="3" t="inlineStr">
@@ -34971,7 +34983,7 @@
       </c>
       <c r="F306" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>ASSERTION 2 — the accounting identity every statement satisfies, exactly.</t>
         </is>
       </c>
       <c r="G306" s="3" t="inlineStr">
@@ -35049,7 +35061,7 @@
       </c>
       <c r="F307" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>── writing ───────────────────────────────────────────────────────────────────────────────────── Add a day.</t>
         </is>
       </c>
       <c r="G307" s="3" t="inlineStr">
@@ -35127,7 +35139,7 @@
       </c>
       <c r="F308" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Re-check verification status from the server (call after the user clicks the email link).</t>
         </is>
       </c>
       <c r="G308" s="3" t="inlineStr">
@@ -35205,7 +35217,7 @@
       </c>
       <c r="F309" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>Issue a NEW recovery code for the signed-in user (the old one stops working).</t>
         </is>
       </c>
       <c r="G309" s="3" t="inlineStr">
@@ -35285,7 +35297,7 @@
       </c>
       <c r="F310" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Returns the new user AND a one-time recovery code the caller MUST show the user to save.</t>
         </is>
       </c>
       <c r="G310" s="3" t="inlineStr">
@@ -35366,7 +35378,7 @@
       </c>
       <c r="F311" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G311" s="3" t="inlineStr">
@@ -35444,7 +35456,7 @@
       </c>
       <c r="F312" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Normalized list of rental properties.</t>
         </is>
       </c>
       <c r="G312" s="3" t="inlineStr">
@@ -35522,7 +35534,7 @@
       </c>
       <c r="F313" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Total net rental income per year, across all properties (income − operating expenses).</t>
         </is>
       </c>
       <c r="G313" s="3" t="inlineStr">
@@ -35600,7 +35612,7 @@
       </c>
       <c r="F314" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G314" s="3" t="inlineStr">
@@ -35678,7 +35690,7 @@
       </c>
       <c r="F315" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>THE YEARLY SAVING: the total annual contribution that reaches TARGET_ODDS on the real plan — the one with their age, their years left, their spending, their big costs.</t>
         </is>
       </c>
       <c r="G315" s="3" t="inlineStr">
@@ -35756,7 +35768,7 @@
       </c>
       <c r="F316" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>$/month still needed to hit the target on time (0 if already funded; null if no date/duration).</t>
         </is>
       </c>
       <c r="G316" s="3" t="inlineStr">
@@ -35835,7 +35847,7 @@
       </c>
       <c r="F317" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The payment reserved/required each month for a debt (planned payment, else the minimum).</t>
         </is>
       </c>
       <c r="G317" s="3" t="inlineStr">
@@ -35913,7 +35925,7 @@
       </c>
       <c r="F318" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Resend the verification email to the signed-in user.</t>
         </is>
       </c>
       <c r="G318" s="3" t="inlineStr">
@@ -35991,7 +36003,7 @@
       </c>
       <c r="F319" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G319" s="3" t="inlineStr">
@@ -36069,7 +36081,7 @@
       </c>
       <c r="F320" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The person's explicit choice (first-run stage question / Settings → Your setup) wins.</t>
         </is>
       </c>
       <c r="G320" s="3" t="inlineStr">
@@ -36147,7 +36159,7 @@
       </c>
       <c r="F321" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The single rule for which net-worth rows a live UI surface should use, so Home + TopBar + the Net Worth screen never disagree (B-49).</t>
         </is>
       </c>
       <c r="G321" s="3" t="inlineStr">
@@ -36229,7 +36241,7 @@
       </c>
       <c r="F322" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Restore the affected accounts to the transaction's pre-apply copies (pure).</t>
         </is>
       </c>
       <c r="G322" s="3" t="inlineStr">
@@ -36307,7 +36319,7 @@
       </c>
       <c r="F323" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>After a password reset, restore data access with the recovery code, then re-lock the data under the NEW password.</t>
         </is>
       </c>
       <c r="G323" s="3" t="inlineStr">
@@ -36387,7 +36399,7 @@
       </c>
       <c r="F324" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Earliest age the projection covers the need, WITH contributions until that age (F4's before/after).</t>
         </is>
       </c>
       <c r="G324" s="3" t="inlineStr">
@@ -36467,7 +36479,7 @@
       </c>
       <c r="F325" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Total nest egg = sum of each account's retirement-earmarked portion.</t>
         </is>
       </c>
       <c r="G325" s="3" t="inlineStr">
@@ -36549,7 +36561,7 @@
       </c>
       <c r="F326" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Years the money must last: retirement → plan-to age (default horizon if unset).</t>
         </is>
       </c>
       <c r="G326" s="3" t="inlineStr">
@@ -36627,7 +36639,7 @@
       </c>
       <c r="F327" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Retirement income (Social Security, pension, withdrawals, RMDs, annuities) per month — taxable.</t>
         </is>
       </c>
       <c r="G327" s="3" t="inlineStr">
@@ -36705,7 +36717,7 @@
       </c>
       <c r="F328" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>All-in monthly retirement spend = base + travel + medical (annual→monthly), adjusted by the expected trajectory (spend less / same / more later) and the retirement location's cost-of-living factor (retLocation).</t>
         </is>
       </c>
       <c r="G328" s="3" t="inlineStr">
@@ -36785,7 +36797,7 @@
       </c>
       <c r="F329" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Review new transactions against an account's history.</t>
         </is>
       </c>
       <c r="G329" s="3" t="inlineStr">
@@ -36863,7 +36875,7 @@
       </c>
       <c r="F330" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Re-lock an existing envelope's password copy under a new password (after a recovery-code restore).</t>
         </is>
       </c>
       <c r="G330" s="3" t="inlineStr">
@@ -36941,7 +36953,7 @@
       </c>
       <c r="F331" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Replace an envelope's recovery copy with a new recovery code (rotate the code).</t>
         </is>
       </c>
       <c r="G331" s="3" t="inlineStr">
@@ -37019,7 +37031,7 @@
       </c>
       <c r="F332" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Required minimum distribution from pre-tax balances at a given age (0 before the start age).</t>
         </is>
       </c>
       <c r="G332" s="3" t="inlineStr">
@@ -37098,7 +37110,7 @@
       </c>
       <c r="F333" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G333" s="3" t="inlineStr">
@@ -37176,7 +37188,7 @@
       </c>
       <c r="F334" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Year-by-year mandated-withdrawal schedule (ESTIMATES: future balances move with returns).</t>
         </is>
       </c>
       <c r="G334" s="3" t="inlineStr">
@@ -37258,7 +37270,7 @@
       </c>
       <c r="F335" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The age required withdrawals begin, by birth year.</t>
         </is>
       </c>
       <c r="G335" s="3" t="inlineStr">
@@ -37336,7 +37348,7 @@
       </c>
       <c r="F336" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>---- Required Minimum Distributions ---- B4 (founder brief 2026-08-20): the rule lives in ONE dated, sourced table — the Calculation Module's rmd engine.</t>
         </is>
       </c>
       <c r="G336" s="3" t="inlineStr">
@@ -37414,7 +37426,7 @@
       </c>
       <c r="F337" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The same rule when only an age is known (birth year ≈ this year − age; ±1 year of precision, which is what an age-only caller has).</t>
         </is>
       </c>
       <c r="G337" s="3" t="inlineStr">
@@ -37492,7 +37504,7 @@
       </c>
       <c r="F338" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Withdrawals already taken THIS year from the pre-tax accounts (the one ledger — no side lists).</t>
         </is>
       </c>
       <c r="G338" s="3" t="inlineStr">
@@ -37570,7 +37582,7 @@
       </c>
       <c r="F339" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>───────────────────────── Roth conversion (fill a low bracket) ───────────────────────── In a low-income year (e.g.</t>
         </is>
       </c>
       <c r="G339" s="3" t="inlineStr">
@@ -37649,7 +37661,7 @@
       </c>
       <c r="F340" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Are you in the low-income "Roth conversion window" (retired, before RMDs/SS push income up)?</t>
         </is>
       </c>
       <c r="G340" s="3" t="inlineStr">
@@ -37727,7 +37739,7 @@
       </c>
       <c r="F341" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Roth vs Traditional lean from current vs expected-retirement marginal rate (decimals).</t>
         </is>
       </c>
       <c r="G341" s="3" t="inlineStr">
@@ -37805,7 +37817,7 @@
       </c>
       <c r="F342" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G342" s="3" t="inlineStr">
@@ -37883,7 +37895,7 @@
       </c>
       <c r="F343" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Calendar year a row vests (first 4 digits of its date; this year if blank).</t>
         </is>
       </c>
       <c r="G343" s="3" t="inlineStr">
@@ -37961,7 +37973,7 @@
       </c>
       <c r="F344" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G344" s="3" t="inlineStr">
@@ -38039,7 +38051,7 @@
       </c>
       <c r="F345" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Annual equity-comp run-rate: total scheduled value spread over the years it vests across (a level annual figure for the income estimate).</t>
         </is>
       </c>
       <c r="G345" s="3" t="inlineStr">
@@ -38119,7 +38131,7 @@
       </c>
       <c r="F346" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Full sync. Returns the number of accounts synced (0 = nothing connected). */</t>
         </is>
       </c>
       <c r="G346" s="3" t="inlineStr">
@@ -38201,7 +38213,7 @@
       </c>
       <c r="F347" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How many months of the year you draw a salary.</t>
         </is>
       </c>
       <c r="G347" s="3" t="inlineStr">
@@ -38281,7 +38293,7 @@
       </c>
       <c r="F348" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Salary income for the year = sum of the per-month gross salary.</t>
         </is>
       </c>
       <c r="G348" s="3" t="inlineStr">
@@ -38361,7 +38373,7 @@
       </c>
       <c r="F349" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Per-month GROSS base salary, Jan→Dec.</t>
         </is>
       </c>
       <c r="G349" s="3" t="inlineStr">
@@ -38441,7 +38453,7 @@
       </c>
       <c r="F350" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The invitation under a sample: name the answers still missing, so a dead end becomes one tap.</t>
         </is>
       </c>
       <c r="G350" s="3" t="inlineStr">
@@ -38519,7 +38531,7 @@
       </c>
       <c r="F351" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The same sentence for the app-wide SAMPLE, always labelled as one.</t>
         </is>
       </c>
       <c r="G351" s="3" t="inlineStr">
@@ -38597,7 +38609,7 @@
       </c>
       <c r="F352" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G352" s="3" t="inlineStr">
@@ -38676,7 +38688,7 @@
       </c>
       <c r="F353" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G353" s="3" t="inlineStr">
@@ -38754,7 +38766,7 @@
       </c>
       <c r="F354" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G354" s="3" t="inlineStr">
@@ -38833,7 +38845,7 @@
       </c>
       <c r="F355" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G355" s="3" t="inlineStr">
@@ -38911,7 +38923,7 @@
       </c>
       <c r="F356" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G356" s="3" t="inlineStr">
@@ -38990,7 +39002,7 @@
       </c>
       <c r="F357" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G357" s="3" t="inlineStr">
@@ -39069,7 +39081,7 @@
       </c>
       <c r="F358" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Sync fields stored ENCRYPTED under users/{uid}.appStateEnc (zero-knowledge — see dataCrypto.ts).</t>
         </is>
       </c>
       <c r="G358" s="3" t="inlineStr">
@@ -39148,7 +39160,7 @@
       </c>
       <c r="F359" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The yearly saving whose PROJECTION reaches a typed target.</t>
         </is>
       </c>
       <c r="G359" s="3" t="inlineStr">
@@ -39227,7 +39239,7 @@
       </c>
       <c r="F360" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Discretionary amount free to save each month = take-home that month (after tax &amp; 401k) minus the spending due that month.</t>
         </is>
       </c>
       <c r="G360" s="3" t="inlineStr">
@@ -39313,7 +39325,7 @@
       </c>
       <c r="F361" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>── Required-withdrawal reminders (FCC Plan r48/r51 — logistics only, no timing advice) ── November 1 nudge ahead of the Dec 31 deadline (this year or a future start year).</t>
         </is>
       </c>
       <c r="G361" s="3" t="inlineStr">
@@ -39391,7 +39403,7 @@
       </c>
       <c r="F362" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>── Social Security claim-window reminder (design r18, built pre-48 per founder decision) ── Fires the month the claim window opens (their 62nd-birthday month), 10:00 on the 1st.</t>
         </is>
       </c>
       <c r="G362" s="3" t="inlineStr">
@@ -39469,7 +39481,7 @@
       </c>
       <c r="F363" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>── Schedule daily streak reminder ─────────────────────────────────</t>
         </is>
       </c>
       <c r="G363" s="3" t="inlineStr">
@@ -39547,7 +39559,7 @@
       </c>
       <c r="F364" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>── Weekly summary notification ────────────────────────────────────</t>
         </is>
       </c>
       <c r="G364" s="3" t="inlineStr">
@@ -39625,7 +39637,7 @@
       </c>
       <c r="F365" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Scholarships/grants placed in the calendar months they actually land (Jan→Dec) — NOT averaged.</t>
         </is>
       </c>
       <c r="G365" s="3" t="inlineStr">
@@ -39703,7 +39715,7 @@
       </c>
       <c r="F366" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The one will-it-last read.</t>
         </is>
       </c>
       <c r="G366" s="3" t="inlineStr">
@@ -39789,7 +39801,7 @@
       </c>
       <c r="F367" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>── Budget alert (fire immediately) ────────────────────────────────</t>
         </is>
       </c>
       <c r="G367" s="3" t="inlineStr">
@@ -39867,7 +39879,7 @@
       </c>
       <c r="F368" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>B-L2 verification: send a harmless test event so you can confirm wiring in the Sentry dashboard (works on the production/TestFlight build).</t>
         </is>
       </c>
       <c r="G368" s="3" t="inlineStr">
@@ -39945,7 +39957,7 @@
       </c>
       <c r="F369" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G369" s="3" t="inlineStr">
@@ -40023,7 +40035,7 @@
       </c>
       <c r="F370" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G370" s="3" t="inlineStr">
@@ -40101,7 +40113,7 @@
       </c>
       <c r="F371" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G371" s="3" t="inlineStr">
@@ -40179,7 +40191,7 @@
       </c>
       <c r="F372" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Write/merge a single-document-per-user collection, stamping last_updated.</t>
         </is>
       </c>
       <c r="G372" s="3" t="inlineStr">
@@ -40257,7 +40269,7 @@
       </c>
       <c r="F373" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Record household membership on the member's own user doc (survives reinstall/new device).</t>
         </is>
       </c>
       <c r="G373" s="3" t="inlineStr">
@@ -40335,7 +40347,7 @@
       </c>
       <c r="F374" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>Tag the current user on reports (call after login; pass null on logout).</t>
         </is>
       </c>
       <c r="G374" s="3" t="inlineStr">
@@ -40413,7 +40425,7 @@
       </c>
       <c r="F375" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The age the middle path first hits zero, from a simulation band — null while it never does.</t>
         </is>
       </c>
       <c r="G375" s="3" t="inlineStr">
@@ -40491,7 +40503,7 @@
       </c>
       <c r="F376" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G376" s="3" t="inlineStr">
@@ -40569,7 +40581,7 @@
       </c>
       <c r="F377" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The signed value, for arithmetic.</t>
         </is>
       </c>
       <c r="G377" s="3" t="inlineStr">
@@ -40647,7 +40659,7 @@
       </c>
       <c r="F378" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>B4 (founder brief 2026-08-20): the RMD rule lives in the ONE dated, sourced table — the Calculation Module's rmd engine.</t>
         </is>
       </c>
       <c r="G378" s="3" t="inlineStr">
@@ -40726,7 +40738,7 @@
       </c>
       <c r="F379" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G379" s="3" t="inlineStr">
@@ -40804,7 +40816,7 @@
       </c>
       <c r="F380" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Snapshot from onboarding answers alone — for headless/test callers (and any surface that runs before Net Worth is set up).</t>
         </is>
       </c>
       <c r="G380" s="3" t="inlineStr">
@@ -40890,7 +40902,7 @@
       </c>
       <c r="F381" s="3" t="inlineStr">
         <is>
-          <t>Reaches outside the app for its answer — a feed, a file or a stored record.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G381" s="3" t="inlineStr">
@@ -40969,7 +40981,7 @@
       </c>
       <c r="F382" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>"Even if you never save another dollar, you can retire at age Y." Earliest retire age where the current pot (no further contributions) already covers the plan.</t>
         </is>
       </c>
       <c r="G382" s="3" t="inlineStr">
@@ -41049,7 +41061,7 @@
       </c>
       <c r="F383" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Largest level monthly draw that keeps chance-of-success ≥ the floor.</t>
         </is>
       </c>
       <c r="G383" s="3" t="inlineStr">
@@ -41129,7 +41141,7 @@
       </c>
       <c r="F384" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>THE source wording (Build-47 walk row 8, audit Strategy #9): one sentence per source, used by every screen that names where an account's numbers come from.</t>
         </is>
       </c>
       <c r="G384" s="3" t="inlineStr">
@@ -41207,7 +41219,7 @@
       </c>
       <c r="F385" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Roll the per-category spending up into the three monthly-normalized buckets.</t>
         </is>
       </c>
       <c r="G385" s="3" t="inlineStr">
@@ -41287,7 +41299,7 @@
       </c>
       <c r="F386" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Spending placed in the calendar months it's actually due (Jan→Dec) — NOT averaged.</t>
         </is>
       </c>
       <c r="G386" s="3" t="inlineStr">
@@ -41368,7 +41380,7 @@
       </c>
       <c r="F387" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What the screen says at a given stepper position — a real run every time, never a bucket.</t>
         </is>
       </c>
       <c r="G387" s="3" t="inlineStr">
@@ -41446,7 +41458,7 @@
       </c>
       <c r="F388" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How much more she could spend, and how much of it is genuinely free.</t>
         </is>
       </c>
       <c r="G388" s="3" t="inlineStr">
@@ -41524,7 +41536,7 @@
       </c>
       <c r="F389" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Monthly benefit at a claim age from the at-FRA statement amount (today's dollars, whole $).</t>
         </is>
       </c>
       <c r="G389" s="3" t="inlineStr">
@@ -41602,7 +41614,7 @@
       </c>
       <c r="F390" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Kept for callers not yet passing a birth year (behaves as born-1960+).</t>
         </is>
       </c>
       <c r="G390" s="3" t="inlineStr">
@@ -41680,7 +41692,7 @@
       </c>
       <c r="F391" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>The pre-table factor, anchored at 67 — unchanged behaviour for anyone born 1960+.</t>
         </is>
       </c>
       <c r="G391" s="3" t="inlineStr">
@@ -41758,7 +41770,7 @@
       </c>
       <c r="F392" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>SSA factor for a claim age (62–70), relative to the statement amount at the person's OWN full retirement age.</t>
         </is>
       </c>
       <c r="G392" s="3" t="inlineStr">
@@ -41836,7 +41848,7 @@
       </c>
       <c r="F393" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Total collected from claim age to a live-to age the USER sets (months × monthly, today's dollars).</t>
         </is>
       </c>
       <c r="G393" s="3" t="inlineStr">
@@ -41914,7 +41926,7 @@
       </c>
       <c r="F394" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The Social Security stream inside an input set, when streams are in use.</t>
         </is>
       </c>
       <c r="G394" s="3" t="inlineStr">
@@ -41992,7 +42004,7 @@
       </c>
       <c r="F395" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Social Security pays roughly 8% more for each year you delay past full retirement age — the claim-later lever has to raise the CHECK, not just move its start date.</t>
         </is>
       </c>
       <c r="G395" s="3" t="inlineStr">
@@ -42070,7 +42082,7 @@
       </c>
       <c r="F396" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>What do we call this connected account internally?</t>
         </is>
       </c>
       <c r="G396" s="3" t="inlineStr">
@@ -42148,7 +42160,7 @@
       </c>
       <c r="F397" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>---- period returns from a price series (price return of the security itself) ----</t>
         </is>
       </c>
       <c r="G397" s="3" t="inlineStr">
@@ -42226,7 +42238,7 @@
       </c>
       <c r="F398" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What state tax rate applies?</t>
         </is>
       </c>
       <c r="G398" s="3" t="inlineStr">
@@ -42304,7 +42316,7 @@
       </c>
       <c r="F399" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>A DATE IS NOT MONEY.</t>
         </is>
       </c>
       <c r="G399" s="3" t="inlineStr">
@@ -42382,7 +42394,7 @@
       </c>
       <c r="F400" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G400" s="3" t="inlineStr">
@@ -42460,7 +42472,7 @@
       </c>
       <c r="F401" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Add money SIGNED and EXACTLY — a credit and its reversal cancel to true zero, so a reconciliation can assert equality rather than a tolerance.</t>
         </is>
       </c>
       <c r="G401" s="3" t="inlineStr">
@@ -42538,7 +42550,7 @@
       </c>
       <c r="F402" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Planned SURPLUS, month by month, AFTER debt (the canonical word, per the 2026-06-23 decision).</t>
         </is>
       </c>
       <c r="G402" s="3" t="inlineStr">
@@ -42624,7 +42636,7 @@
       </c>
       <c r="F403" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Bottom-bar order per lens (design pin: "Tab order is set once from stage; identical across sessions").</t>
         </is>
       </c>
       <c r="G403" s="3" t="inlineStr">
@@ -42702,7 +42714,7 @@
       </c>
       <c r="F404" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>True take-home per month: after tax AND after the 401(k) deduction (the cash that hits your account).</t>
         </is>
       </c>
       <c r="G404" s="3" t="inlineStr">
@@ -42788,7 +42800,7 @@
       </c>
       <c r="F405" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>THE TARGET: the balance on day one of retirement that reaches TARGET_ODDS.</t>
         </is>
       </c>
       <c r="G405" s="3" t="inlineStr">
@@ -42866,7 +42878,7 @@
       </c>
       <c r="F406" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How is the retirement money split by the tax that will be owed on it?</t>
         </is>
       </c>
       <c r="G406" s="3" t="inlineStr">
@@ -42947,7 +42959,7 @@
       </c>
       <c r="F407" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G407" s="3" t="inlineStr">
@@ -43033,7 +43045,7 @@
       </c>
       <c r="F408" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Federal tax owed: progressive brackets applied to income after the standard deduction.</t>
         </is>
       </c>
       <c r="G408" s="3" t="inlineStr">
@@ -43111,7 +43123,7 @@
       </c>
       <c r="F409" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Federal tax owed under a filing status, plus an optional user-set FLAT state rate applied to TAXABLE income (E10) — states differ wildly, so one honest user-entered percent beats fifty guessed tables, and it never taxes the deduction.</t>
         </is>
       </c>
       <c r="G409" s="3" t="inlineStr">
@@ -43189,7 +43201,7 @@
       </c>
       <c r="F410" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>HOW the account is taxed (wrapper).</t>
         </is>
       </c>
       <c r="G410" s="3" t="inlineStr">
@@ -43267,7 +43279,7 @@
       </c>
       <c r="F411" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Taxable annual income (excludes non-taxable benefits/support/scholarships) — the base for tax estimates.</t>
         </is>
       </c>
       <c r="G411" s="3" t="inlineStr">
@@ -43353,7 +43365,7 @@
       </c>
       <c r="F412" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The calendar-year TAXABLE profile (Jan→Dec) — the same placement rules incomeMonthlyGrid uses, extracted so the rate vector and the grid can never drift apart.</t>
         </is>
       </c>
       <c r="G412" s="3" t="inlineStr">
@@ -43439,7 +43451,7 @@
       </c>
       <c r="F413" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Taxable income after the standard deduction.</t>
         </is>
       </c>
       <c r="G413" s="3" t="inlineStr">
@@ -43517,7 +43529,7 @@
       </c>
       <c r="F414" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What income is taxed, given how this person files?</t>
         </is>
       </c>
       <c r="G414" s="3" t="inlineStr">
@@ -43595,7 +43607,7 @@
       </c>
       <c r="F415" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Tips are part of employment income — they only count in the months the job is active, and the annual figure is prorated like salary (a temp job that ends stops the tips too).</t>
         </is>
       </c>
       <c r="G415" s="3" t="inlineStr">
@@ -43676,7 +43688,7 @@
       </c>
       <c r="F416" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Read one institution row into one ledger row.</t>
         </is>
       </c>
       <c r="G416" s="3" t="inlineStr">
@@ -43757,7 +43769,7 @@
       </c>
       <c r="F417" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>What number did the person actually type?</t>
         </is>
       </c>
       <c r="G417" s="3" t="inlineStr">
@@ -43835,7 +43847,7 @@
       </c>
       <c r="F418" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Institution files write money as text: "$8,502.00 ", "($0.53)", "--", "1,234.56".</t>
         </is>
       </c>
       <c r="G418" s="3" t="inlineStr">
@@ -43913,7 +43925,7 @@
       </c>
       <c r="F419" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Build the public read-model (profile + derived planning values).</t>
         </is>
       </c>
       <c r="G419" s="3" t="inlineStr">
@@ -43993,7 +44005,7 @@
       </c>
       <c r="F420" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The holding-concentration FACT (Invest main + the insights engine share this one rule): the largest single holding as a % of invested money, reported only at 25%+ with 2+ holdings — below that it isn't a fact worth a card.</t>
         </is>
       </c>
       <c r="G420" s="3" t="inlineStr">
@@ -44071,7 +44083,7 @@
       </c>
       <c r="F421" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G421" s="3" t="inlineStr">
@@ -44149,7 +44161,7 @@
       </c>
       <c r="F422" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Σ outstanding debt BALANCE — what you still owe (not a monthly payment).</t>
         </is>
       </c>
       <c r="G422" s="3" t="inlineStr">
@@ -44227,7 +44239,7 @@
       </c>
       <c r="F423" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Total monthly debt obligation across all debts (override-aware).</t>
         </is>
       </c>
       <c r="G423" s="3" t="inlineStr">
@@ -44305,7 +44317,7 @@
       </c>
       <c r="F424" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Total annual income across every inflow (salary for months worked + bonus + signing + equity + net rental + self-employment/investment/benefits/support/scholarship/other).</t>
         </is>
       </c>
       <c r="G424" s="3" t="inlineStr">
@@ -44391,7 +44403,7 @@
       </c>
       <c r="F425" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>A total, summed SIGNED and EXACT — a reversal reduces its total instead of inflating it.</t>
         </is>
       </c>
       <c r="G425" s="3" t="inlineStr">
@@ -44469,7 +44481,7 @@
       </c>
       <c r="F426" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Total return since purchase = gain / cost basis (decimal).</t>
         </is>
       </c>
       <c r="G426" s="3" t="inlineStr">
@@ -44551,7 +44563,7 @@
       </c>
       <c r="F427" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>---- cost basis &amp; value (lot math) ----</t>
         </is>
       </c>
       <c r="G427" s="3" t="inlineStr">
@@ -44629,7 +44641,7 @@
       </c>
       <c r="F428" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Does this event add to that total?</t>
         </is>
       </c>
       <c r="G428" s="3" t="inlineStr">
@@ -44707,7 +44719,7 @@
       </c>
       <c r="F429" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Chart series = monthly snapshots + daily points, chronological ('YYYY-MM' sorts before its days).</t>
         </is>
       </c>
       <c r="G429" s="3" t="inlineStr">
@@ -44786,7 +44798,7 @@
       </c>
       <c r="F430" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>One hint per active goal: the SAME weigher re-run with that dial reduced — a pre-run of the slider, so applying the hint's amount reproduces its numbers exactly (the pin).</t>
         </is>
       </c>
       <c r="G430" s="3" t="inlineStr">
@@ -44872,7 +44884,7 @@
       </c>
       <c r="F431" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What do we call this kind of row on screen?</t>
         </is>
       </c>
       <c r="G431" s="3" t="inlineStr">
@@ -44950,7 +44962,7 @@
       </c>
       <c r="F432" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G432" s="3" t="inlineStr">
@@ -45028,7 +45040,7 @@
       </c>
       <c r="F433" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Group per-class totals into the three uber-groups, keeping class order inside each.</t>
         </is>
       </c>
       <c r="G433" s="3" t="inlineStr">
@@ -45107,7 +45119,7 @@
       </c>
       <c r="F434" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Everything we could not name, for the honest line on screen: "12 entries we could not classify".</t>
         </is>
       </c>
       <c r="G434" s="3" t="inlineStr">
@@ -45185,7 +45197,7 @@
       </c>
       <c r="F435" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>Deep copies of the affected accounts, taken BEFORE applyTransaction.</t>
         </is>
       </c>
       <c r="G435" s="3" t="inlineStr">
@@ -45263,7 +45275,7 @@
       </c>
       <c r="F436" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>How many units of one holding were held on a date — what the trend chart needs and never had.</t>
         </is>
       </c>
       <c r="G436" s="3" t="inlineStr">
@@ -45341,7 +45353,7 @@
       </c>
       <c r="F437" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Unrealized gain = market value − cost basis (null price → 0).</t>
         </is>
       </c>
       <c r="G437" s="3" t="inlineStr">
@@ -45422,7 +45434,7 @@
       </c>
       <c r="F438" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Unlock the DEK with the password (null if the password is wrong / was reset).</t>
         </is>
       </c>
       <c r="G438" s="3" t="inlineStr">
@@ -45500,7 +45512,7 @@
       </c>
       <c r="F439" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Unlock the DEK with the recovery code (null if the code is wrong).</t>
         </is>
       </c>
       <c r="G439" s="3" t="inlineStr">
@@ -45578,7 +45590,7 @@
       </c>
       <c r="F440" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G440" s="3" t="inlineStr">
@@ -45664,7 +45676,7 @@
       </c>
       <c r="F441" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>USD cash across the balances list (v1 is USD-only; other currencies are ignored, not guessed).</t>
         </is>
       </c>
       <c r="G441" s="3" t="inlineStr">
@@ -45742,7 +45754,7 @@
       </c>
       <c r="F442" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, but no chain from it reaches a screen.</t>
+          <t>PRD F3#17 — the user's OWN capital-gains rates (long: 0/15/20 ladder by filing status; short: their marginal bracket), each plus the flat state rate.</t>
         </is>
       </c>
       <c r="G442" s="3" t="inlineStr">
@@ -45828,7 +45840,7 @@
       </c>
       <c r="F443" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>The user's dated flows for a measured set of accounts, investor-sign convention: money the user PUT IN is negative, money TAKEN OUT is positive.</t>
         </is>
       </c>
       <c r="G443" s="3" t="inlineStr">
@@ -45906,7 +45918,7 @@
       </c>
       <c r="F444" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Manual-value freshness (FCC): how old a hand-entered value is, and whether it needs a nudge.</t>
         </is>
       </c>
       <c r="G444" s="3" t="inlineStr">
@@ -45984,7 +45996,7 @@
       </c>
       <c r="F445" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>── reading ───────────────────────────────────────────────────────────────────────────────────── What one account was worth on a date — the figure the old code had to back-solve.</t>
         </is>
       </c>
       <c r="G445" s="3" t="inlineStr">
@@ -46063,7 +46075,7 @@
       </c>
       <c r="F446" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Same volatility convention as the cockpit: higher return ⇒ more volatility.</t>
         </is>
       </c>
       <c r="G446" s="3" t="inlineStr">
@@ -46142,7 +46154,7 @@
       </c>
       <c r="F447" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G447" s="3" t="inlineStr">
@@ -46220,7 +46232,7 @@
       </c>
       <c r="F448" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>Run the whole combination once.</t>
         </is>
       </c>
       <c r="G448" s="3" t="inlineStr">
@@ -46306,7 +46318,7 @@
       </c>
       <c r="F449" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>What goes into working out the odds?</t>
         </is>
       </c>
       <c r="G449" s="3" t="inlineStr">
@@ -46392,7 +46404,7 @@
       </c>
       <c r="F450" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G450" s="3" t="inlineStr">
@@ -46470,7 +46482,7 @@
       </c>
       <c r="F451" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>An input set with its Social Security stream replaced — the ONE way a decision screen patches a claim scenario, so the flat streams ride along untouched and the legacy fields stay in step for anything still reading them.</t>
         </is>
       </c>
       <c r="G451" s="3" t="inlineStr">
@@ -46548,7 +46560,7 @@
       </c>
       <c r="F452" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G452" s="3" t="inlineStr">
@@ -46629,7 +46641,7 @@
       </c>
       <c r="F453" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G453" s="3" t="inlineStr">
@@ -46707,7 +46719,7 @@
       </c>
       <c r="F454" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>The person picked how this account is taxed — what does that make it?</t>
         </is>
       </c>
       <c r="G454" s="3" t="inlineStr">
@@ -46785,7 +46797,7 @@
       </c>
       <c r="F455" s="3" t="inlineStr">
         <is>
-          <t>Produces nothing that is displayed — it does something: saves, syncs or records.</t>
+          <t>NOT DETERMINED — the code carries no note saying what this is for, and it has no row in the old inventory. Needs reading.</t>
         </is>
       </c>
       <c r="G455" s="3" t="inlineStr">
@@ -46863,7 +46875,7 @@
       </c>
       <c r="F456" s="3" t="inlineStr">
         <is>
-          <t>A screen calls it directly, so its answer is on a screen.</t>
+          <t>How long until this bond pays back?</t>
         </is>
       </c>
       <c r="G456" s="3" t="inlineStr">
@@ -46941,7 +46953,7 @@
       </c>
       <c r="F457" s="3" t="inlineStr">
         <is>
-          <t>Its answer feeds another function, and that chain ends at a screen.</t>
+          <t>Years until the target retirement age (never negative).</t>
         </is>
       </c>
       <c r="G457" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Assumptions now name the actual value, not the shape of the problem
They said things like "carries a built-in rate that nobody chose". They
now say which rate and how much: if the return is missing it uses 6% ·
never lets the answer fall below 5% or rise above 20% · if the tax rate
on a required withdrawal is missing it uses 22% · if the number of runs
is missing it uses 500 · treats a year as twelve equal months.

Names are turned into words a person would say, and rates written as
percentages rather than decimals.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
+++ b/MoneyKeel/documents/other/moneykeel_calc_master_calculation-master_v01.xlsx
@@ -11173,10 +11173,10 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If cash balance is missing it uses 0.
+· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If value is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -11930,8 +11930,8 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If amount is missing it uses 0.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -12188,8 +12188,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If allocated this month is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -12272,9 +12271,8 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If by kind[k] is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -12357,8 +12355,9 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -13031,7 +13030,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If operating expenses is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -13114,7 +13113,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 12 instead of refusing.
+          <t>· If salary freq] is missing it uses 12.
 · Treats a year as twelve equal months.</t>
         </is>
       </c>
@@ -13198,8 +13197,11 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If price is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If amount is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -13283,8 +13285,8 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -13368,7 +13370,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -13705,7 +13707,8 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -13871,9 +13874,8 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Applies a built-in rate of 25% to avg.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -14207,7 +14209,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0.06 instead of refusing.</t>
+          <t>· If return is missing it uses 6%.</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -14373,7 +14375,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -14540,7 +14542,8 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -14627,8 +14630,9 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0.12 instead of refusing.
-· Rounds the answer.</t>
+          <t>· If v is missing it uses 12%.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -14714,7 +14718,9 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If face value is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If coupon rate is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
@@ -14797,10 +14803,9 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Applies a built-in rate of 99% to v.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
@@ -14884,8 +14889,9 @@
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
@@ -15060,7 +15066,8 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
@@ -15147,8 +15154,8 @@
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
@@ -15231,7 +15238,7 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If monthly spending is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
@@ -15314,8 +15321,11 @@
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If contributions is missing it uses 0.
+· If withdrawals is missing it uses 0.
+· If dividends is missing it uses 0.
+· If interest is missing it uses 0.
+· If debt principal is missing it uses 0.</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
@@ -15398,11 +15408,16 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Uses today's date from the device clock.
+          <t>· If year is missing it uses 0.
+· If a year is missing it uses 0.
+· If start balance is missing it uses 0.
+· Uses a built-in s of 0.
+· Uses a built-in q of 0.
+· Uses a built-in t of 0.
 · Treats a year as twelve equal months.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
@@ -15493,10 +15508,12 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it uses 0.
+· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If cost per share is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses a built-in d a i l y y e a r s of 2.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -15579,7 +15596,7 @@
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
@@ -15750,9 +15767,10 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
+          <t>· Uses a built-in i of 0.
 · Treats a year as twelve equal months.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
@@ -15840,7 +15858,7 @@
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
@@ -15923,7 +15941,8 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If value is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If coupon rate is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
@@ -16091,9 +16110,11 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 80 instead of refusing.
-· Uses today's date from the device clock.
-· Treats a year as twelve equal months.</t>
+          <t>· If chance floor is missing it uses 80.
+· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
@@ -16184,8 +16205,8 @@
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
@@ -16276,7 +16297,7 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 500 instead of refusing.</t>
+          <t>· If paths is missing it uses 500.</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
@@ -16360,9 +16381,9 @@
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 35 instead of refusing.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If current age is missing it uses 35.
+· If target retirement age is missing it uses 65.
+· If plan to age is missing it uses 90.</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
@@ -16702,7 +16723,7 @@
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
@@ -16785,9 +16806,9 @@
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
@@ -16953,7 +16974,9 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If price is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If amount is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
@@ -17036,7 +17059,7 @@
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
@@ -17123,10 +17146,12 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
+          <t>· Uses a built-in beyond window of 0.
+· Uses a built-in s of 0.
 · Treats a year as twelve equal months.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
@@ -17217,7 +17242,8 @@
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>· Treats a year as twelve equal months.</t>
+          <t>· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
@@ -17383,7 +17409,7 @@
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
@@ -17549,7 +17575,7 @@
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in i of 0.</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
@@ -17881,9 +17907,10 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Shows 2 decimal place(s).
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Uses a built-in lifetime of 0.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Shows 2 decimal places.</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
@@ -18049,7 +18076,7 @@
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
@@ -18216,7 +18243,8 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If cost per share is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
@@ -18299,7 +18327,8 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.</t>
+          <t>· Uses a built-in d e f a u l t b o n d y i e l d of 4.2%.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
@@ -18801,7 +18830,7 @@
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
@@ -18967,7 +18996,7 @@
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
@@ -19299,7 +19328,7 @@
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K100" s="3" t="inlineStr">
@@ -19382,8 +19411,9 @@
       </c>
       <c r="J101" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Treats a year as 365 days.</t>
+          <t>· If shares is missing it uses 0.
+· Treats a year as 365 days.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K101" s="3" t="inlineStr">
@@ -19549,7 +19579,7 @@
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.</t>
+          <t>· Uses a built-in t o x i c a p r of 7%.</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
@@ -19632,7 +19662,7 @@
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K104" s="3" t="inlineStr">
@@ -19800,7 +19830,10 @@
       </c>
       <c r="J106" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in start of 0.
+· Uses a built-in nul of 0.
+· Uses a built-in i of 0.
+· Caps length at 400.</t>
         </is>
       </c>
       <c r="K106" s="3" t="inlineStr">
@@ -20051,7 +20084,7 @@
       </c>
       <c r="J109" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K109" s="3" t="inlineStr">
@@ -20387,9 +20420,8 @@
       </c>
       <c r="J113" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If pre tax share is missing it uses 0.
+· If required withdrawal tax rate is missing it uses 22%.</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">
@@ -20557,8 +20589,7 @@
       </c>
       <c r="J115" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K115" s="3" t="inlineStr">
@@ -20641,9 +20672,10 @@
       </c>
       <c r="J116" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0.22 instead of refusing.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If ordinary rate is missing it uses 22%.
+· If cap gains rate is missing it uses 15%.
+· If gain share is missing it uses 50%.
+· Uses a built-in taxes of 0.</t>
         </is>
       </c>
       <c r="K116" s="3" t="inlineStr">
@@ -20729,7 +20761,7 @@
       </c>
       <c r="J117" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K117" s="3" t="inlineStr">
@@ -20896,8 +20928,7 @@
       </c>
       <c r="J119" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K119" s="3" t="inlineStr">
@@ -20982,7 +21013,8 @@
       </c>
       <c r="J120" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.</t>
+          <t>· Uses a built-in d e f a u l t r e t u r n of 7%.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K120" s="3" t="inlineStr">
@@ -21067,10 +21099,12 @@
       </c>
       <c r="J121" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
+          <t>· Uses a built-in future total cost of 0.
+· Uses a built-in y of 0.
 · Treats a year as twelve equal months.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Caps the answer at a limit rather than letting it run.</t>
+· Turns a monthly figure into a year by multiplying by twelve.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K121" s="3" t="inlineStr">
@@ -21153,7 +21187,7 @@
       </c>
       <c r="J122" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K122" s="3" t="inlineStr">
@@ -21244,7 +21278,7 @@
       </c>
       <c r="J123" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K123" s="3" t="inlineStr">
@@ -21501,10 +21535,12 @@
       </c>
       <c r="J126" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 12 instead of refusing.
+          <t>· If landing month is missing it uses 12.
+· If landing month is missing it uses 1.
+· If operating expenses is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses a built-in i of 0.
 · Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+· Never lets manual effective tax rate fall below 0.</t>
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr">
@@ -21587,7 +21623,7 @@
       </c>
       <c r="J127" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K127" s="3" t="inlineStr">
@@ -21761,7 +21797,7 @@
       </c>
       <c r="J129" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If employer match amount is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K129" s="3" t="inlineStr">
@@ -22177,8 +22213,10 @@
       </c>
       <c r="J134" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in total of 0.
+· Uses a built-in i of 0.
+· Uses a built-in d a y m s of 86400000.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K134" s="3" t="inlineStr">
@@ -22264,7 +22302,7 @@
       </c>
       <c r="J135" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K135" s="3" t="inlineStr">
@@ -22348,7 +22386,7 @@
       </c>
       <c r="J136" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K136" s="3" t="inlineStr">
@@ -22431,7 +22469,7 @@
       </c>
       <c r="J137" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in total v of 0.</t>
         </is>
       </c>
       <c r="K137" s="3" t="inlineStr">
@@ -22683,7 +22721,7 @@
       </c>
       <c r="J140" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K140" s="3" t="inlineStr">
@@ -22766,9 +22804,9 @@
       </c>
       <c r="J141" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K141" s="3" t="inlineStr">
@@ -22851,7 +22889,7 @@
       </c>
       <c r="J142" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K142" s="3" t="inlineStr">
@@ -23183,7 +23221,7 @@
       </c>
       <c r="J146" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K146" s="3" t="inlineStr">
@@ -23266,7 +23304,7 @@
       </c>
       <c r="J147" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K147" s="3" t="inlineStr">
@@ -23432,7 +23470,8 @@
       </c>
       <c r="J149" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K149" s="3" t="inlineStr">
@@ -23764,7 +23803,7 @@
       </c>
       <c r="J153" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in i of 0.</t>
         </is>
       </c>
       <c r="K153" s="3" t="inlineStr">
@@ -24360,7 +24399,7 @@
       </c>
       <c r="J160" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K160" s="3" t="inlineStr">
@@ -24443,10 +24482,10 @@
       </c>
       <c r="J161" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If target is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If saved is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K161" s="3" t="inlineStr">
@@ -24529,8 +24568,10 @@
       </c>
       <c r="J162" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If saved is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If target is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If funded this month is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K162" s="3" t="inlineStr">
@@ -24614,7 +24655,7 @@
       </c>
       <c r="J163" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K163" s="3" t="inlineStr">
@@ -24781,7 +24822,8 @@
       </c>
       <c r="J165" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Uses a built-in i of 0.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K165" s="3" t="inlineStr">
@@ -24864,7 +24906,7 @@
       </c>
       <c r="J166" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K166" s="3" t="inlineStr">
@@ -24949,7 +24991,7 @@
       </c>
       <c r="J167" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If rate is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K167" s="3" t="inlineStr">
@@ -25032,7 +25074,7 @@
       </c>
       <c r="J168" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 1 instead of refusing.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K168" s="3" t="inlineStr">
@@ -25115,9 +25157,10 @@
       </c>
       <c r="J169" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
+          <t>· Uses a built-in q of 0.
+· Uses a built-in s of 0.
 · Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K169" s="3" t="inlineStr">
@@ -25200,10 +25243,11 @@
       </c>
       <c r="J170" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.
-· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Treats a month as 30 days.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K170" s="3" t="inlineStr">
@@ -25286,7 +25330,9 @@
       </c>
       <c r="J171" s="3" t="inlineStr">
         <is>
-          <t>· Treats a year as 365 days.</t>
+          <t>· Uses a built-in v of 0.
+· Treats a year as 365 days.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K171" s="3" t="inlineStr">
@@ -25452,8 +25498,7 @@
       </c>
       <c r="J173" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K173" s="3" t="inlineStr">
@@ -25537,7 +25582,7 @@
       </c>
       <c r="J174" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in skipped of 0.</t>
         </is>
       </c>
       <c r="K174" s="3" t="inlineStr">
@@ -25788,7 +25833,7 @@
       <c r="J177" s="3" t="inlineStr">
         <is>
           <t>· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K177" s="3" t="inlineStr">
@@ -25879,9 +25924,8 @@
       </c>
       <c r="J178" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Treats a year as twelve equal months.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K178" s="3" t="inlineStr">
@@ -26055,11 +26099,16 @@
       </c>
       <c r="J180" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Uses today's date from the device clock.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If cost per share is missing it uses 0.
+· If target return is missing it uses 8%.
+· If balance is missing it uses 0.
+· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If cost per share is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If value is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K180" s="3" t="inlineStr">
@@ -26233,9 +26282,12 @@
       </c>
       <c r="J182" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If coupon rate is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If face value is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses a built-in pv of 0.
+· Uses a built-in t of 1.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K182" s="3" t="inlineStr">
@@ -26489,7 +26541,8 @@
       </c>
       <c r="J185" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K185" s="3" t="inlineStr">
@@ -26572,8 +26625,9 @@
       </c>
       <c r="J186" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If amount is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K186" s="3" t="inlineStr">
@@ -27237,7 +27291,14 @@
       </c>
       <c r="J194" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in l a r g e m u l t i p l e of 3.
+· Uses a built-in l a r g e f l o o r of 500.
+· Uses a built-in l a r g e c o l d s t a r t of 1000.
+· Uses a built-in m i n h i s t o r y of 5.
+· Uses a built-in p a y e e f l o o r of 250.
+· Uses a built-in p a t t e r n c o u n t of 3.
+· Uses a built-in p a t t e r n t o t a l of 1000.
+· Uses a built-in h i s t o r y d a y s of 90.</t>
         </is>
       </c>
       <c r="K194" s="3" t="inlineStr">
@@ -27486,7 +27547,8 @@
       </c>
       <c r="J197" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K197" s="3" t="inlineStr">
@@ -27570,7 +27632,7 @@
       </c>
       <c r="J198" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If lump balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K198" s="3" t="inlineStr">
@@ -27740,7 +27802,7 @@
       </c>
       <c r="J200" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If value is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K200" s="3" t="inlineStr">
@@ -27823,7 +27885,7 @@
       </c>
       <c r="J201" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K201" s="3" t="inlineStr">
@@ -27991,8 +28053,7 @@
       </c>
       <c r="J203" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K203" s="3" t="inlineStr">
@@ -28158,9 +28219,12 @@
       </c>
       <c r="J205" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 2 instead of refusing.
-· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If retire later years is missing it uses 2.
+· If spend cut monthly is missing it uses 400.
+· If claim age is missing it uses 70.
+· If guaranteed monthly income is missing it uses 0.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K205" s="3" t="inlineStr">
@@ -28245,7 +28309,7 @@
       </c>
       <c r="J206" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K206" s="3" t="inlineStr">
@@ -28996,8 +29060,9 @@
       </c>
       <c r="J215" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Treats a year as twelve equal months.</t>
+          <t>· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K215" s="3" t="inlineStr">
@@ -29250,8 +29315,8 @@
       </c>
       <c r="J218" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K218" s="3" t="inlineStr">
@@ -29750,7 +29815,7 @@
       </c>
       <c r="J224" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K224" s="3" t="inlineStr">
@@ -29916,7 +29981,7 @@
       </c>
       <c r="J226" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>· If amount is missing it uses 0.</t>
         </is>
       </c>
       <c r="K226" s="3" t="inlineStr">
@@ -29999,9 +30064,10 @@
       </c>
       <c r="J227" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· If units is missing it uses 0.
+· If price is missing it uses 0.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K227" s="3" t="inlineStr">
@@ -30084,7 +30150,9 @@
       </c>
       <c r="J228" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>· If units is missing it uses 0.
+· If quantity is missing it uses 0.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K228" s="3" t="inlineStr">
@@ -30417,7 +30485,8 @@
       </c>
       <c r="J232" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K232" s="3" t="inlineStr">
@@ -30667,7 +30736,7 @@
       </c>
       <c r="J235" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K235" s="3" t="inlineStr">
@@ -30833,7 +30902,7 @@
       </c>
       <c r="J237" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in floor of 0.</t>
         </is>
       </c>
       <c r="K237" s="3" t="inlineStr">
@@ -30916,8 +30985,8 @@
       </c>
       <c r="J238" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Shows 1 decimal place(s).</t>
+          <t>· Rounds the answer to a whole number.
+· Shows 1 decimal place.</t>
         </is>
       </c>
       <c r="K238" s="3" t="inlineStr">
@@ -31000,7 +31069,7 @@
       </c>
       <c r="J239" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If minimum monthly payment is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K239" s="3" t="inlineStr">
@@ -31250,8 +31319,8 @@
       </c>
       <c r="J242" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Shows 2 decimal place(s).</t>
+          <t>· Rounds the answer to a whole number.
+· Shows 2 decimal places.</t>
         </is>
       </c>
       <c r="K242" s="3" t="inlineStr">
@@ -31334,9 +31403,10 @@
       </c>
       <c r="J243" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in i of 0.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K243" s="3" t="inlineStr">
@@ -31587,7 +31657,7 @@
       </c>
       <c r="J246" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in ess of 0.</t>
         </is>
       </c>
       <c r="K246" s="3" t="inlineStr">
@@ -31769,9 +31839,7 @@
       </c>
       <c r="J248" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K248" s="3" t="inlineStr">
@@ -31945,8 +32013,8 @@
       </c>
       <c r="J250" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If target is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If saved is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K250" s="3" t="inlineStr">
@@ -32029,7 +32097,7 @@
       </c>
       <c r="J251" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K251" s="3" t="inlineStr">
@@ -32112,7 +32180,8 @@
       </c>
       <c r="J252" s="3" t="inlineStr">
         <is>
-          <t>· Treats a year as twelve equal months.</t>
+          <t>· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K252" s="3" t="inlineStr">
@@ -32280,9 +32349,11 @@
       </c>
       <c r="J254" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· If price is missing it uses 0.
+· If balances cash is missing it uses 0.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K254" s="3" t="inlineStr">
@@ -32365,7 +32436,7 @@
       </c>
       <c r="J255" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K255" s="3" t="inlineStr">
@@ -32448,8 +32519,10 @@
       </c>
       <c r="J256" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses a built-in s a m p l e c h a n c e of 84.
+· Uses a built-in s a m p l e h o r i z o n of 90.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K256" s="3" t="inlineStr">
@@ -32535,7 +32608,8 @@
       </c>
       <c r="J257" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K257" s="3" t="inlineStr">
@@ -33117,9 +33191,8 @@
       </c>
       <c r="J264" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If leftover at horizon is missing it uses 0.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K264" s="3" t="inlineStr">
@@ -33285,7 +33358,7 @@
       </c>
       <c r="J266" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K266" s="3" t="inlineStr">
@@ -33368,7 +33441,7 @@
       </c>
       <c r="J267" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K267" s="3" t="inlineStr">
@@ -33451,7 +33524,8 @@
       </c>
       <c r="J268" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in i of 0.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K268" s="3" t="inlineStr">
@@ -33617,8 +33691,12 @@
       </c>
       <c r="J270" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Uses today's date from the device clock.</t>
+          <t>· Uses a built-in strong t of 0.
+· Uses a built-in weak t of 0.
+· Uses a built-in subtotal of 0.
+· Uses a built-in largest safe of 0.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K270" s="3" t="inlineStr">
@@ -33868,7 +33946,7 @@
       <c r="J273" s="3" t="inlineStr">
         <is>
           <t>· Treats a year as twelve equal months.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.</t>
         </is>
       </c>
       <c r="K273" s="3" t="inlineStr">
@@ -33951,10 +34029,11 @@
       </c>
       <c r="J274" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
+          <t>· Uses a built-in month of 0.
 · Treats a year as twelve equal months.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K274" s="3" t="inlineStr">
@@ -34038,8 +34117,9 @@
       </c>
       <c r="J275" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K275" s="3" t="inlineStr">
@@ -34122,7 +34202,7 @@
       </c>
       <c r="J276" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K276" s="3" t="inlineStr">
@@ -34205,8 +34285,8 @@
       </c>
       <c r="J277" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K277" s="3" t="inlineStr">
@@ -34290,8 +34370,8 @@
       </c>
       <c r="J278" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K278" s="3" t="inlineStr">
@@ -34540,8 +34620,9 @@
       </c>
       <c r="J281" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K281" s="3" t="inlineStr">
@@ -34624,7 +34705,7 @@
       </c>
       <c r="J282" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K282" s="3" t="inlineStr">
@@ -34712,11 +34793,10 @@
       </c>
       <c r="J283" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Rounds the answer.
+          <t>· If annual contribution is missing it uses 0.
 · Treats a year as twelve equal months.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Caps the answer at a limit rather than letting it run.</t>
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K283" s="3" t="inlineStr">
@@ -34804,8 +34884,7 @@
       </c>
       <c r="J284" s="3" t="inlineStr">
         <is>
-          <t>· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Treats a year as twelve equal months.</t>
         </is>
       </c>
       <c r="K284" s="3" t="inlineStr">
@@ -34896,7 +34975,8 @@
       </c>
       <c r="J285" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K285" s="3" t="inlineStr">
@@ -34981,7 +35061,7 @@
       </c>
       <c r="J286" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K286" s="3" t="inlineStr">
@@ -35064,7 +35144,8 @@
       </c>
       <c r="J287" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K287" s="3" t="inlineStr">
@@ -35147,9 +35228,10 @@
       </c>
       <c r="J288" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Uses a built-in n of 12.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K288" s="3" t="inlineStr">
@@ -35316,7 +35398,8 @@
       </c>
       <c r="J290" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K290" s="3" t="inlineStr">
@@ -35399,7 +35482,7 @@
       </c>
       <c r="J291" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K291" s="3" t="inlineStr">
@@ -35482,8 +35565,7 @@
       </c>
       <c r="J292" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K292" s="3" t="inlineStr">
@@ -35567,9 +35649,11 @@
       </c>
       <c r="J293" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If contribution growth is missing it uses 0.
+· If monthly is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses a built-in y of 0.
+· Uses a built-in need of 0.
+· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K293" s="3" t="inlineStr">
@@ -35654,7 +35738,7 @@
       </c>
       <c r="J294" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K294" s="3" t="inlineStr">
@@ -35737,7 +35821,7 @@
       </c>
       <c r="J295" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K295" s="3" t="inlineStr">
@@ -35986,7 +36070,7 @@
       </c>
       <c r="J298" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K298" s="3" t="inlineStr">
@@ -36318,11 +36402,11 @@
       </c>
       <c r="J302" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Uses today's date from the device clock.
-· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If shares is missing it uses 0.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K302" s="3" t="inlineStr">
@@ -36405,7 +36489,7 @@
       </c>
       <c r="J303" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in changed of 0.</t>
         </is>
       </c>
       <c r="K303" s="3" t="inlineStr">
@@ -36490,7 +36574,8 @@
       </c>
       <c r="J304" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>· If cash is missing it uses 0.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K304" s="3" t="inlineStr">
@@ -36739,7 +36824,7 @@
       </c>
       <c r="J307" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K307" s="3" t="inlineStr">
@@ -37159,7 +37244,7 @@
       </c>
       <c r="J312" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K312" s="3" t="inlineStr">
@@ -37242,7 +37327,7 @@
       </c>
       <c r="J313" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K313" s="3" t="inlineStr">
@@ -37408,8 +37493,7 @@
       </c>
       <c r="J315" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If annual contribution is missing it uses 0.</t>
         </is>
       </c>
       <c r="K315" s="3" t="inlineStr">
@@ -37492,9 +37576,9 @@
       </c>
       <c r="J316" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If target is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If saved is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K316" s="3" t="inlineStr">
@@ -37578,8 +37662,7 @@
       </c>
       <c r="J317" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If monthly payment is missing it uses 0.</t>
         </is>
       </c>
       <c r="K317" s="3" t="inlineStr">
@@ -38166,7 +38249,7 @@
       </c>
       <c r="J324" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K324" s="3" t="inlineStr">
@@ -38421,7 +38504,7 @@
       </c>
       <c r="J327" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 1 instead of refusing.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K327" s="3" t="inlineStr">
@@ -38504,10 +38587,8 @@
       </c>
       <c r="J328" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· Treats a year as twelve equal months.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K328" s="3" t="inlineStr">
@@ -38592,8 +38673,9 @@
       </c>
       <c r="J329" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Uses today's date from the device clock.</t>
+          <t>· If amount is missing it uses 0.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K329" s="3" t="inlineStr">
@@ -38926,7 +39008,7 @@
       </c>
       <c r="J333" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K333" s="3" t="inlineStr">
@@ -39009,10 +39091,10 @@
       </c>
       <c r="J334" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If exp return is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses a built-in i of 0.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K334" s="3" t="inlineStr">
@@ -39182,7 +39264,7 @@
       </c>
       <c r="J336" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K336" s="3" t="inlineStr">
@@ -39348,8 +39430,9 @@
       </c>
       <c r="J338" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If amount is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K338" s="3" t="inlineStr">
@@ -39516,7 +39599,7 @@
       </c>
       <c r="J340" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K340" s="3" t="inlineStr">
@@ -39599,7 +39682,7 @@
       </c>
       <c r="J341" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K341" s="3" t="inlineStr">
@@ -39682,8 +39765,8 @@
       </c>
       <c r="J342" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K342" s="3" t="inlineStr">
@@ -39766,7 +39849,7 @@
       </c>
       <c r="J343" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K343" s="3" t="inlineStr">
@@ -39849,7 +39932,7 @@
       </c>
       <c r="J344" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K344" s="3" t="inlineStr">
@@ -39932,7 +40015,7 @@
       </c>
       <c r="J345" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K345" s="3" t="inlineStr">
@@ -40017,7 +40100,8 @@
       </c>
       <c r="J346" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K346" s="3" t="inlineStr">
@@ -40104,7 +40188,8 @@
       </c>
       <c r="J347" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K347" s="3" t="inlineStr">
@@ -40189,7 +40274,7 @@
       </c>
       <c r="J348" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K348" s="3" t="inlineStr">
@@ -41111,8 +41196,7 @@
       </c>
       <c r="J359" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If annual contribution is missing it uses 0.</t>
         </is>
       </c>
       <c r="K359" s="3" t="inlineStr">
@@ -41287,7 +41371,7 @@
       </c>
       <c r="J361" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K361" s="3" t="inlineStr">
@@ -41370,7 +41454,7 @@
       </c>
       <c r="J362" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K362" s="3" t="inlineStr">
@@ -41619,8 +41703,8 @@
       </c>
       <c r="J365" s="3" t="inlineStr">
         <is>
-          <t>· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in i of 0.
+· Treats a year as twelve equal months.</t>
         </is>
       </c>
       <c r="K365" s="3" t="inlineStr">
@@ -41794,7 +41878,7 @@
       </c>
       <c r="J367" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K367" s="3" t="inlineStr">
@@ -42541,7 +42625,8 @@
       </c>
       <c r="J376" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in page of 0.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K376" s="3" t="inlineStr">
@@ -42707,13 +42792,24 @@
       </c>
       <c r="J378" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 500 instead of refusing.
-· Rounds the answer.
+          <t>· If paths is missing it uses 500.
+· If seed is missing it uses 12345.
+· If now year is missing it uses 2026.
+· If contribution growth is missing it uses 0.
+· If pre tax share is missing it uses 0.
+· If required withdrawal tax rate is missing it uses 22%.
+· If monthly is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If one off by year[off] is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If recurring by year[y] is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If contrib by year[y] is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Uses a built-in y of 1.
+· Uses a built-in successes of 0.
+· Uses a built-in p of 0.
+· Uses a built-in y of 0.
 · Treats a year as twelve equal months.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+· Turns a monthly figure into a year by multiplying by twelve.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K378" s="3" t="inlineStr">
@@ -42797,8 +42893,8 @@
       </c>
       <c r="J379" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K379" s="3" t="inlineStr">
@@ -43141,9 +43237,10 @@
       </c>
       <c r="J383" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 300 instead of refusing.
-· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If paths is missing it uses 300.
+· If seed is missing it uses 42.
+· Uses a built-in i of 0.
+· Treats a year as twelve equal months.</t>
         </is>
       </c>
       <c r="K383" s="3" t="inlineStr">
@@ -43396,8 +43493,9 @@
       </c>
       <c r="J386" s="3" t="inlineStr">
         <is>
-          <t>· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses a built-in i of 0.
+· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.</t>
         </is>
       </c>
       <c r="K386" s="3" t="inlineStr">
@@ -43483,7 +43581,7 @@
       </c>
       <c r="J387" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K387" s="3" t="inlineStr">
@@ -43566,7 +43664,7 @@
       </c>
       <c r="J388" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Uses a built-in free of 0.</t>
         </is>
       </c>
       <c r="K388" s="3" t="inlineStr">
@@ -43649,8 +43747,8 @@
       </c>
       <c r="J389" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If statement monthly is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K389" s="3" t="inlineStr">
@@ -43899,9 +43997,9 @@
       </c>
       <c r="J392" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K392" s="3" t="inlineStr">
@@ -43984,8 +44082,8 @@
       </c>
       <c r="J393" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K393" s="3" t="inlineStr">
@@ -44151,8 +44249,7 @@
       </c>
       <c r="J395" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K395" s="3" t="inlineStr">
@@ -44401,8 +44498,7 @@
       </c>
       <c r="J398" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K398" s="3" t="inlineStr">
@@ -45168,9 +45264,11 @@
       </c>
       <c r="J407" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K407" s="3" t="inlineStr">
@@ -45261,7 +45359,7 @@
       </c>
       <c r="J408" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K408" s="3" t="inlineStr">
@@ -45344,8 +45442,7 @@
       </c>
       <c r="J409" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K409" s="3" t="inlineStr">
@@ -45511,7 +45608,8 @@
       </c>
       <c r="J411" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K411" s="3" t="inlineStr">
@@ -45602,9 +45700,8 @@
       </c>
       <c r="J412" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Treats a year as twelve equal months.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Treats a year as twelve equal months.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K412" s="3" t="inlineStr">
@@ -45695,7 +45792,7 @@
       </c>
       <c r="J413" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K413" s="3" t="inlineStr">
@@ -45778,7 +45875,7 @@
       </c>
       <c r="J414" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K414" s="3" t="inlineStr">
@@ -45861,7 +45958,7 @@
       </c>
       <c r="J415" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K415" s="3" t="inlineStr">
@@ -45947,7 +46044,7 @@
       </c>
       <c r="J416" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K416" s="3" t="inlineStr">
@@ -46199,7 +46296,7 @@
       </c>
       <c r="J419" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K419" s="3" t="inlineStr">
@@ -46284,8 +46381,8 @@
       </c>
       <c r="J420" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K420" s="3" t="inlineStr">
@@ -46368,7 +46465,7 @@
       </c>
       <c r="J421" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K421" s="3" t="inlineStr">
@@ -46451,7 +46548,7 @@
       </c>
       <c r="J422" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If remaining balance is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K422" s="3" t="inlineStr">
@@ -46617,7 +46714,8 @@
       </c>
       <c r="J424" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K424" s="3" t="inlineStr">
@@ -46791,7 +46889,7 @@
       </c>
       <c r="J426" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K426" s="3" t="inlineStr">
@@ -46878,7 +46976,7 @@
       </c>
       <c r="J427" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.</t>
         </is>
       </c>
       <c r="K427" s="3" t="inlineStr">
@@ -47128,10 +47226,9 @@
       </c>
       <c r="J430" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K430" s="3" t="inlineStr">
@@ -47388,7 +47485,7 @@
       </c>
       <c r="J433" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K433" s="3" t="inlineStr">
@@ -47472,8 +47569,9 @@
       </c>
       <c r="J434" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Multiplies by 100 — a percentage, or an option contract of 100 shares.</t>
+          <t>· Multiplies by 100 — a percentage, or an option contract treated as 100 shares. Worth checking which.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K434" s="3" t="inlineStr">
@@ -47556,7 +47654,7 @@
       </c>
       <c r="J435" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K435" s="3" t="inlineStr">
@@ -47974,11 +48072,14 @@
       </c>
       <c r="J440" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 2 instead of refusing.
-· Uses today's date from the device clock.
+          <t>· If buffer days is missing it uses 2.
+· If ask lead days is missing it uses 10.
+· If horizon days is missing it uses 365.
 · Treats a year as twelve equal months.
+· Turns a monthly figure into a year by multiplying by twelve.
 · Treats a year as 365 days.
-· Caps the answer at a limit rather than letting it run.</t>
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K440" s="3" t="inlineStr">
@@ -48069,7 +48170,8 @@
       </c>
       <c r="J441" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>· If cash is missing it uses 0.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K441" s="3" t="inlineStr">
@@ -48243,7 +48345,10 @@
       </c>
       <c r="J443" s="3" t="inlineStr">
         <is>
-          <t>· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If amount is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If shares is missing it counts as zero, so nothing recorded and a real zero look the same.
+· If price is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K443" s="3" t="inlineStr">
@@ -48326,8 +48431,8 @@
       </c>
       <c r="J444" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K444" s="3" t="inlineStr">
@@ -48410,7 +48515,8 @@
       </c>
       <c r="J445" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.</t>
+          <t>· If typed value is missing it uses 0.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K445" s="3" t="inlineStr">
@@ -48494,8 +48600,7 @@
       </c>
       <c r="J446" s="3" t="inlineStr">
         <is>
-          <t>· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Never lets the answer fall below 5% or rise above 20%.</t>
         </is>
       </c>
       <c r="K446" s="3" t="inlineStr">
@@ -48579,8 +48684,9 @@
       </c>
       <c r="J447" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· If emergency gap is missing it uses 0.
+· If toxic debt is missing it uses 0.
+· If employer match monthly is missing it uses 0.</t>
         </is>
       </c>
       <c r="K447" s="3" t="inlineStr">
@@ -48663,10 +48769,12 @@
       </c>
       <c r="J448" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 0 instead of refusing.
-· Uses today's date from the device clock.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If extra debt monthly is missing it uses 0.
+· If saved is missing it uses 0.
+· If monthly amount is missing it counts as zero, so nothing recorded and a real zero look the same.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K448" s="3" t="inlineStr">
@@ -48757,12 +48865,14 @@
       </c>
       <c r="J449" s="3" t="inlineStr">
         <is>
-          <t>· When the value is missing it uses 2.5 instead of refusing.
-· Uses today's date from the device clock.
-· Rounds the answer.
-· Carries a built-in rate or share that nobody chose on a screen.
-· Caps the answer at a limit rather than letting it run.
-· Treats a missing number as zero, so nothing recorded and genuinely zero look the same.</t>
+          <t>· If inflation rate is missing it uses 2.5.
+· If social security claim age is missing it uses 67.
+· If monthly is missing it uses 0.
+· If salary growth is missing it uses 0.
+· Turns a monthly figure into a year by multiplying by twelve.
+· Uses today's date from the device clock, so the answer changes by itself overnight.
+· Rounds the answer to a whole number.
+· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K449" s="3" t="inlineStr">
@@ -48853,7 +48963,7 @@
       </c>
       <c r="J450" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.</t>
+          <t>· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K450" s="3" t="inlineStr">
@@ -48936,7 +49046,7 @@
       </c>
       <c r="J451" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K451" s="3" t="inlineStr">
@@ -49019,7 +49129,7 @@
       </c>
       <c r="J452" s="3" t="inlineStr">
         <is>
-          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
+          <t>· Leaves some rows out of the answer — check which.</t>
         </is>
       </c>
       <c r="K452" s="3" t="inlineStr">
@@ -49105,8 +49215,8 @@
       </c>
       <c r="J453" s="3" t="inlineStr">
         <is>
-          <t>· Rounds the answer.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Turns a monthly figure into a year by multiplying by twelve.
+· Rounds the answer to a whole number.</t>
         </is>
       </c>
       <c r="K453" s="3" t="inlineStr">
@@ -49355,8 +49465,7 @@
       </c>
       <c r="J456" s="3" t="inlineStr">
         <is>
-          <t>· Uses today's date from the device clock.
-· Caps the answer at a limit rather than letting it run.</t>
+          <t>· Uses today's date from the device clock, so the answer changes by itself overnight.</t>
         </is>
       </c>
       <c r="K456" s="3" t="inlineStr">
@@ -49439,7 +49548,7 @@
       </c>
       <c r="J457" s="3" t="inlineStr">
         <is>
-          <t>· Caps the answer at a limit rather than letting it run.</t>
+          <t>None found in this function — anything it assumes comes from the functions it depends on.</t>
         </is>
       </c>
       <c r="K457" s="3" t="inlineStr">

</xml_diff>